<commit_message>
Add offset PDF generation and enhance employee offset workflow
</commit_message>
<xml_diff>
--- a/public/templates/forms/HRMS-PD Form 03.xlsx
+++ b/public/templates/forms/HRMS-PD Form 03.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bmacl\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/novu-rey/Documents/opappru_v5/hris_opap/public/templates/forms/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1165822-E99B-473C-82F5-428315D9015F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77584CAA-7787-F84D-8947-37210E9D28FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4320" yWindow="600" windowWidth="24480" windowHeight="15060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
   <si>
     <t>Civil Service Form No. 6</t>
   </si>
@@ -945,16 +945,50 @@
   <si>
     <t>Presidential Assistant for Internal Management System</t>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Wellness Leave (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="5.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Republic Act No. 11223</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+  </si>
+  <si>
+    <t>Wellness Leave</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
-    <numFmt numFmtId="166" formatCode="_([$PHP]\ * #,##0.00_);_([$PHP]\ * \(#,##0.00\);_([$PHP]\ * &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="167" formatCode="_(* #,##0.000_);_(* \(#,##0.000\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
+    <numFmt numFmtId="165" formatCode="_([$PHP]\ * #,##0.00_);_([$PHP]\ * \(#,##0.00\);_([$PHP]\ * &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0.000_);_(* \(#,##0.000\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="26" x14ac:knownFonts="1">
     <font>
@@ -1307,9 +1341,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1321,7 +1355,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="10" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1330,7 +1364,7 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="2" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="10" fillId="2" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1369,7 +1403,7 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="18" fillId="2" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="18" fillId="2" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1442,7 +1476,7 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1492,6 +1526,9 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1591,9 +1628,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1631,7 +1668,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1737,7 +1774,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1879,7 +1916,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1887,1047 +1924,983 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:WVX116"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="13.8" zeroHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:WVY117"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="14" zeroHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="2.21875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="1.77734375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="2.21875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="0.77734375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="14.44140625" style="2" customWidth="1"/>
-    <col min="6" max="7" width="14.5546875" style="2" customWidth="1"/>
-    <col min="8" max="8" width="3.21875" style="2" customWidth="1"/>
-    <col min="9" max="9" width="1.77734375" style="2" customWidth="1"/>
-    <col min="10" max="10" width="2.21875" style="2" customWidth="1"/>
-    <col min="11" max="11" width="0.77734375" style="2" customWidth="1"/>
-    <col min="12" max="12" width="13.77734375" style="2" customWidth="1"/>
-    <col min="13" max="13" width="3.21875" style="2" customWidth="1"/>
-    <col min="14" max="14" width="9.44140625" style="2" customWidth="1"/>
-    <col min="15" max="15" width="12.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="2.21875" style="2" customWidth="1"/>
-    <col min="17" max="256" width="9.21875" style="2" hidden="1"/>
-    <col min="257" max="257" width="2.21875" style="2" hidden="1"/>
-    <col min="258" max="258" width="1.77734375" style="2" hidden="1"/>
-    <col min="259" max="259" width="2.21875" style="2" hidden="1"/>
-    <col min="260" max="260" width="0.77734375" style="2" hidden="1"/>
-    <col min="261" max="261" width="14.44140625" style="2" hidden="1"/>
-    <col min="262" max="263" width="14.5546875" style="2" hidden="1"/>
-    <col min="264" max="264" width="3.21875" style="2" hidden="1"/>
-    <col min="265" max="265" width="1.77734375" style="2" hidden="1"/>
-    <col min="266" max="266" width="2.21875" style="2" hidden="1"/>
-    <col min="267" max="267" width="0.77734375" style="2" hidden="1"/>
-    <col min="268" max="268" width="13.77734375" style="2" hidden="1"/>
-    <col min="269" max="269" width="3.21875" style="2" hidden="1"/>
-    <col min="270" max="270" width="9.44140625" style="2" hidden="1"/>
-    <col min="271" max="271" width="12.21875" style="2" hidden="1"/>
-    <col min="272" max="272" width="2.21875" style="2" hidden="1"/>
-    <col min="273" max="512" width="9.21875" style="2" hidden="1"/>
-    <col min="513" max="513" width="2.21875" style="2" hidden="1"/>
-    <col min="514" max="514" width="1.77734375" style="2" hidden="1"/>
-    <col min="515" max="515" width="2.21875" style="2" hidden="1"/>
-    <col min="516" max="516" width="0.77734375" style="2" hidden="1"/>
-    <col min="517" max="517" width="14.44140625" style="2" hidden="1"/>
-    <col min="518" max="519" width="14.5546875" style="2" hidden="1"/>
-    <col min="520" max="520" width="3.21875" style="2" hidden="1"/>
-    <col min="521" max="521" width="1.77734375" style="2" hidden="1"/>
-    <col min="522" max="522" width="2.21875" style="2" hidden="1"/>
-    <col min="523" max="523" width="0.77734375" style="2" hidden="1"/>
-    <col min="524" max="524" width="13.77734375" style="2" hidden="1"/>
-    <col min="525" max="525" width="3.21875" style="2" hidden="1"/>
-    <col min="526" max="526" width="9.44140625" style="2" hidden="1"/>
-    <col min="527" max="527" width="12.21875" style="2" hidden="1"/>
-    <col min="528" max="528" width="2.21875" style="2" hidden="1"/>
-    <col min="529" max="768" width="9.21875" style="2" hidden="1"/>
-    <col min="769" max="769" width="2.21875" style="2" hidden="1"/>
-    <col min="770" max="770" width="1.77734375" style="2" hidden="1"/>
-    <col min="771" max="771" width="2.21875" style="2" hidden="1"/>
-    <col min="772" max="772" width="0.77734375" style="2" hidden="1"/>
-    <col min="773" max="773" width="14.44140625" style="2" hidden="1"/>
-    <col min="774" max="775" width="14.5546875" style="2" hidden="1"/>
-    <col min="776" max="776" width="3.21875" style="2" hidden="1"/>
-    <col min="777" max="777" width="1.77734375" style="2" hidden="1"/>
-    <col min="778" max="778" width="2.21875" style="2" hidden="1"/>
-    <col min="779" max="779" width="0.77734375" style="2" hidden="1"/>
-    <col min="780" max="780" width="13.77734375" style="2" hidden="1"/>
-    <col min="781" max="781" width="3.21875" style="2" hidden="1"/>
-    <col min="782" max="782" width="9.44140625" style="2" hidden="1"/>
-    <col min="783" max="783" width="12.21875" style="2" hidden="1"/>
-    <col min="784" max="784" width="2.21875" style="2" hidden="1"/>
-    <col min="785" max="1024" width="9.21875" style="2" hidden="1"/>
-    <col min="1025" max="1025" width="2.21875" style="2" hidden="1"/>
-    <col min="1026" max="1026" width="1.77734375" style="2" hidden="1"/>
-    <col min="1027" max="1027" width="2.21875" style="2" hidden="1"/>
-    <col min="1028" max="1028" width="0.77734375" style="2" hidden="1"/>
-    <col min="1029" max="1029" width="14.44140625" style="2" hidden="1"/>
-    <col min="1030" max="1031" width="14.5546875" style="2" hidden="1"/>
-    <col min="1032" max="1032" width="3.21875" style="2" hidden="1"/>
-    <col min="1033" max="1033" width="1.77734375" style="2" hidden="1"/>
-    <col min="1034" max="1034" width="2.21875" style="2" hidden="1"/>
-    <col min="1035" max="1035" width="0.77734375" style="2" hidden="1"/>
-    <col min="1036" max="1036" width="13.77734375" style="2" hidden="1"/>
-    <col min="1037" max="1037" width="3.21875" style="2" hidden="1"/>
-    <col min="1038" max="1038" width="9.44140625" style="2" hidden="1"/>
-    <col min="1039" max="1039" width="12.21875" style="2" hidden="1"/>
-    <col min="1040" max="1040" width="2.21875" style="2" hidden="1"/>
-    <col min="1041" max="1280" width="9.21875" style="2" hidden="1"/>
-    <col min="1281" max="1281" width="2.21875" style="2" hidden="1"/>
-    <col min="1282" max="1282" width="1.77734375" style="2" hidden="1"/>
-    <col min="1283" max="1283" width="2.21875" style="2" hidden="1"/>
-    <col min="1284" max="1284" width="0.77734375" style="2" hidden="1"/>
-    <col min="1285" max="1285" width="14.44140625" style="2" hidden="1"/>
-    <col min="1286" max="1287" width="14.5546875" style="2" hidden="1"/>
-    <col min="1288" max="1288" width="3.21875" style="2" hidden="1"/>
-    <col min="1289" max="1289" width="1.77734375" style="2" hidden="1"/>
-    <col min="1290" max="1290" width="2.21875" style="2" hidden="1"/>
-    <col min="1291" max="1291" width="0.77734375" style="2" hidden="1"/>
-    <col min="1292" max="1292" width="13.77734375" style="2" hidden="1"/>
-    <col min="1293" max="1293" width="3.21875" style="2" hidden="1"/>
-    <col min="1294" max="1294" width="9.44140625" style="2" hidden="1"/>
-    <col min="1295" max="1295" width="12.21875" style="2" hidden="1"/>
-    <col min="1296" max="1296" width="2.21875" style="2" hidden="1"/>
-    <col min="1297" max="1536" width="9.21875" style="2" hidden="1"/>
-    <col min="1537" max="1537" width="2.21875" style="2" hidden="1"/>
-    <col min="1538" max="1538" width="1.77734375" style="2" hidden="1"/>
-    <col min="1539" max="1539" width="2.21875" style="2" hidden="1"/>
-    <col min="1540" max="1540" width="0.77734375" style="2" hidden="1"/>
-    <col min="1541" max="1541" width="14.44140625" style="2" hidden="1"/>
-    <col min="1542" max="1543" width="14.5546875" style="2" hidden="1"/>
-    <col min="1544" max="1544" width="3.21875" style="2" hidden="1"/>
-    <col min="1545" max="1545" width="1.77734375" style="2" hidden="1"/>
-    <col min="1546" max="1546" width="2.21875" style="2" hidden="1"/>
-    <col min="1547" max="1547" width="0.77734375" style="2" hidden="1"/>
-    <col min="1548" max="1548" width="13.77734375" style="2" hidden="1"/>
-    <col min="1549" max="1549" width="3.21875" style="2" hidden="1"/>
-    <col min="1550" max="1550" width="9.44140625" style="2" hidden="1"/>
-    <col min="1551" max="1551" width="12.21875" style="2" hidden="1"/>
-    <col min="1552" max="1552" width="2.21875" style="2" hidden="1"/>
-    <col min="1553" max="1792" width="9.21875" style="2" hidden="1"/>
-    <col min="1793" max="1793" width="2.21875" style="2" hidden="1"/>
-    <col min="1794" max="1794" width="1.77734375" style="2" hidden="1"/>
-    <col min="1795" max="1795" width="2.21875" style="2" hidden="1"/>
-    <col min="1796" max="1796" width="0.77734375" style="2" hidden="1"/>
-    <col min="1797" max="1797" width="14.44140625" style="2" hidden="1"/>
-    <col min="1798" max="1799" width="14.5546875" style="2" hidden="1"/>
-    <col min="1800" max="1800" width="3.21875" style="2" hidden="1"/>
-    <col min="1801" max="1801" width="1.77734375" style="2" hidden="1"/>
-    <col min="1802" max="1802" width="2.21875" style="2" hidden="1"/>
-    <col min="1803" max="1803" width="0.77734375" style="2" hidden="1"/>
-    <col min="1804" max="1804" width="13.77734375" style="2" hidden="1"/>
-    <col min="1805" max="1805" width="3.21875" style="2" hidden="1"/>
-    <col min="1806" max="1806" width="9.44140625" style="2" hidden="1"/>
-    <col min="1807" max="1807" width="12.21875" style="2" hidden="1"/>
-    <col min="1808" max="1808" width="2.21875" style="2" hidden="1"/>
-    <col min="1809" max="2048" width="9.21875" style="2" hidden="1"/>
-    <col min="2049" max="2049" width="2.21875" style="2" hidden="1"/>
-    <col min="2050" max="2050" width="1.77734375" style="2" hidden="1"/>
-    <col min="2051" max="2051" width="2.21875" style="2" hidden="1"/>
-    <col min="2052" max="2052" width="0.77734375" style="2" hidden="1"/>
-    <col min="2053" max="2053" width="14.44140625" style="2" hidden="1"/>
-    <col min="2054" max="2055" width="14.5546875" style="2" hidden="1"/>
-    <col min="2056" max="2056" width="3.21875" style="2" hidden="1"/>
-    <col min="2057" max="2057" width="1.77734375" style="2" hidden="1"/>
-    <col min="2058" max="2058" width="2.21875" style="2" hidden="1"/>
-    <col min="2059" max="2059" width="0.77734375" style="2" hidden="1"/>
-    <col min="2060" max="2060" width="13.77734375" style="2" hidden="1"/>
-    <col min="2061" max="2061" width="3.21875" style="2" hidden="1"/>
-    <col min="2062" max="2062" width="9.44140625" style="2" hidden="1"/>
-    <col min="2063" max="2063" width="12.21875" style="2" hidden="1"/>
-    <col min="2064" max="2064" width="2.21875" style="2" hidden="1"/>
-    <col min="2065" max="2304" width="9.21875" style="2" hidden="1"/>
-    <col min="2305" max="2305" width="2.21875" style="2" hidden="1"/>
-    <col min="2306" max="2306" width="1.77734375" style="2" hidden="1"/>
-    <col min="2307" max="2307" width="2.21875" style="2" hidden="1"/>
-    <col min="2308" max="2308" width="0.77734375" style="2" hidden="1"/>
-    <col min="2309" max="2309" width="14.44140625" style="2" hidden="1"/>
-    <col min="2310" max="2311" width="14.5546875" style="2" hidden="1"/>
-    <col min="2312" max="2312" width="3.21875" style="2" hidden="1"/>
-    <col min="2313" max="2313" width="1.77734375" style="2" hidden="1"/>
-    <col min="2314" max="2314" width="2.21875" style="2" hidden="1"/>
-    <col min="2315" max="2315" width="0.77734375" style="2" hidden="1"/>
-    <col min="2316" max="2316" width="13.77734375" style="2" hidden="1"/>
-    <col min="2317" max="2317" width="3.21875" style="2" hidden="1"/>
-    <col min="2318" max="2318" width="9.44140625" style="2" hidden="1"/>
-    <col min="2319" max="2319" width="12.21875" style="2" hidden="1"/>
-    <col min="2320" max="2320" width="2.21875" style="2" hidden="1"/>
-    <col min="2321" max="2560" width="9.21875" style="2" hidden="1"/>
-    <col min="2561" max="2561" width="2.21875" style="2" hidden="1"/>
-    <col min="2562" max="2562" width="1.77734375" style="2" hidden="1"/>
-    <col min="2563" max="2563" width="2.21875" style="2" hidden="1"/>
-    <col min="2564" max="2564" width="0.77734375" style="2" hidden="1"/>
-    <col min="2565" max="2565" width="14.44140625" style="2" hidden="1"/>
-    <col min="2566" max="2567" width="14.5546875" style="2" hidden="1"/>
-    <col min="2568" max="2568" width="3.21875" style="2" hidden="1"/>
-    <col min="2569" max="2569" width="1.77734375" style="2" hidden="1"/>
-    <col min="2570" max="2570" width="2.21875" style="2" hidden="1"/>
-    <col min="2571" max="2571" width="0.77734375" style="2" hidden="1"/>
-    <col min="2572" max="2572" width="13.77734375" style="2" hidden="1"/>
-    <col min="2573" max="2573" width="3.21875" style="2" hidden="1"/>
-    <col min="2574" max="2574" width="9.44140625" style="2" hidden="1"/>
-    <col min="2575" max="2575" width="12.21875" style="2" hidden="1"/>
-    <col min="2576" max="2576" width="2.21875" style="2" hidden="1"/>
-    <col min="2577" max="2816" width="9.21875" style="2" hidden="1"/>
-    <col min="2817" max="2817" width="2.21875" style="2" hidden="1"/>
-    <col min="2818" max="2818" width="1.77734375" style="2" hidden="1"/>
-    <col min="2819" max="2819" width="2.21875" style="2" hidden="1"/>
-    <col min="2820" max="2820" width="0.77734375" style="2" hidden="1"/>
-    <col min="2821" max="2821" width="14.44140625" style="2" hidden="1"/>
-    <col min="2822" max="2823" width="14.5546875" style="2" hidden="1"/>
-    <col min="2824" max="2824" width="3.21875" style="2" hidden="1"/>
-    <col min="2825" max="2825" width="1.77734375" style="2" hidden="1"/>
-    <col min="2826" max="2826" width="2.21875" style="2" hidden="1"/>
-    <col min="2827" max="2827" width="0.77734375" style="2" hidden="1"/>
-    <col min="2828" max="2828" width="13.77734375" style="2" hidden="1"/>
-    <col min="2829" max="2829" width="3.21875" style="2" hidden="1"/>
-    <col min="2830" max="2830" width="9.44140625" style="2" hidden="1"/>
-    <col min="2831" max="2831" width="12.21875" style="2" hidden="1"/>
-    <col min="2832" max="2832" width="2.21875" style="2" hidden="1"/>
-    <col min="2833" max="3072" width="9.21875" style="2" hidden="1"/>
-    <col min="3073" max="3073" width="2.21875" style="2" hidden="1"/>
-    <col min="3074" max="3074" width="1.77734375" style="2" hidden="1"/>
-    <col min="3075" max="3075" width="2.21875" style="2" hidden="1"/>
-    <col min="3076" max="3076" width="0.77734375" style="2" hidden="1"/>
-    <col min="3077" max="3077" width="14.44140625" style="2" hidden="1"/>
-    <col min="3078" max="3079" width="14.5546875" style="2" hidden="1"/>
-    <col min="3080" max="3080" width="3.21875" style="2" hidden="1"/>
-    <col min="3081" max="3081" width="1.77734375" style="2" hidden="1"/>
-    <col min="3082" max="3082" width="2.21875" style="2" hidden="1"/>
-    <col min="3083" max="3083" width="0.77734375" style="2" hidden="1"/>
-    <col min="3084" max="3084" width="13.77734375" style="2" hidden="1"/>
-    <col min="3085" max="3085" width="3.21875" style="2" hidden="1"/>
-    <col min="3086" max="3086" width="9.44140625" style="2" hidden="1"/>
-    <col min="3087" max="3087" width="12.21875" style="2" hidden="1"/>
-    <col min="3088" max="3088" width="2.21875" style="2" hidden="1"/>
-    <col min="3089" max="3328" width="9.21875" style="2" hidden="1"/>
-    <col min="3329" max="3329" width="2.21875" style="2" hidden="1"/>
-    <col min="3330" max="3330" width="1.77734375" style="2" hidden="1"/>
-    <col min="3331" max="3331" width="2.21875" style="2" hidden="1"/>
-    <col min="3332" max="3332" width="0.77734375" style="2" hidden="1"/>
-    <col min="3333" max="3333" width="14.44140625" style="2" hidden="1"/>
-    <col min="3334" max="3335" width="14.5546875" style="2" hidden="1"/>
-    <col min="3336" max="3336" width="3.21875" style="2" hidden="1"/>
-    <col min="3337" max="3337" width="1.77734375" style="2" hidden="1"/>
-    <col min="3338" max="3338" width="2.21875" style="2" hidden="1"/>
-    <col min="3339" max="3339" width="0.77734375" style="2" hidden="1"/>
-    <col min="3340" max="3340" width="13.77734375" style="2" hidden="1"/>
-    <col min="3341" max="3341" width="3.21875" style="2" hidden="1"/>
-    <col min="3342" max="3342" width="9.44140625" style="2" hidden="1"/>
-    <col min="3343" max="3343" width="12.21875" style="2" hidden="1"/>
-    <col min="3344" max="3344" width="2.21875" style="2" hidden="1"/>
-    <col min="3345" max="3584" width="9.21875" style="2" hidden="1"/>
-    <col min="3585" max="3585" width="2.21875" style="2" hidden="1"/>
-    <col min="3586" max="3586" width="1.77734375" style="2" hidden="1"/>
-    <col min="3587" max="3587" width="2.21875" style="2" hidden="1"/>
-    <col min="3588" max="3588" width="0.77734375" style="2" hidden="1"/>
-    <col min="3589" max="3589" width="14.44140625" style="2" hidden="1"/>
-    <col min="3590" max="3591" width="14.5546875" style="2" hidden="1"/>
-    <col min="3592" max="3592" width="3.21875" style="2" hidden="1"/>
-    <col min="3593" max="3593" width="1.77734375" style="2" hidden="1"/>
-    <col min="3594" max="3594" width="2.21875" style="2" hidden="1"/>
-    <col min="3595" max="3595" width="0.77734375" style="2" hidden="1"/>
-    <col min="3596" max="3596" width="13.77734375" style="2" hidden="1"/>
-    <col min="3597" max="3597" width="3.21875" style="2" hidden="1"/>
-    <col min="3598" max="3598" width="9.44140625" style="2" hidden="1"/>
-    <col min="3599" max="3599" width="12.21875" style="2" hidden="1"/>
-    <col min="3600" max="3600" width="2.21875" style="2" hidden="1"/>
-    <col min="3601" max="3840" width="9.21875" style="2" hidden="1"/>
-    <col min="3841" max="3841" width="2.21875" style="2" hidden="1"/>
-    <col min="3842" max="3842" width="1.77734375" style="2" hidden="1"/>
-    <col min="3843" max="3843" width="2.21875" style="2" hidden="1"/>
-    <col min="3844" max="3844" width="0.77734375" style="2" hidden="1"/>
-    <col min="3845" max="3845" width="14.44140625" style="2" hidden="1"/>
-    <col min="3846" max="3847" width="14.5546875" style="2" hidden="1"/>
-    <col min="3848" max="3848" width="3.21875" style="2" hidden="1"/>
-    <col min="3849" max="3849" width="1.77734375" style="2" hidden="1"/>
-    <col min="3850" max="3850" width="2.21875" style="2" hidden="1"/>
-    <col min="3851" max="3851" width="0.77734375" style="2" hidden="1"/>
-    <col min="3852" max="3852" width="13.77734375" style="2" hidden="1"/>
-    <col min="3853" max="3853" width="3.21875" style="2" hidden="1"/>
-    <col min="3854" max="3854" width="9.44140625" style="2" hidden="1"/>
-    <col min="3855" max="3855" width="12.21875" style="2" hidden="1"/>
-    <col min="3856" max="3856" width="2.21875" style="2" hidden="1"/>
-    <col min="3857" max="4096" width="9.21875" style="2" hidden="1"/>
-    <col min="4097" max="4097" width="2.21875" style="2" hidden="1"/>
-    <col min="4098" max="4098" width="1.77734375" style="2" hidden="1"/>
-    <col min="4099" max="4099" width="2.21875" style="2" hidden="1"/>
-    <col min="4100" max="4100" width="0.77734375" style="2" hidden="1"/>
-    <col min="4101" max="4101" width="14.44140625" style="2" hidden="1"/>
-    <col min="4102" max="4103" width="14.5546875" style="2" hidden="1"/>
-    <col min="4104" max="4104" width="3.21875" style="2" hidden="1"/>
-    <col min="4105" max="4105" width="1.77734375" style="2" hidden="1"/>
-    <col min="4106" max="4106" width="2.21875" style="2" hidden="1"/>
-    <col min="4107" max="4107" width="0.77734375" style="2" hidden="1"/>
-    <col min="4108" max="4108" width="13.77734375" style="2" hidden="1"/>
-    <col min="4109" max="4109" width="3.21875" style="2" hidden="1"/>
-    <col min="4110" max="4110" width="9.44140625" style="2" hidden="1"/>
-    <col min="4111" max="4111" width="12.21875" style="2" hidden="1"/>
-    <col min="4112" max="4112" width="2.21875" style="2" hidden="1"/>
-    <col min="4113" max="4352" width="9.21875" style="2" hidden="1"/>
-    <col min="4353" max="4353" width="2.21875" style="2" hidden="1"/>
-    <col min="4354" max="4354" width="1.77734375" style="2" hidden="1"/>
-    <col min="4355" max="4355" width="2.21875" style="2" hidden="1"/>
-    <col min="4356" max="4356" width="0.77734375" style="2" hidden="1"/>
-    <col min="4357" max="4357" width="14.44140625" style="2" hidden="1"/>
-    <col min="4358" max="4359" width="14.5546875" style="2" hidden="1"/>
-    <col min="4360" max="4360" width="3.21875" style="2" hidden="1"/>
-    <col min="4361" max="4361" width="1.77734375" style="2" hidden="1"/>
-    <col min="4362" max="4362" width="2.21875" style="2" hidden="1"/>
-    <col min="4363" max="4363" width="0.77734375" style="2" hidden="1"/>
-    <col min="4364" max="4364" width="13.77734375" style="2" hidden="1"/>
-    <col min="4365" max="4365" width="3.21875" style="2" hidden="1"/>
-    <col min="4366" max="4366" width="9.44140625" style="2" hidden="1"/>
-    <col min="4367" max="4367" width="12.21875" style="2" hidden="1"/>
-    <col min="4368" max="4368" width="2.21875" style="2" hidden="1"/>
-    <col min="4369" max="4608" width="9.21875" style="2" hidden="1"/>
-    <col min="4609" max="4609" width="2.21875" style="2" hidden="1"/>
-    <col min="4610" max="4610" width="1.77734375" style="2" hidden="1"/>
-    <col min="4611" max="4611" width="2.21875" style="2" hidden="1"/>
-    <col min="4612" max="4612" width="0.77734375" style="2" hidden="1"/>
-    <col min="4613" max="4613" width="14.44140625" style="2" hidden="1"/>
-    <col min="4614" max="4615" width="14.5546875" style="2" hidden="1"/>
-    <col min="4616" max="4616" width="3.21875" style="2" hidden="1"/>
-    <col min="4617" max="4617" width="1.77734375" style="2" hidden="1"/>
-    <col min="4618" max="4618" width="2.21875" style="2" hidden="1"/>
-    <col min="4619" max="4619" width="0.77734375" style="2" hidden="1"/>
-    <col min="4620" max="4620" width="13.77734375" style="2" hidden="1"/>
-    <col min="4621" max="4621" width="3.21875" style="2" hidden="1"/>
-    <col min="4622" max="4622" width="9.44140625" style="2" hidden="1"/>
-    <col min="4623" max="4623" width="12.21875" style="2" hidden="1"/>
-    <col min="4624" max="4624" width="2.21875" style="2" hidden="1"/>
-    <col min="4625" max="4864" width="9.21875" style="2" hidden="1"/>
-    <col min="4865" max="4865" width="2.21875" style="2" hidden="1"/>
-    <col min="4866" max="4866" width="1.77734375" style="2" hidden="1"/>
-    <col min="4867" max="4867" width="2.21875" style="2" hidden="1"/>
-    <col min="4868" max="4868" width="0.77734375" style="2" hidden="1"/>
-    <col min="4869" max="4869" width="14.44140625" style="2" hidden="1"/>
-    <col min="4870" max="4871" width="14.5546875" style="2" hidden="1"/>
-    <col min="4872" max="4872" width="3.21875" style="2" hidden="1"/>
-    <col min="4873" max="4873" width="1.77734375" style="2" hidden="1"/>
-    <col min="4874" max="4874" width="2.21875" style="2" hidden="1"/>
-    <col min="4875" max="4875" width="0.77734375" style="2" hidden="1"/>
-    <col min="4876" max="4876" width="13.77734375" style="2" hidden="1"/>
-    <col min="4877" max="4877" width="3.21875" style="2" hidden="1"/>
-    <col min="4878" max="4878" width="9.44140625" style="2" hidden="1"/>
-    <col min="4879" max="4879" width="12.21875" style="2" hidden="1"/>
-    <col min="4880" max="4880" width="2.21875" style="2" hidden="1"/>
-    <col min="4881" max="5120" width="9.21875" style="2" hidden="1"/>
-    <col min="5121" max="5121" width="2.21875" style="2" hidden="1"/>
-    <col min="5122" max="5122" width="1.77734375" style="2" hidden="1"/>
-    <col min="5123" max="5123" width="2.21875" style="2" hidden="1"/>
-    <col min="5124" max="5124" width="0.77734375" style="2" hidden="1"/>
-    <col min="5125" max="5125" width="14.44140625" style="2" hidden="1"/>
-    <col min="5126" max="5127" width="14.5546875" style="2" hidden="1"/>
-    <col min="5128" max="5128" width="3.21875" style="2" hidden="1"/>
-    <col min="5129" max="5129" width="1.77734375" style="2" hidden="1"/>
-    <col min="5130" max="5130" width="2.21875" style="2" hidden="1"/>
-    <col min="5131" max="5131" width="0.77734375" style="2" hidden="1"/>
-    <col min="5132" max="5132" width="13.77734375" style="2" hidden="1"/>
-    <col min="5133" max="5133" width="3.21875" style="2" hidden="1"/>
-    <col min="5134" max="5134" width="9.44140625" style="2" hidden="1"/>
-    <col min="5135" max="5135" width="12.21875" style="2" hidden="1"/>
-    <col min="5136" max="5136" width="2.21875" style="2" hidden="1"/>
-    <col min="5137" max="5376" width="9.21875" style="2" hidden="1"/>
-    <col min="5377" max="5377" width="2.21875" style="2" hidden="1"/>
-    <col min="5378" max="5378" width="1.77734375" style="2" hidden="1"/>
-    <col min="5379" max="5379" width="2.21875" style="2" hidden="1"/>
-    <col min="5380" max="5380" width="0.77734375" style="2" hidden="1"/>
-    <col min="5381" max="5381" width="14.44140625" style="2" hidden="1"/>
-    <col min="5382" max="5383" width="14.5546875" style="2" hidden="1"/>
-    <col min="5384" max="5384" width="3.21875" style="2" hidden="1"/>
-    <col min="5385" max="5385" width="1.77734375" style="2" hidden="1"/>
-    <col min="5386" max="5386" width="2.21875" style="2" hidden="1"/>
-    <col min="5387" max="5387" width="0.77734375" style="2" hidden="1"/>
-    <col min="5388" max="5388" width="13.77734375" style="2" hidden="1"/>
-    <col min="5389" max="5389" width="3.21875" style="2" hidden="1"/>
-    <col min="5390" max="5390" width="9.44140625" style="2" hidden="1"/>
-    <col min="5391" max="5391" width="12.21875" style="2" hidden="1"/>
-    <col min="5392" max="5392" width="2.21875" style="2" hidden="1"/>
-    <col min="5393" max="5632" width="9.21875" style="2" hidden="1"/>
-    <col min="5633" max="5633" width="2.21875" style="2" hidden="1"/>
-    <col min="5634" max="5634" width="1.77734375" style="2" hidden="1"/>
-    <col min="5635" max="5635" width="2.21875" style="2" hidden="1"/>
-    <col min="5636" max="5636" width="0.77734375" style="2" hidden="1"/>
-    <col min="5637" max="5637" width="14.44140625" style="2" hidden="1"/>
-    <col min="5638" max="5639" width="14.5546875" style="2" hidden="1"/>
-    <col min="5640" max="5640" width="3.21875" style="2" hidden="1"/>
-    <col min="5641" max="5641" width="1.77734375" style="2" hidden="1"/>
-    <col min="5642" max="5642" width="2.21875" style="2" hidden="1"/>
-    <col min="5643" max="5643" width="0.77734375" style="2" hidden="1"/>
-    <col min="5644" max="5644" width="13.77734375" style="2" hidden="1"/>
-    <col min="5645" max="5645" width="3.21875" style="2" hidden="1"/>
-    <col min="5646" max="5646" width="9.44140625" style="2" hidden="1"/>
-    <col min="5647" max="5647" width="12.21875" style="2" hidden="1"/>
-    <col min="5648" max="5648" width="2.21875" style="2" hidden="1"/>
-    <col min="5649" max="5888" width="9.21875" style="2" hidden="1"/>
-    <col min="5889" max="5889" width="2.21875" style="2" hidden="1"/>
-    <col min="5890" max="5890" width="1.77734375" style="2" hidden="1"/>
-    <col min="5891" max="5891" width="2.21875" style="2" hidden="1"/>
-    <col min="5892" max="5892" width="0.77734375" style="2" hidden="1"/>
-    <col min="5893" max="5893" width="14.44140625" style="2" hidden="1"/>
-    <col min="5894" max="5895" width="14.5546875" style="2" hidden="1"/>
-    <col min="5896" max="5896" width="3.21875" style="2" hidden="1"/>
-    <col min="5897" max="5897" width="1.77734375" style="2" hidden="1"/>
-    <col min="5898" max="5898" width="2.21875" style="2" hidden="1"/>
-    <col min="5899" max="5899" width="0.77734375" style="2" hidden="1"/>
-    <col min="5900" max="5900" width="13.77734375" style="2" hidden="1"/>
-    <col min="5901" max="5901" width="3.21875" style="2" hidden="1"/>
-    <col min="5902" max="5902" width="9.44140625" style="2" hidden="1"/>
-    <col min="5903" max="5903" width="12.21875" style="2" hidden="1"/>
-    <col min="5904" max="5904" width="2.21875" style="2" hidden="1"/>
-    <col min="5905" max="6144" width="9.21875" style="2" hidden="1"/>
-    <col min="6145" max="6145" width="2.21875" style="2" hidden="1"/>
-    <col min="6146" max="6146" width="1.77734375" style="2" hidden="1"/>
-    <col min="6147" max="6147" width="2.21875" style="2" hidden="1"/>
-    <col min="6148" max="6148" width="0.77734375" style="2" hidden="1"/>
-    <col min="6149" max="6149" width="14.44140625" style="2" hidden="1"/>
-    <col min="6150" max="6151" width="14.5546875" style="2" hidden="1"/>
-    <col min="6152" max="6152" width="3.21875" style="2" hidden="1"/>
-    <col min="6153" max="6153" width="1.77734375" style="2" hidden="1"/>
-    <col min="6154" max="6154" width="2.21875" style="2" hidden="1"/>
-    <col min="6155" max="6155" width="0.77734375" style="2" hidden="1"/>
-    <col min="6156" max="6156" width="13.77734375" style="2" hidden="1"/>
-    <col min="6157" max="6157" width="3.21875" style="2" hidden="1"/>
-    <col min="6158" max="6158" width="9.44140625" style="2" hidden="1"/>
-    <col min="6159" max="6159" width="12.21875" style="2" hidden="1"/>
-    <col min="6160" max="6160" width="2.21875" style="2" hidden="1"/>
-    <col min="6161" max="6400" width="9.21875" style="2" hidden="1"/>
-    <col min="6401" max="6401" width="2.21875" style="2" hidden="1"/>
-    <col min="6402" max="6402" width="1.77734375" style="2" hidden="1"/>
-    <col min="6403" max="6403" width="2.21875" style="2" hidden="1"/>
-    <col min="6404" max="6404" width="0.77734375" style="2" hidden="1"/>
-    <col min="6405" max="6405" width="14.44140625" style="2" hidden="1"/>
-    <col min="6406" max="6407" width="14.5546875" style="2" hidden="1"/>
-    <col min="6408" max="6408" width="3.21875" style="2" hidden="1"/>
-    <col min="6409" max="6409" width="1.77734375" style="2" hidden="1"/>
-    <col min="6410" max="6410" width="2.21875" style="2" hidden="1"/>
-    <col min="6411" max="6411" width="0.77734375" style="2" hidden="1"/>
-    <col min="6412" max="6412" width="13.77734375" style="2" hidden="1"/>
-    <col min="6413" max="6413" width="3.21875" style="2" hidden="1"/>
-    <col min="6414" max="6414" width="9.44140625" style="2" hidden="1"/>
-    <col min="6415" max="6415" width="12.21875" style="2" hidden="1"/>
-    <col min="6416" max="6416" width="2.21875" style="2" hidden="1"/>
-    <col min="6417" max="6656" width="9.21875" style="2" hidden="1"/>
-    <col min="6657" max="6657" width="2.21875" style="2" hidden="1"/>
-    <col min="6658" max="6658" width="1.77734375" style="2" hidden="1"/>
-    <col min="6659" max="6659" width="2.21875" style="2" hidden="1"/>
-    <col min="6660" max="6660" width="0.77734375" style="2" hidden="1"/>
-    <col min="6661" max="6661" width="14.44140625" style="2" hidden="1"/>
-    <col min="6662" max="6663" width="14.5546875" style="2" hidden="1"/>
-    <col min="6664" max="6664" width="3.21875" style="2" hidden="1"/>
-    <col min="6665" max="6665" width="1.77734375" style="2" hidden="1"/>
-    <col min="6666" max="6666" width="2.21875" style="2" hidden="1"/>
-    <col min="6667" max="6667" width="0.77734375" style="2" hidden="1"/>
-    <col min="6668" max="6668" width="13.77734375" style="2" hidden="1"/>
-    <col min="6669" max="6669" width="3.21875" style="2" hidden="1"/>
-    <col min="6670" max="6670" width="9.44140625" style="2" hidden="1"/>
-    <col min="6671" max="6671" width="12.21875" style="2" hidden="1"/>
-    <col min="6672" max="6672" width="2.21875" style="2" hidden="1"/>
-    <col min="6673" max="6912" width="9.21875" style="2" hidden="1"/>
-    <col min="6913" max="6913" width="2.21875" style="2" hidden="1"/>
-    <col min="6914" max="6914" width="1.77734375" style="2" hidden="1"/>
-    <col min="6915" max="6915" width="2.21875" style="2" hidden="1"/>
-    <col min="6916" max="6916" width="0.77734375" style="2" hidden="1"/>
-    <col min="6917" max="6917" width="14.44140625" style="2" hidden="1"/>
-    <col min="6918" max="6919" width="14.5546875" style="2" hidden="1"/>
-    <col min="6920" max="6920" width="3.21875" style="2" hidden="1"/>
-    <col min="6921" max="6921" width="1.77734375" style="2" hidden="1"/>
-    <col min="6922" max="6922" width="2.21875" style="2" hidden="1"/>
-    <col min="6923" max="6923" width="0.77734375" style="2" hidden="1"/>
-    <col min="6924" max="6924" width="13.77734375" style="2" hidden="1"/>
-    <col min="6925" max="6925" width="3.21875" style="2" hidden="1"/>
-    <col min="6926" max="6926" width="9.44140625" style="2" hidden="1"/>
-    <col min="6927" max="6927" width="12.21875" style="2" hidden="1"/>
-    <col min="6928" max="6928" width="2.21875" style="2" hidden="1"/>
-    <col min="6929" max="7168" width="9.21875" style="2" hidden="1"/>
-    <col min="7169" max="7169" width="2.21875" style="2" hidden="1"/>
-    <col min="7170" max="7170" width="1.77734375" style="2" hidden="1"/>
-    <col min="7171" max="7171" width="2.21875" style="2" hidden="1"/>
-    <col min="7172" max="7172" width="0.77734375" style="2" hidden="1"/>
-    <col min="7173" max="7173" width="14.44140625" style="2" hidden="1"/>
-    <col min="7174" max="7175" width="14.5546875" style="2" hidden="1"/>
-    <col min="7176" max="7176" width="3.21875" style="2" hidden="1"/>
-    <col min="7177" max="7177" width="1.77734375" style="2" hidden="1"/>
-    <col min="7178" max="7178" width="2.21875" style="2" hidden="1"/>
-    <col min="7179" max="7179" width="0.77734375" style="2" hidden="1"/>
-    <col min="7180" max="7180" width="13.77734375" style="2" hidden="1"/>
-    <col min="7181" max="7181" width="3.21875" style="2" hidden="1"/>
-    <col min="7182" max="7182" width="9.44140625" style="2" hidden="1"/>
-    <col min="7183" max="7183" width="12.21875" style="2" hidden="1"/>
-    <col min="7184" max="7184" width="2.21875" style="2" hidden="1"/>
-    <col min="7185" max="7424" width="9.21875" style="2" hidden="1"/>
-    <col min="7425" max="7425" width="2.21875" style="2" hidden="1"/>
-    <col min="7426" max="7426" width="1.77734375" style="2" hidden="1"/>
-    <col min="7427" max="7427" width="2.21875" style="2" hidden="1"/>
-    <col min="7428" max="7428" width="0.77734375" style="2" hidden="1"/>
-    <col min="7429" max="7429" width="14.44140625" style="2" hidden="1"/>
-    <col min="7430" max="7431" width="14.5546875" style="2" hidden="1"/>
-    <col min="7432" max="7432" width="3.21875" style="2" hidden="1"/>
-    <col min="7433" max="7433" width="1.77734375" style="2" hidden="1"/>
-    <col min="7434" max="7434" width="2.21875" style="2" hidden="1"/>
-    <col min="7435" max="7435" width="0.77734375" style="2" hidden="1"/>
-    <col min="7436" max="7436" width="13.77734375" style="2" hidden="1"/>
-    <col min="7437" max="7437" width="3.21875" style="2" hidden="1"/>
-    <col min="7438" max="7438" width="9.44140625" style="2" hidden="1"/>
-    <col min="7439" max="7439" width="12.21875" style="2" hidden="1"/>
-    <col min="7440" max="7440" width="2.21875" style="2" hidden="1"/>
-    <col min="7441" max="7680" width="9.21875" style="2" hidden="1"/>
-    <col min="7681" max="7681" width="2.21875" style="2" hidden="1"/>
-    <col min="7682" max="7682" width="1.77734375" style="2" hidden="1"/>
-    <col min="7683" max="7683" width="2.21875" style="2" hidden="1"/>
-    <col min="7684" max="7684" width="0.77734375" style="2" hidden="1"/>
-    <col min="7685" max="7685" width="14.44140625" style="2" hidden="1"/>
-    <col min="7686" max="7687" width="14.5546875" style="2" hidden="1"/>
-    <col min="7688" max="7688" width="3.21875" style="2" hidden="1"/>
-    <col min="7689" max="7689" width="1.77734375" style="2" hidden="1"/>
-    <col min="7690" max="7690" width="2.21875" style="2" hidden="1"/>
-    <col min="7691" max="7691" width="0.77734375" style="2" hidden="1"/>
-    <col min="7692" max="7692" width="13.77734375" style="2" hidden="1"/>
-    <col min="7693" max="7693" width="3.21875" style="2" hidden="1"/>
-    <col min="7694" max="7694" width="9.44140625" style="2" hidden="1"/>
-    <col min="7695" max="7695" width="12.21875" style="2" hidden="1"/>
-    <col min="7696" max="7696" width="2.21875" style="2" hidden="1"/>
-    <col min="7697" max="7936" width="9.21875" style="2" hidden="1"/>
-    <col min="7937" max="7937" width="2.21875" style="2" hidden="1"/>
-    <col min="7938" max="7938" width="1.77734375" style="2" hidden="1"/>
-    <col min="7939" max="7939" width="2.21875" style="2" hidden="1"/>
-    <col min="7940" max="7940" width="0.77734375" style="2" hidden="1"/>
-    <col min="7941" max="7941" width="14.44140625" style="2" hidden="1"/>
-    <col min="7942" max="7943" width="14.5546875" style="2" hidden="1"/>
-    <col min="7944" max="7944" width="3.21875" style="2" hidden="1"/>
-    <col min="7945" max="7945" width="1.77734375" style="2" hidden="1"/>
-    <col min="7946" max="7946" width="2.21875" style="2" hidden="1"/>
-    <col min="7947" max="7947" width="0.77734375" style="2" hidden="1"/>
-    <col min="7948" max="7948" width="13.77734375" style="2" hidden="1"/>
-    <col min="7949" max="7949" width="3.21875" style="2" hidden="1"/>
-    <col min="7950" max="7950" width="9.44140625" style="2" hidden="1"/>
-    <col min="7951" max="7951" width="12.21875" style="2" hidden="1"/>
-    <col min="7952" max="7952" width="2.21875" style="2" hidden="1"/>
-    <col min="7953" max="8192" width="9.21875" style="2" hidden="1"/>
-    <col min="8193" max="8193" width="2.21875" style="2" hidden="1"/>
-    <col min="8194" max="8194" width="1.77734375" style="2" hidden="1"/>
-    <col min="8195" max="8195" width="2.21875" style="2" hidden="1"/>
-    <col min="8196" max="8196" width="0.77734375" style="2" hidden="1"/>
-    <col min="8197" max="8197" width="14.44140625" style="2" hidden="1"/>
-    <col min="8198" max="8199" width="14.5546875" style="2" hidden="1"/>
-    <col min="8200" max="8200" width="3.21875" style="2" hidden="1"/>
-    <col min="8201" max="8201" width="1.77734375" style="2" hidden="1"/>
-    <col min="8202" max="8202" width="2.21875" style="2" hidden="1"/>
-    <col min="8203" max="8203" width="0.77734375" style="2" hidden="1"/>
-    <col min="8204" max="8204" width="13.77734375" style="2" hidden="1"/>
-    <col min="8205" max="8205" width="3.21875" style="2" hidden="1"/>
-    <col min="8206" max="8206" width="9.44140625" style="2" hidden="1"/>
-    <col min="8207" max="8207" width="12.21875" style="2" hidden="1"/>
-    <col min="8208" max="8208" width="2.21875" style="2" hidden="1"/>
-    <col min="8209" max="8448" width="9.21875" style="2" hidden="1"/>
-    <col min="8449" max="8449" width="2.21875" style="2" hidden="1"/>
-    <col min="8450" max="8450" width="1.77734375" style="2" hidden="1"/>
-    <col min="8451" max="8451" width="2.21875" style="2" hidden="1"/>
-    <col min="8452" max="8452" width="0.77734375" style="2" hidden="1"/>
-    <col min="8453" max="8453" width="14.44140625" style="2" hidden="1"/>
-    <col min="8454" max="8455" width="14.5546875" style="2" hidden="1"/>
-    <col min="8456" max="8456" width="3.21875" style="2" hidden="1"/>
-    <col min="8457" max="8457" width="1.77734375" style="2" hidden="1"/>
-    <col min="8458" max="8458" width="2.21875" style="2" hidden="1"/>
-    <col min="8459" max="8459" width="0.77734375" style="2" hidden="1"/>
-    <col min="8460" max="8460" width="13.77734375" style="2" hidden="1"/>
-    <col min="8461" max="8461" width="3.21875" style="2" hidden="1"/>
-    <col min="8462" max="8462" width="9.44140625" style="2" hidden="1"/>
-    <col min="8463" max="8463" width="12.21875" style="2" hidden="1"/>
-    <col min="8464" max="8464" width="2.21875" style="2" hidden="1"/>
-    <col min="8465" max="8704" width="9.21875" style="2" hidden="1"/>
-    <col min="8705" max="8705" width="2.21875" style="2" hidden="1"/>
-    <col min="8706" max="8706" width="1.77734375" style="2" hidden="1"/>
-    <col min="8707" max="8707" width="2.21875" style="2" hidden="1"/>
-    <col min="8708" max="8708" width="0.77734375" style="2" hidden="1"/>
-    <col min="8709" max="8709" width="14.44140625" style="2" hidden="1"/>
-    <col min="8710" max="8711" width="14.5546875" style="2" hidden="1"/>
-    <col min="8712" max="8712" width="3.21875" style="2" hidden="1"/>
-    <col min="8713" max="8713" width="1.77734375" style="2" hidden="1"/>
-    <col min="8714" max="8714" width="2.21875" style="2" hidden="1"/>
-    <col min="8715" max="8715" width="0.77734375" style="2" hidden="1"/>
-    <col min="8716" max="8716" width="13.77734375" style="2" hidden="1"/>
-    <col min="8717" max="8717" width="3.21875" style="2" hidden="1"/>
-    <col min="8718" max="8718" width="9.44140625" style="2" hidden="1"/>
-    <col min="8719" max="8719" width="12.21875" style="2" hidden="1"/>
-    <col min="8720" max="8720" width="2.21875" style="2" hidden="1"/>
-    <col min="8721" max="8960" width="9.21875" style="2" hidden="1"/>
-    <col min="8961" max="8961" width="2.21875" style="2" hidden="1"/>
-    <col min="8962" max="8962" width="1.77734375" style="2" hidden="1"/>
-    <col min="8963" max="8963" width="2.21875" style="2" hidden="1"/>
-    <col min="8964" max="8964" width="0.77734375" style="2" hidden="1"/>
-    <col min="8965" max="8965" width="14.44140625" style="2" hidden="1"/>
-    <col min="8966" max="8967" width="14.5546875" style="2" hidden="1"/>
-    <col min="8968" max="8968" width="3.21875" style="2" hidden="1"/>
-    <col min="8969" max="8969" width="1.77734375" style="2" hidden="1"/>
-    <col min="8970" max="8970" width="2.21875" style="2" hidden="1"/>
-    <col min="8971" max="8971" width="0.77734375" style="2" hidden="1"/>
-    <col min="8972" max="8972" width="13.77734375" style="2" hidden="1"/>
-    <col min="8973" max="8973" width="3.21875" style="2" hidden="1"/>
-    <col min="8974" max="8974" width="9.44140625" style="2" hidden="1"/>
-    <col min="8975" max="8975" width="12.21875" style="2" hidden="1"/>
-    <col min="8976" max="8976" width="2.21875" style="2" hidden="1"/>
-    <col min="8977" max="9216" width="9.21875" style="2" hidden="1"/>
-    <col min="9217" max="9217" width="2.21875" style="2" hidden="1"/>
-    <col min="9218" max="9218" width="1.77734375" style="2" hidden="1"/>
-    <col min="9219" max="9219" width="2.21875" style="2" hidden="1"/>
-    <col min="9220" max="9220" width="0.77734375" style="2" hidden="1"/>
-    <col min="9221" max="9221" width="14.44140625" style="2" hidden="1"/>
-    <col min="9222" max="9223" width="14.5546875" style="2" hidden="1"/>
-    <col min="9224" max="9224" width="3.21875" style="2" hidden="1"/>
-    <col min="9225" max="9225" width="1.77734375" style="2" hidden="1"/>
-    <col min="9226" max="9226" width="2.21875" style="2" hidden="1"/>
-    <col min="9227" max="9227" width="0.77734375" style="2" hidden="1"/>
-    <col min="9228" max="9228" width="13.77734375" style="2" hidden="1"/>
-    <col min="9229" max="9229" width="3.21875" style="2" hidden="1"/>
-    <col min="9230" max="9230" width="9.44140625" style="2" hidden="1"/>
-    <col min="9231" max="9231" width="12.21875" style="2" hidden="1"/>
-    <col min="9232" max="9232" width="2.21875" style="2" hidden="1"/>
-    <col min="9233" max="9472" width="9.21875" style="2" hidden="1"/>
-    <col min="9473" max="9473" width="2.21875" style="2" hidden="1"/>
-    <col min="9474" max="9474" width="1.77734375" style="2" hidden="1"/>
-    <col min="9475" max="9475" width="2.21875" style="2" hidden="1"/>
-    <col min="9476" max="9476" width="0.77734375" style="2" hidden="1"/>
-    <col min="9477" max="9477" width="14.44140625" style="2" hidden="1"/>
-    <col min="9478" max="9479" width="14.5546875" style="2" hidden="1"/>
-    <col min="9480" max="9480" width="3.21875" style="2" hidden="1"/>
-    <col min="9481" max="9481" width="1.77734375" style="2" hidden="1"/>
-    <col min="9482" max="9482" width="2.21875" style="2" hidden="1"/>
-    <col min="9483" max="9483" width="0.77734375" style="2" hidden="1"/>
-    <col min="9484" max="9484" width="13.77734375" style="2" hidden="1"/>
-    <col min="9485" max="9485" width="3.21875" style="2" hidden="1"/>
-    <col min="9486" max="9486" width="9.44140625" style="2" hidden="1"/>
-    <col min="9487" max="9487" width="12.21875" style="2" hidden="1"/>
-    <col min="9488" max="9488" width="2.21875" style="2" hidden="1"/>
-    <col min="9489" max="9728" width="9.21875" style="2" hidden="1"/>
-    <col min="9729" max="9729" width="2.21875" style="2" hidden="1"/>
-    <col min="9730" max="9730" width="1.77734375" style="2" hidden="1"/>
-    <col min="9731" max="9731" width="2.21875" style="2" hidden="1"/>
-    <col min="9732" max="9732" width="0.77734375" style="2" hidden="1"/>
-    <col min="9733" max="9733" width="14.44140625" style="2" hidden="1"/>
-    <col min="9734" max="9735" width="14.5546875" style="2" hidden="1"/>
-    <col min="9736" max="9736" width="3.21875" style="2" hidden="1"/>
-    <col min="9737" max="9737" width="1.77734375" style="2" hidden="1"/>
-    <col min="9738" max="9738" width="2.21875" style="2" hidden="1"/>
-    <col min="9739" max="9739" width="0.77734375" style="2" hidden="1"/>
-    <col min="9740" max="9740" width="13.77734375" style="2" hidden="1"/>
-    <col min="9741" max="9741" width="3.21875" style="2" hidden="1"/>
-    <col min="9742" max="9742" width="9.44140625" style="2" hidden="1"/>
-    <col min="9743" max="9743" width="12.21875" style="2" hidden="1"/>
-    <col min="9744" max="9744" width="2.21875" style="2" hidden="1"/>
-    <col min="9745" max="9984" width="9.21875" style="2" hidden="1"/>
-    <col min="9985" max="9985" width="2.21875" style="2" hidden="1"/>
-    <col min="9986" max="9986" width="1.77734375" style="2" hidden="1"/>
-    <col min="9987" max="9987" width="2.21875" style="2" hidden="1"/>
-    <col min="9988" max="9988" width="0.77734375" style="2" hidden="1"/>
-    <col min="9989" max="9989" width="14.44140625" style="2" hidden="1"/>
-    <col min="9990" max="9991" width="14.5546875" style="2" hidden="1"/>
-    <col min="9992" max="9992" width="3.21875" style="2" hidden="1"/>
-    <col min="9993" max="9993" width="1.77734375" style="2" hidden="1"/>
-    <col min="9994" max="9994" width="2.21875" style="2" hidden="1"/>
-    <col min="9995" max="9995" width="0.77734375" style="2" hidden="1"/>
-    <col min="9996" max="9996" width="13.77734375" style="2" hidden="1"/>
-    <col min="9997" max="9997" width="3.21875" style="2" hidden="1"/>
-    <col min="9998" max="9998" width="9.44140625" style="2" hidden="1"/>
-    <col min="9999" max="9999" width="12.21875" style="2" hidden="1"/>
-    <col min="10000" max="10000" width="2.21875" style="2" hidden="1"/>
-    <col min="10001" max="10240" width="9.21875" style="2" hidden="1"/>
-    <col min="10241" max="10241" width="2.21875" style="2" hidden="1"/>
-    <col min="10242" max="10242" width="1.77734375" style="2" hidden="1"/>
-    <col min="10243" max="10243" width="2.21875" style="2" hidden="1"/>
-    <col min="10244" max="10244" width="0.77734375" style="2" hidden="1"/>
-    <col min="10245" max="10245" width="14.44140625" style="2" hidden="1"/>
-    <col min="10246" max="10247" width="14.5546875" style="2" hidden="1"/>
-    <col min="10248" max="10248" width="3.21875" style="2" hidden="1"/>
-    <col min="10249" max="10249" width="1.77734375" style="2" hidden="1"/>
-    <col min="10250" max="10250" width="2.21875" style="2" hidden="1"/>
-    <col min="10251" max="10251" width="0.77734375" style="2" hidden="1"/>
-    <col min="10252" max="10252" width="13.77734375" style="2" hidden="1"/>
-    <col min="10253" max="10253" width="3.21875" style="2" hidden="1"/>
-    <col min="10254" max="10254" width="9.44140625" style="2" hidden="1"/>
-    <col min="10255" max="10255" width="12.21875" style="2" hidden="1"/>
-    <col min="10256" max="10256" width="2.21875" style="2" hidden="1"/>
-    <col min="10257" max="10496" width="9.21875" style="2" hidden="1"/>
-    <col min="10497" max="10497" width="2.21875" style="2" hidden="1"/>
-    <col min="10498" max="10498" width="1.77734375" style="2" hidden="1"/>
-    <col min="10499" max="10499" width="2.21875" style="2" hidden="1"/>
-    <col min="10500" max="10500" width="0.77734375" style="2" hidden="1"/>
-    <col min="10501" max="10501" width="14.44140625" style="2" hidden="1"/>
-    <col min="10502" max="10503" width="14.5546875" style="2" hidden="1"/>
-    <col min="10504" max="10504" width="3.21875" style="2" hidden="1"/>
-    <col min="10505" max="10505" width="1.77734375" style="2" hidden="1"/>
-    <col min="10506" max="10506" width="2.21875" style="2" hidden="1"/>
-    <col min="10507" max="10507" width="0.77734375" style="2" hidden="1"/>
-    <col min="10508" max="10508" width="13.77734375" style="2" hidden="1"/>
-    <col min="10509" max="10509" width="3.21875" style="2" hidden="1"/>
-    <col min="10510" max="10510" width="9.44140625" style="2" hidden="1"/>
-    <col min="10511" max="10511" width="12.21875" style="2" hidden="1"/>
-    <col min="10512" max="10512" width="2.21875" style="2" hidden="1"/>
-    <col min="10513" max="10752" width="9.21875" style="2" hidden="1"/>
-    <col min="10753" max="10753" width="2.21875" style="2" hidden="1"/>
-    <col min="10754" max="10754" width="1.77734375" style="2" hidden="1"/>
-    <col min="10755" max="10755" width="2.21875" style="2" hidden="1"/>
-    <col min="10756" max="10756" width="0.77734375" style="2" hidden="1"/>
-    <col min="10757" max="10757" width="14.44140625" style="2" hidden="1"/>
-    <col min="10758" max="10759" width="14.5546875" style="2" hidden="1"/>
-    <col min="10760" max="10760" width="3.21875" style="2" hidden="1"/>
-    <col min="10761" max="10761" width="1.77734375" style="2" hidden="1"/>
-    <col min="10762" max="10762" width="2.21875" style="2" hidden="1"/>
-    <col min="10763" max="10763" width="0.77734375" style="2" hidden="1"/>
-    <col min="10764" max="10764" width="13.77734375" style="2" hidden="1"/>
-    <col min="10765" max="10765" width="3.21875" style="2" hidden="1"/>
-    <col min="10766" max="10766" width="9.44140625" style="2" hidden="1"/>
-    <col min="10767" max="10767" width="12.21875" style="2" hidden="1"/>
-    <col min="10768" max="10768" width="2.21875" style="2" hidden="1"/>
-    <col min="10769" max="11008" width="9.21875" style="2" hidden="1"/>
-    <col min="11009" max="11009" width="2.21875" style="2" hidden="1"/>
-    <col min="11010" max="11010" width="1.77734375" style="2" hidden="1"/>
-    <col min="11011" max="11011" width="2.21875" style="2" hidden="1"/>
-    <col min="11012" max="11012" width="0.77734375" style="2" hidden="1"/>
-    <col min="11013" max="11013" width="14.44140625" style="2" hidden="1"/>
-    <col min="11014" max="11015" width="14.5546875" style="2" hidden="1"/>
-    <col min="11016" max="11016" width="3.21875" style="2" hidden="1"/>
-    <col min="11017" max="11017" width="1.77734375" style="2" hidden="1"/>
-    <col min="11018" max="11018" width="2.21875" style="2" hidden="1"/>
-    <col min="11019" max="11019" width="0.77734375" style="2" hidden="1"/>
-    <col min="11020" max="11020" width="13.77734375" style="2" hidden="1"/>
-    <col min="11021" max="11021" width="3.21875" style="2" hidden="1"/>
-    <col min="11022" max="11022" width="9.44140625" style="2" hidden="1"/>
-    <col min="11023" max="11023" width="12.21875" style="2" hidden="1"/>
-    <col min="11024" max="11024" width="2.21875" style="2" hidden="1"/>
-    <col min="11025" max="11264" width="9.21875" style="2" hidden="1"/>
-    <col min="11265" max="11265" width="2.21875" style="2" hidden="1"/>
-    <col min="11266" max="11266" width="1.77734375" style="2" hidden="1"/>
-    <col min="11267" max="11267" width="2.21875" style="2" hidden="1"/>
-    <col min="11268" max="11268" width="0.77734375" style="2" hidden="1"/>
-    <col min="11269" max="11269" width="14.44140625" style="2" hidden="1"/>
-    <col min="11270" max="11271" width="14.5546875" style="2" hidden="1"/>
-    <col min="11272" max="11272" width="3.21875" style="2" hidden="1"/>
-    <col min="11273" max="11273" width="1.77734375" style="2" hidden="1"/>
-    <col min="11274" max="11274" width="2.21875" style="2" hidden="1"/>
-    <col min="11275" max="11275" width="0.77734375" style="2" hidden="1"/>
-    <col min="11276" max="11276" width="13.77734375" style="2" hidden="1"/>
-    <col min="11277" max="11277" width="3.21875" style="2" hidden="1"/>
-    <col min="11278" max="11278" width="9.44140625" style="2" hidden="1"/>
-    <col min="11279" max="11279" width="12.21875" style="2" hidden="1"/>
-    <col min="11280" max="11280" width="2.21875" style="2" hidden="1"/>
-    <col min="11281" max="11520" width="9.21875" style="2" hidden="1"/>
-    <col min="11521" max="11521" width="2.21875" style="2" hidden="1"/>
-    <col min="11522" max="11522" width="1.77734375" style="2" hidden="1"/>
-    <col min="11523" max="11523" width="2.21875" style="2" hidden="1"/>
-    <col min="11524" max="11524" width="0.77734375" style="2" hidden="1"/>
-    <col min="11525" max="11525" width="14.44140625" style="2" hidden="1"/>
-    <col min="11526" max="11527" width="14.5546875" style="2" hidden="1"/>
-    <col min="11528" max="11528" width="3.21875" style="2" hidden="1"/>
-    <col min="11529" max="11529" width="1.77734375" style="2" hidden="1"/>
-    <col min="11530" max="11530" width="2.21875" style="2" hidden="1"/>
-    <col min="11531" max="11531" width="0.77734375" style="2" hidden="1"/>
-    <col min="11532" max="11532" width="13.77734375" style="2" hidden="1"/>
-    <col min="11533" max="11533" width="3.21875" style="2" hidden="1"/>
-    <col min="11534" max="11534" width="9.44140625" style="2" hidden="1"/>
-    <col min="11535" max="11535" width="12.21875" style="2" hidden="1"/>
-    <col min="11536" max="11536" width="2.21875" style="2" hidden="1"/>
-    <col min="11537" max="11776" width="9.21875" style="2" hidden="1"/>
-    <col min="11777" max="11777" width="2.21875" style="2" hidden="1"/>
-    <col min="11778" max="11778" width="1.77734375" style="2" hidden="1"/>
-    <col min="11779" max="11779" width="2.21875" style="2" hidden="1"/>
-    <col min="11780" max="11780" width="0.77734375" style="2" hidden="1"/>
-    <col min="11781" max="11781" width="14.44140625" style="2" hidden="1"/>
-    <col min="11782" max="11783" width="14.5546875" style="2" hidden="1"/>
-    <col min="11784" max="11784" width="3.21875" style="2" hidden="1"/>
-    <col min="11785" max="11785" width="1.77734375" style="2" hidden="1"/>
-    <col min="11786" max="11786" width="2.21875" style="2" hidden="1"/>
-    <col min="11787" max="11787" width="0.77734375" style="2" hidden="1"/>
-    <col min="11788" max="11788" width="13.77734375" style="2" hidden="1"/>
-    <col min="11789" max="11789" width="3.21875" style="2" hidden="1"/>
-    <col min="11790" max="11790" width="9.44140625" style="2" hidden="1"/>
-    <col min="11791" max="11791" width="12.21875" style="2" hidden="1"/>
-    <col min="11792" max="11792" width="2.21875" style="2" hidden="1"/>
-    <col min="11793" max="12032" width="9.21875" style="2" hidden="1"/>
-    <col min="12033" max="12033" width="2.21875" style="2" hidden="1"/>
-    <col min="12034" max="12034" width="1.77734375" style="2" hidden="1"/>
-    <col min="12035" max="12035" width="2.21875" style="2" hidden="1"/>
-    <col min="12036" max="12036" width="0.77734375" style="2" hidden="1"/>
-    <col min="12037" max="12037" width="14.44140625" style="2" hidden="1"/>
-    <col min="12038" max="12039" width="14.5546875" style="2" hidden="1"/>
-    <col min="12040" max="12040" width="3.21875" style="2" hidden="1"/>
-    <col min="12041" max="12041" width="1.77734375" style="2" hidden="1"/>
-    <col min="12042" max="12042" width="2.21875" style="2" hidden="1"/>
-    <col min="12043" max="12043" width="0.77734375" style="2" hidden="1"/>
-    <col min="12044" max="12044" width="13.77734375" style="2" hidden="1"/>
-    <col min="12045" max="12045" width="3.21875" style="2" hidden="1"/>
-    <col min="12046" max="12046" width="9.44140625" style="2" hidden="1"/>
-    <col min="12047" max="12047" width="12.21875" style="2" hidden="1"/>
-    <col min="12048" max="12048" width="2.21875" style="2" hidden="1"/>
-    <col min="12049" max="12288" width="9.21875" style="2" hidden="1"/>
-    <col min="12289" max="12289" width="2.21875" style="2" hidden="1"/>
-    <col min="12290" max="12290" width="1.77734375" style="2" hidden="1"/>
-    <col min="12291" max="12291" width="2.21875" style="2" hidden="1"/>
-    <col min="12292" max="12292" width="0.77734375" style="2" hidden="1"/>
-    <col min="12293" max="12293" width="14.44140625" style="2" hidden="1"/>
-    <col min="12294" max="12295" width="14.5546875" style="2" hidden="1"/>
-    <col min="12296" max="12296" width="3.21875" style="2" hidden="1"/>
-    <col min="12297" max="12297" width="1.77734375" style="2" hidden="1"/>
-    <col min="12298" max="12298" width="2.21875" style="2" hidden="1"/>
-    <col min="12299" max="12299" width="0.77734375" style="2" hidden="1"/>
-    <col min="12300" max="12300" width="13.77734375" style="2" hidden="1"/>
-    <col min="12301" max="12301" width="3.21875" style="2" hidden="1"/>
-    <col min="12302" max="12302" width="9.44140625" style="2" hidden="1"/>
-    <col min="12303" max="12303" width="12.21875" style="2" hidden="1"/>
-    <col min="12304" max="12304" width="2.21875" style="2" hidden="1"/>
-    <col min="12305" max="12544" width="9.21875" style="2" hidden="1"/>
-    <col min="12545" max="12545" width="2.21875" style="2" hidden="1"/>
-    <col min="12546" max="12546" width="1.77734375" style="2" hidden="1"/>
-    <col min="12547" max="12547" width="2.21875" style="2" hidden="1"/>
-    <col min="12548" max="12548" width="0.77734375" style="2" hidden="1"/>
-    <col min="12549" max="12549" width="14.44140625" style="2" hidden="1"/>
-    <col min="12550" max="12551" width="14.5546875" style="2" hidden="1"/>
-    <col min="12552" max="12552" width="3.21875" style="2" hidden="1"/>
-    <col min="12553" max="12553" width="1.77734375" style="2" hidden="1"/>
-    <col min="12554" max="12554" width="2.21875" style="2" hidden="1"/>
-    <col min="12555" max="12555" width="0.77734375" style="2" hidden="1"/>
-    <col min="12556" max="12556" width="13.77734375" style="2" hidden="1"/>
-    <col min="12557" max="12557" width="3.21875" style="2" hidden="1"/>
-    <col min="12558" max="12558" width="9.44140625" style="2" hidden="1"/>
-    <col min="12559" max="12559" width="12.21875" style="2" hidden="1"/>
-    <col min="12560" max="12560" width="2.21875" style="2" hidden="1"/>
-    <col min="12561" max="12800" width="9.21875" style="2" hidden="1"/>
-    <col min="12801" max="12801" width="2.21875" style="2" hidden="1"/>
-    <col min="12802" max="12802" width="1.77734375" style="2" hidden="1"/>
-    <col min="12803" max="12803" width="2.21875" style="2" hidden="1"/>
-    <col min="12804" max="12804" width="0.77734375" style="2" hidden="1"/>
-    <col min="12805" max="12805" width="14.44140625" style="2" hidden="1"/>
-    <col min="12806" max="12807" width="14.5546875" style="2" hidden="1"/>
-    <col min="12808" max="12808" width="3.21875" style="2" hidden="1"/>
-    <col min="12809" max="12809" width="1.77734375" style="2" hidden="1"/>
-    <col min="12810" max="12810" width="2.21875" style="2" hidden="1"/>
-    <col min="12811" max="12811" width="0.77734375" style="2" hidden="1"/>
-    <col min="12812" max="12812" width="13.77734375" style="2" hidden="1"/>
-    <col min="12813" max="12813" width="3.21875" style="2" hidden="1"/>
-    <col min="12814" max="12814" width="9.44140625" style="2" hidden="1"/>
-    <col min="12815" max="12815" width="12.21875" style="2" hidden="1"/>
-    <col min="12816" max="12816" width="2.21875" style="2" hidden="1"/>
-    <col min="12817" max="13056" width="9.21875" style="2" hidden="1"/>
-    <col min="13057" max="13057" width="2.21875" style="2" hidden="1"/>
-    <col min="13058" max="13058" width="1.77734375" style="2" hidden="1"/>
-    <col min="13059" max="13059" width="2.21875" style="2" hidden="1"/>
-    <col min="13060" max="13060" width="0.77734375" style="2" hidden="1"/>
-    <col min="13061" max="13061" width="14.44140625" style="2" hidden="1"/>
-    <col min="13062" max="13063" width="14.5546875" style="2" hidden="1"/>
-    <col min="13064" max="13064" width="3.21875" style="2" hidden="1"/>
-    <col min="13065" max="13065" width="1.77734375" style="2" hidden="1"/>
-    <col min="13066" max="13066" width="2.21875" style="2" hidden="1"/>
-    <col min="13067" max="13067" width="0.77734375" style="2" hidden="1"/>
-    <col min="13068" max="13068" width="13.77734375" style="2" hidden="1"/>
-    <col min="13069" max="13069" width="3.21875" style="2" hidden="1"/>
-    <col min="13070" max="13070" width="9.44140625" style="2" hidden="1"/>
-    <col min="13071" max="13071" width="12.21875" style="2" hidden="1"/>
-    <col min="13072" max="13072" width="2.21875" style="2" hidden="1"/>
-    <col min="13073" max="13312" width="9.21875" style="2" hidden="1"/>
-    <col min="13313" max="13313" width="2.21875" style="2" hidden="1"/>
-    <col min="13314" max="13314" width="1.77734375" style="2" hidden="1"/>
-    <col min="13315" max="13315" width="2.21875" style="2" hidden="1"/>
-    <col min="13316" max="13316" width="0.77734375" style="2" hidden="1"/>
-    <col min="13317" max="13317" width="14.44140625" style="2" hidden="1"/>
-    <col min="13318" max="13319" width="14.5546875" style="2" hidden="1"/>
-    <col min="13320" max="13320" width="3.21875" style="2" hidden="1"/>
-    <col min="13321" max="13321" width="1.77734375" style="2" hidden="1"/>
-    <col min="13322" max="13322" width="2.21875" style="2" hidden="1"/>
-    <col min="13323" max="13323" width="0.77734375" style="2" hidden="1"/>
-    <col min="13324" max="13324" width="13.77734375" style="2" hidden="1"/>
-    <col min="13325" max="13325" width="3.21875" style="2" hidden="1"/>
-    <col min="13326" max="13326" width="9.44140625" style="2" hidden="1"/>
-    <col min="13327" max="13327" width="12.21875" style="2" hidden="1"/>
-    <col min="13328" max="13328" width="2.21875" style="2" hidden="1"/>
-    <col min="13329" max="13568" width="9.21875" style="2" hidden="1"/>
-    <col min="13569" max="13569" width="2.21875" style="2" hidden="1"/>
-    <col min="13570" max="13570" width="1.77734375" style="2" hidden="1"/>
-    <col min="13571" max="13571" width="2.21875" style="2" hidden="1"/>
-    <col min="13572" max="13572" width="0.77734375" style="2" hidden="1"/>
-    <col min="13573" max="13573" width="14.44140625" style="2" hidden="1"/>
-    <col min="13574" max="13575" width="14.5546875" style="2" hidden="1"/>
-    <col min="13576" max="13576" width="3.21875" style="2" hidden="1"/>
-    <col min="13577" max="13577" width="1.77734375" style="2" hidden="1"/>
-    <col min="13578" max="13578" width="2.21875" style="2" hidden="1"/>
-    <col min="13579" max="13579" width="0.77734375" style="2" hidden="1"/>
-    <col min="13580" max="13580" width="13.77734375" style="2" hidden="1"/>
-    <col min="13581" max="13581" width="3.21875" style="2" hidden="1"/>
-    <col min="13582" max="13582" width="9.44140625" style="2" hidden="1"/>
-    <col min="13583" max="13583" width="12.21875" style="2" hidden="1"/>
-    <col min="13584" max="13584" width="2.21875" style="2" hidden="1"/>
-    <col min="13585" max="13824" width="9.21875" style="2" hidden="1"/>
-    <col min="13825" max="13825" width="2.21875" style="2" hidden="1"/>
-    <col min="13826" max="13826" width="1.77734375" style="2" hidden="1"/>
-    <col min="13827" max="13827" width="2.21875" style="2" hidden="1"/>
-    <col min="13828" max="13828" width="0.77734375" style="2" hidden="1"/>
-    <col min="13829" max="13829" width="14.44140625" style="2" hidden="1"/>
-    <col min="13830" max="13831" width="14.5546875" style="2" hidden="1"/>
-    <col min="13832" max="13832" width="3.21875" style="2" hidden="1"/>
-    <col min="13833" max="13833" width="1.77734375" style="2" hidden="1"/>
-    <col min="13834" max="13834" width="2.21875" style="2" hidden="1"/>
-    <col min="13835" max="13835" width="0.77734375" style="2" hidden="1"/>
-    <col min="13836" max="13836" width="13.77734375" style="2" hidden="1"/>
-    <col min="13837" max="13837" width="3.21875" style="2" hidden="1"/>
-    <col min="13838" max="13838" width="9.44140625" style="2" hidden="1"/>
-    <col min="13839" max="13839" width="12.21875" style="2" hidden="1"/>
-    <col min="13840" max="13840" width="2.21875" style="2" hidden="1"/>
-    <col min="13841" max="14080" width="9.21875" style="2" hidden="1"/>
-    <col min="14081" max="14081" width="2.21875" style="2" hidden="1"/>
-    <col min="14082" max="14082" width="1.77734375" style="2" hidden="1"/>
-    <col min="14083" max="14083" width="2.21875" style="2" hidden="1"/>
-    <col min="14084" max="14084" width="0.77734375" style="2" hidden="1"/>
-    <col min="14085" max="14085" width="14.44140625" style="2" hidden="1"/>
-    <col min="14086" max="14087" width="14.5546875" style="2" hidden="1"/>
-    <col min="14088" max="14088" width="3.21875" style="2" hidden="1"/>
-    <col min="14089" max="14089" width="1.77734375" style="2" hidden="1"/>
-    <col min="14090" max="14090" width="2.21875" style="2" hidden="1"/>
-    <col min="14091" max="14091" width="0.77734375" style="2" hidden="1"/>
-    <col min="14092" max="14092" width="13.77734375" style="2" hidden="1"/>
-    <col min="14093" max="14093" width="3.21875" style="2" hidden="1"/>
-    <col min="14094" max="14094" width="9.44140625" style="2" hidden="1"/>
-    <col min="14095" max="14095" width="12.21875" style="2" hidden="1"/>
-    <col min="14096" max="14096" width="2.21875" style="2" hidden="1"/>
-    <col min="14097" max="14336" width="9.21875" style="2" hidden="1"/>
-    <col min="14337" max="14337" width="2.21875" style="2" hidden="1"/>
-    <col min="14338" max="14338" width="1.77734375" style="2" hidden="1"/>
-    <col min="14339" max="14339" width="2.21875" style="2" hidden="1"/>
-    <col min="14340" max="14340" width="0.77734375" style="2" hidden="1"/>
-    <col min="14341" max="14341" width="14.44140625" style="2" hidden="1"/>
-    <col min="14342" max="14343" width="14.5546875" style="2" hidden="1"/>
-    <col min="14344" max="14344" width="3.21875" style="2" hidden="1"/>
-    <col min="14345" max="14345" width="1.77734375" style="2" hidden="1"/>
-    <col min="14346" max="14346" width="2.21875" style="2" hidden="1"/>
-    <col min="14347" max="14347" width="0.77734375" style="2" hidden="1"/>
-    <col min="14348" max="14348" width="13.77734375" style="2" hidden="1"/>
-    <col min="14349" max="14349" width="3.21875" style="2" hidden="1"/>
-    <col min="14350" max="14350" width="9.44140625" style="2" hidden="1"/>
-    <col min="14351" max="14351" width="12.21875" style="2" hidden="1"/>
-    <col min="14352" max="14352" width="2.21875" style="2" hidden="1"/>
-    <col min="14353" max="14592" width="9.21875" style="2" hidden="1"/>
-    <col min="14593" max="14593" width="2.21875" style="2" hidden="1"/>
-    <col min="14594" max="14594" width="1.77734375" style="2" hidden="1"/>
-    <col min="14595" max="14595" width="2.21875" style="2" hidden="1"/>
-    <col min="14596" max="14596" width="0.77734375" style="2" hidden="1"/>
-    <col min="14597" max="14597" width="14.44140625" style="2" hidden="1"/>
-    <col min="14598" max="14599" width="14.5546875" style="2" hidden="1"/>
-    <col min="14600" max="14600" width="3.21875" style="2" hidden="1"/>
-    <col min="14601" max="14601" width="1.77734375" style="2" hidden="1"/>
-    <col min="14602" max="14602" width="2.21875" style="2" hidden="1"/>
-    <col min="14603" max="14603" width="0.77734375" style="2" hidden="1"/>
-    <col min="14604" max="14604" width="13.77734375" style="2" hidden="1"/>
-    <col min="14605" max="14605" width="3.21875" style="2" hidden="1"/>
-    <col min="14606" max="14606" width="9.44140625" style="2" hidden="1"/>
-    <col min="14607" max="14607" width="12.21875" style="2" hidden="1"/>
-    <col min="14608" max="14608" width="2.21875" style="2" hidden="1"/>
-    <col min="14609" max="14848" width="9.21875" style="2" hidden="1"/>
-    <col min="14849" max="14849" width="2.21875" style="2" hidden="1"/>
-    <col min="14850" max="14850" width="1.77734375" style="2" hidden="1"/>
-    <col min="14851" max="14851" width="2.21875" style="2" hidden="1"/>
-    <col min="14852" max="14852" width="0.77734375" style="2" hidden="1"/>
-    <col min="14853" max="14853" width="14.44140625" style="2" hidden="1"/>
-    <col min="14854" max="14855" width="14.5546875" style="2" hidden="1"/>
-    <col min="14856" max="14856" width="3.21875" style="2" hidden="1"/>
-    <col min="14857" max="14857" width="1.77734375" style="2" hidden="1"/>
-    <col min="14858" max="14858" width="2.21875" style="2" hidden="1"/>
-    <col min="14859" max="14859" width="0.77734375" style="2" hidden="1"/>
-    <col min="14860" max="14860" width="13.77734375" style="2" hidden="1"/>
-    <col min="14861" max="14861" width="3.21875" style="2" hidden="1"/>
-    <col min="14862" max="14862" width="9.44140625" style="2" hidden="1"/>
-    <col min="14863" max="14863" width="12.21875" style="2" hidden="1"/>
-    <col min="14864" max="14864" width="2.21875" style="2" hidden="1"/>
-    <col min="14865" max="15104" width="9.21875" style="2" hidden="1"/>
-    <col min="15105" max="15105" width="2.21875" style="2" hidden="1"/>
-    <col min="15106" max="15106" width="1.77734375" style="2" hidden="1"/>
-    <col min="15107" max="15107" width="2.21875" style="2" hidden="1"/>
-    <col min="15108" max="15108" width="0.77734375" style="2" hidden="1"/>
-    <col min="15109" max="15109" width="14.44140625" style="2" hidden="1"/>
-    <col min="15110" max="15111" width="14.5546875" style="2" hidden="1"/>
-    <col min="15112" max="15112" width="3.21875" style="2" hidden="1"/>
-    <col min="15113" max="15113" width="1.77734375" style="2" hidden="1"/>
-    <col min="15114" max="15114" width="2.21875" style="2" hidden="1"/>
-    <col min="15115" max="15115" width="0.77734375" style="2" hidden="1"/>
-    <col min="15116" max="15116" width="13.77734375" style="2" hidden="1"/>
-    <col min="15117" max="15117" width="3.21875" style="2" hidden="1"/>
-    <col min="15118" max="15118" width="9.44140625" style="2" hidden="1"/>
-    <col min="15119" max="15119" width="12.21875" style="2" hidden="1"/>
-    <col min="15120" max="15120" width="2.21875" style="2" hidden="1"/>
-    <col min="15121" max="15360" width="9.21875" style="2" hidden="1"/>
-    <col min="15361" max="15361" width="2.21875" style="2" hidden="1"/>
-    <col min="15362" max="15362" width="1.77734375" style="2" hidden="1"/>
-    <col min="15363" max="15363" width="2.21875" style="2" hidden="1"/>
-    <col min="15364" max="15364" width="0.77734375" style="2" hidden="1"/>
-    <col min="15365" max="15365" width="14.44140625" style="2" hidden="1"/>
-    <col min="15366" max="15367" width="14.5546875" style="2" hidden="1"/>
-    <col min="15368" max="15368" width="3.21875" style="2" hidden="1"/>
-    <col min="15369" max="15369" width="1.77734375" style="2" hidden="1"/>
-    <col min="15370" max="15370" width="2.21875" style="2" hidden="1"/>
-    <col min="15371" max="15371" width="0.77734375" style="2" hidden="1"/>
-    <col min="15372" max="15372" width="13.77734375" style="2" hidden="1"/>
-    <col min="15373" max="15373" width="3.21875" style="2" hidden="1"/>
-    <col min="15374" max="15374" width="9.44140625" style="2" hidden="1"/>
-    <col min="15375" max="15375" width="12.21875" style="2" hidden="1"/>
-    <col min="15376" max="15376" width="2.21875" style="2" hidden="1"/>
-    <col min="15377" max="15616" width="9.21875" style="2" hidden="1"/>
-    <col min="15617" max="15617" width="2.21875" style="2" hidden="1"/>
-    <col min="15618" max="15618" width="1.77734375" style="2" hidden="1"/>
-    <col min="15619" max="15619" width="2.21875" style="2" hidden="1"/>
-    <col min="15620" max="15620" width="0.77734375" style="2" hidden="1"/>
-    <col min="15621" max="15621" width="14.44140625" style="2" hidden="1"/>
-    <col min="15622" max="15623" width="14.5546875" style="2" hidden="1"/>
-    <col min="15624" max="15624" width="3.21875" style="2" hidden="1"/>
-    <col min="15625" max="15625" width="1.77734375" style="2" hidden="1"/>
-    <col min="15626" max="15626" width="2.21875" style="2" hidden="1"/>
-    <col min="15627" max="15627" width="0.77734375" style="2" hidden="1"/>
-    <col min="15628" max="15628" width="13.77734375" style="2" hidden="1"/>
-    <col min="15629" max="15629" width="3.21875" style="2" hidden="1"/>
-    <col min="15630" max="15630" width="9.44140625" style="2" hidden="1"/>
-    <col min="15631" max="15631" width="12.21875" style="2" hidden="1"/>
-    <col min="15632" max="15632" width="2.21875" style="2" hidden="1"/>
-    <col min="15633" max="15872" width="9.21875" style="2" hidden="1"/>
-    <col min="15873" max="15873" width="2.21875" style="2" hidden="1"/>
-    <col min="15874" max="15874" width="1.77734375" style="2" hidden="1"/>
-    <col min="15875" max="15875" width="2.21875" style="2" hidden="1"/>
-    <col min="15876" max="15876" width="0.77734375" style="2" hidden="1"/>
-    <col min="15877" max="15877" width="14.44140625" style="2" hidden="1"/>
-    <col min="15878" max="15879" width="14.5546875" style="2" hidden="1"/>
-    <col min="15880" max="15880" width="3.21875" style="2" hidden="1"/>
-    <col min="15881" max="15881" width="1.77734375" style="2" hidden="1"/>
-    <col min="15882" max="15882" width="2.21875" style="2" hidden="1"/>
-    <col min="15883" max="15883" width="0.77734375" style="2" hidden="1"/>
-    <col min="15884" max="15884" width="13.77734375" style="2" hidden="1"/>
-    <col min="15885" max="15885" width="3.21875" style="2" hidden="1"/>
-    <col min="15886" max="15886" width="9.44140625" style="2" hidden="1"/>
-    <col min="15887" max="15887" width="12.21875" style="2" hidden="1"/>
-    <col min="15888" max="15888" width="2.21875" style="2" hidden="1"/>
-    <col min="15889" max="16128" width="9.21875" style="2" hidden="1"/>
-    <col min="16129" max="16129" width="2.21875" style="2" hidden="1"/>
-    <col min="16130" max="16130" width="1.77734375" style="2" hidden="1"/>
-    <col min="16131" max="16131" width="2.21875" style="2" hidden="1"/>
-    <col min="16132" max="16132" width="0.77734375" style="2" hidden="1"/>
-    <col min="16133" max="16133" width="14.44140625" style="2" hidden="1"/>
-    <col min="16134" max="16135" width="14.5546875" style="2" hidden="1"/>
-    <col min="16136" max="16136" width="3.21875" style="2" hidden="1"/>
-    <col min="16137" max="16137" width="1.77734375" style="2" hidden="1"/>
-    <col min="16138" max="16138" width="2.21875" style="2" hidden="1"/>
-    <col min="16139" max="16139" width="0.77734375" style="2" hidden="1"/>
-    <col min="16140" max="16140" width="13.77734375" style="2" hidden="1"/>
-    <col min="16141" max="16141" width="3.21875" style="2" hidden="1"/>
-    <col min="16142" max="16142" width="9.44140625" style="2" hidden="1"/>
-    <col min="16143" max="16143" width="12.21875" style="2" hidden="1"/>
-    <col min="16144" max="16144" width="2.21875" style="2" hidden="1"/>
-    <col min="16145" max="16384" width="9.21875" style="2" hidden="1"/>
+    <col min="1" max="1" width="2.1640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="1.83203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="2.1640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="0.83203125" style="2" customWidth="1"/>
+    <col min="5" max="8" width="14.5" style="2" customWidth="1"/>
+    <col min="9" max="9" width="3.1640625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="1.83203125" style="2" customWidth="1"/>
+    <col min="11" max="11" width="2.1640625" style="2" customWidth="1"/>
+    <col min="12" max="12" width="0.83203125" style="2" customWidth="1"/>
+    <col min="13" max="13" width="13.83203125" style="2" customWidth="1"/>
+    <col min="14" max="14" width="3.1640625" style="2" customWidth="1"/>
+    <col min="15" max="15" width="9.5" style="2" customWidth="1"/>
+    <col min="16" max="16" width="12.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="2.1640625" style="2" customWidth="1"/>
+    <col min="18" max="257" width="9.1640625" style="2" hidden="1"/>
+    <col min="258" max="258" width="2.1640625" style="2" hidden="1"/>
+    <col min="259" max="259" width="1.83203125" style="2" hidden="1"/>
+    <col min="260" max="260" width="2.1640625" style="2" hidden="1"/>
+    <col min="261" max="261" width="0.83203125" style="2" hidden="1"/>
+    <col min="262" max="264" width="14.5" style="2" hidden="1"/>
+    <col min="265" max="265" width="3.1640625" style="2" hidden="1"/>
+    <col min="266" max="266" width="1.83203125" style="2" hidden="1"/>
+    <col min="267" max="267" width="2.1640625" style="2" hidden="1"/>
+    <col min="268" max="268" width="0.83203125" style="2" hidden="1"/>
+    <col min="269" max="269" width="13.83203125" style="2" hidden="1"/>
+    <col min="270" max="270" width="3.1640625" style="2" hidden="1"/>
+    <col min="271" max="271" width="9.5" style="2" hidden="1"/>
+    <col min="272" max="272" width="12.1640625" style="2" hidden="1"/>
+    <col min="273" max="273" width="2.1640625" style="2" hidden="1"/>
+    <col min="274" max="513" width="9.1640625" style="2" hidden="1"/>
+    <col min="514" max="514" width="2.1640625" style="2" hidden="1"/>
+    <col min="515" max="515" width="1.83203125" style="2" hidden="1"/>
+    <col min="516" max="516" width="2.1640625" style="2" hidden="1"/>
+    <col min="517" max="517" width="0.83203125" style="2" hidden="1"/>
+    <col min="518" max="520" width="14.5" style="2" hidden="1"/>
+    <col min="521" max="521" width="3.1640625" style="2" hidden="1"/>
+    <col min="522" max="522" width="1.83203125" style="2" hidden="1"/>
+    <col min="523" max="523" width="2.1640625" style="2" hidden="1"/>
+    <col min="524" max="524" width="0.83203125" style="2" hidden="1"/>
+    <col min="525" max="525" width="13.83203125" style="2" hidden="1"/>
+    <col min="526" max="526" width="3.1640625" style="2" hidden="1"/>
+    <col min="527" max="527" width="9.5" style="2" hidden="1"/>
+    <col min="528" max="528" width="12.1640625" style="2" hidden="1"/>
+    <col min="529" max="529" width="2.1640625" style="2" hidden="1"/>
+    <col min="530" max="769" width="9.1640625" style="2" hidden="1"/>
+    <col min="770" max="770" width="2.1640625" style="2" hidden="1"/>
+    <col min="771" max="771" width="1.83203125" style="2" hidden="1"/>
+    <col min="772" max="772" width="2.1640625" style="2" hidden="1"/>
+    <col min="773" max="773" width="0.83203125" style="2" hidden="1"/>
+    <col min="774" max="776" width="14.5" style="2" hidden="1"/>
+    <col min="777" max="777" width="3.1640625" style="2" hidden="1"/>
+    <col min="778" max="778" width="1.83203125" style="2" hidden="1"/>
+    <col min="779" max="779" width="2.1640625" style="2" hidden="1"/>
+    <col min="780" max="780" width="0.83203125" style="2" hidden="1"/>
+    <col min="781" max="781" width="13.83203125" style="2" hidden="1"/>
+    <col min="782" max="782" width="3.1640625" style="2" hidden="1"/>
+    <col min="783" max="783" width="9.5" style="2" hidden="1"/>
+    <col min="784" max="784" width="12.1640625" style="2" hidden="1"/>
+    <col min="785" max="785" width="2.1640625" style="2" hidden="1"/>
+    <col min="786" max="1025" width="9.1640625" style="2" hidden="1"/>
+    <col min="1026" max="1026" width="2.1640625" style="2" hidden="1"/>
+    <col min="1027" max="1027" width="1.83203125" style="2" hidden="1"/>
+    <col min="1028" max="1028" width="2.1640625" style="2" hidden="1"/>
+    <col min="1029" max="1029" width="0.83203125" style="2" hidden="1"/>
+    <col min="1030" max="1032" width="14.5" style="2" hidden="1"/>
+    <col min="1033" max="1033" width="3.1640625" style="2" hidden="1"/>
+    <col min="1034" max="1034" width="1.83203125" style="2" hidden="1"/>
+    <col min="1035" max="1035" width="2.1640625" style="2" hidden="1"/>
+    <col min="1036" max="1036" width="0.83203125" style="2" hidden="1"/>
+    <col min="1037" max="1037" width="13.83203125" style="2" hidden="1"/>
+    <col min="1038" max="1038" width="3.1640625" style="2" hidden="1"/>
+    <col min="1039" max="1039" width="9.5" style="2" hidden="1"/>
+    <col min="1040" max="1040" width="12.1640625" style="2" hidden="1"/>
+    <col min="1041" max="1041" width="2.1640625" style="2" hidden="1"/>
+    <col min="1042" max="1281" width="9.1640625" style="2" hidden="1"/>
+    <col min="1282" max="1282" width="2.1640625" style="2" hidden="1"/>
+    <col min="1283" max="1283" width="1.83203125" style="2" hidden="1"/>
+    <col min="1284" max="1284" width="2.1640625" style="2" hidden="1"/>
+    <col min="1285" max="1285" width="0.83203125" style="2" hidden="1"/>
+    <col min="1286" max="1288" width="14.5" style="2" hidden="1"/>
+    <col min="1289" max="1289" width="3.1640625" style="2" hidden="1"/>
+    <col min="1290" max="1290" width="1.83203125" style="2" hidden="1"/>
+    <col min="1291" max="1291" width="2.1640625" style="2" hidden="1"/>
+    <col min="1292" max="1292" width="0.83203125" style="2" hidden="1"/>
+    <col min="1293" max="1293" width="13.83203125" style="2" hidden="1"/>
+    <col min="1294" max="1294" width="3.1640625" style="2" hidden="1"/>
+    <col min="1295" max="1295" width="9.5" style="2" hidden="1"/>
+    <col min="1296" max="1296" width="12.1640625" style="2" hidden="1"/>
+    <col min="1297" max="1297" width="2.1640625" style="2" hidden="1"/>
+    <col min="1298" max="1537" width="9.1640625" style="2" hidden="1"/>
+    <col min="1538" max="1538" width="2.1640625" style="2" hidden="1"/>
+    <col min="1539" max="1539" width="1.83203125" style="2" hidden="1"/>
+    <col min="1540" max="1540" width="2.1640625" style="2" hidden="1"/>
+    <col min="1541" max="1541" width="0.83203125" style="2" hidden="1"/>
+    <col min="1542" max="1544" width="14.5" style="2" hidden="1"/>
+    <col min="1545" max="1545" width="3.1640625" style="2" hidden="1"/>
+    <col min="1546" max="1546" width="1.83203125" style="2" hidden="1"/>
+    <col min="1547" max="1547" width="2.1640625" style="2" hidden="1"/>
+    <col min="1548" max="1548" width="0.83203125" style="2" hidden="1"/>
+    <col min="1549" max="1549" width="13.83203125" style="2" hidden="1"/>
+    <col min="1550" max="1550" width="3.1640625" style="2" hidden="1"/>
+    <col min="1551" max="1551" width="9.5" style="2" hidden="1"/>
+    <col min="1552" max="1552" width="12.1640625" style="2" hidden="1"/>
+    <col min="1553" max="1553" width="2.1640625" style="2" hidden="1"/>
+    <col min="1554" max="1793" width="9.1640625" style="2" hidden="1"/>
+    <col min="1794" max="1794" width="2.1640625" style="2" hidden="1"/>
+    <col min="1795" max="1795" width="1.83203125" style="2" hidden="1"/>
+    <col min="1796" max="1796" width="2.1640625" style="2" hidden="1"/>
+    <col min="1797" max="1797" width="0.83203125" style="2" hidden="1"/>
+    <col min="1798" max="1800" width="14.5" style="2" hidden="1"/>
+    <col min="1801" max="1801" width="3.1640625" style="2" hidden="1"/>
+    <col min="1802" max="1802" width="1.83203125" style="2" hidden="1"/>
+    <col min="1803" max="1803" width="2.1640625" style="2" hidden="1"/>
+    <col min="1804" max="1804" width="0.83203125" style="2" hidden="1"/>
+    <col min="1805" max="1805" width="13.83203125" style="2" hidden="1"/>
+    <col min="1806" max="1806" width="3.1640625" style="2" hidden="1"/>
+    <col min="1807" max="1807" width="9.5" style="2" hidden="1"/>
+    <col min="1808" max="1808" width="12.1640625" style="2" hidden="1"/>
+    <col min="1809" max="1809" width="2.1640625" style="2" hidden="1"/>
+    <col min="1810" max="2049" width="9.1640625" style="2" hidden="1"/>
+    <col min="2050" max="2050" width="2.1640625" style="2" hidden="1"/>
+    <col min="2051" max="2051" width="1.83203125" style="2" hidden="1"/>
+    <col min="2052" max="2052" width="2.1640625" style="2" hidden="1"/>
+    <col min="2053" max="2053" width="0.83203125" style="2" hidden="1"/>
+    <col min="2054" max="2056" width="14.5" style="2" hidden="1"/>
+    <col min="2057" max="2057" width="3.1640625" style="2" hidden="1"/>
+    <col min="2058" max="2058" width="1.83203125" style="2" hidden="1"/>
+    <col min="2059" max="2059" width="2.1640625" style="2" hidden="1"/>
+    <col min="2060" max="2060" width="0.83203125" style="2" hidden="1"/>
+    <col min="2061" max="2061" width="13.83203125" style="2" hidden="1"/>
+    <col min="2062" max="2062" width="3.1640625" style="2" hidden="1"/>
+    <col min="2063" max="2063" width="9.5" style="2" hidden="1"/>
+    <col min="2064" max="2064" width="12.1640625" style="2" hidden="1"/>
+    <col min="2065" max="2065" width="2.1640625" style="2" hidden="1"/>
+    <col min="2066" max="2305" width="9.1640625" style="2" hidden="1"/>
+    <col min="2306" max="2306" width="2.1640625" style="2" hidden="1"/>
+    <col min="2307" max="2307" width="1.83203125" style="2" hidden="1"/>
+    <col min="2308" max="2308" width="2.1640625" style="2" hidden="1"/>
+    <col min="2309" max="2309" width="0.83203125" style="2" hidden="1"/>
+    <col min="2310" max="2312" width="14.5" style="2" hidden="1"/>
+    <col min="2313" max="2313" width="3.1640625" style="2" hidden="1"/>
+    <col min="2314" max="2314" width="1.83203125" style="2" hidden="1"/>
+    <col min="2315" max="2315" width="2.1640625" style="2" hidden="1"/>
+    <col min="2316" max="2316" width="0.83203125" style="2" hidden="1"/>
+    <col min="2317" max="2317" width="13.83203125" style="2" hidden="1"/>
+    <col min="2318" max="2318" width="3.1640625" style="2" hidden="1"/>
+    <col min="2319" max="2319" width="9.5" style="2" hidden="1"/>
+    <col min="2320" max="2320" width="12.1640625" style="2" hidden="1"/>
+    <col min="2321" max="2321" width="2.1640625" style="2" hidden="1"/>
+    <col min="2322" max="2561" width="9.1640625" style="2" hidden="1"/>
+    <col min="2562" max="2562" width="2.1640625" style="2" hidden="1"/>
+    <col min="2563" max="2563" width="1.83203125" style="2" hidden="1"/>
+    <col min="2564" max="2564" width="2.1640625" style="2" hidden="1"/>
+    <col min="2565" max="2565" width="0.83203125" style="2" hidden="1"/>
+    <col min="2566" max="2568" width="14.5" style="2" hidden="1"/>
+    <col min="2569" max="2569" width="3.1640625" style="2" hidden="1"/>
+    <col min="2570" max="2570" width="1.83203125" style="2" hidden="1"/>
+    <col min="2571" max="2571" width="2.1640625" style="2" hidden="1"/>
+    <col min="2572" max="2572" width="0.83203125" style="2" hidden="1"/>
+    <col min="2573" max="2573" width="13.83203125" style="2" hidden="1"/>
+    <col min="2574" max="2574" width="3.1640625" style="2" hidden="1"/>
+    <col min="2575" max="2575" width="9.5" style="2" hidden="1"/>
+    <col min="2576" max="2576" width="12.1640625" style="2" hidden="1"/>
+    <col min="2577" max="2577" width="2.1640625" style="2" hidden="1"/>
+    <col min="2578" max="2817" width="9.1640625" style="2" hidden="1"/>
+    <col min="2818" max="2818" width="2.1640625" style="2" hidden="1"/>
+    <col min="2819" max="2819" width="1.83203125" style="2" hidden="1"/>
+    <col min="2820" max="2820" width="2.1640625" style="2" hidden="1"/>
+    <col min="2821" max="2821" width="0.83203125" style="2" hidden="1"/>
+    <col min="2822" max="2824" width="14.5" style="2" hidden="1"/>
+    <col min="2825" max="2825" width="3.1640625" style="2" hidden="1"/>
+    <col min="2826" max="2826" width="1.83203125" style="2" hidden="1"/>
+    <col min="2827" max="2827" width="2.1640625" style="2" hidden="1"/>
+    <col min="2828" max="2828" width="0.83203125" style="2" hidden="1"/>
+    <col min="2829" max="2829" width="13.83203125" style="2" hidden="1"/>
+    <col min="2830" max="2830" width="3.1640625" style="2" hidden="1"/>
+    <col min="2831" max="2831" width="9.5" style="2" hidden="1"/>
+    <col min="2832" max="2832" width="12.1640625" style="2" hidden="1"/>
+    <col min="2833" max="2833" width="2.1640625" style="2" hidden="1"/>
+    <col min="2834" max="3073" width="9.1640625" style="2" hidden="1"/>
+    <col min="3074" max="3074" width="2.1640625" style="2" hidden="1"/>
+    <col min="3075" max="3075" width="1.83203125" style="2" hidden="1"/>
+    <col min="3076" max="3076" width="2.1640625" style="2" hidden="1"/>
+    <col min="3077" max="3077" width="0.83203125" style="2" hidden="1"/>
+    <col min="3078" max="3080" width="14.5" style="2" hidden="1"/>
+    <col min="3081" max="3081" width="3.1640625" style="2" hidden="1"/>
+    <col min="3082" max="3082" width="1.83203125" style="2" hidden="1"/>
+    <col min="3083" max="3083" width="2.1640625" style="2" hidden="1"/>
+    <col min="3084" max="3084" width="0.83203125" style="2" hidden="1"/>
+    <col min="3085" max="3085" width="13.83203125" style="2" hidden="1"/>
+    <col min="3086" max="3086" width="3.1640625" style="2" hidden="1"/>
+    <col min="3087" max="3087" width="9.5" style="2" hidden="1"/>
+    <col min="3088" max="3088" width="12.1640625" style="2" hidden="1"/>
+    <col min="3089" max="3089" width="2.1640625" style="2" hidden="1"/>
+    <col min="3090" max="3329" width="9.1640625" style="2" hidden="1"/>
+    <col min="3330" max="3330" width="2.1640625" style="2" hidden="1"/>
+    <col min="3331" max="3331" width="1.83203125" style="2" hidden="1"/>
+    <col min="3332" max="3332" width="2.1640625" style="2" hidden="1"/>
+    <col min="3333" max="3333" width="0.83203125" style="2" hidden="1"/>
+    <col min="3334" max="3336" width="14.5" style="2" hidden="1"/>
+    <col min="3337" max="3337" width="3.1640625" style="2" hidden="1"/>
+    <col min="3338" max="3338" width="1.83203125" style="2" hidden="1"/>
+    <col min="3339" max="3339" width="2.1640625" style="2" hidden="1"/>
+    <col min="3340" max="3340" width="0.83203125" style="2" hidden="1"/>
+    <col min="3341" max="3341" width="13.83203125" style="2" hidden="1"/>
+    <col min="3342" max="3342" width="3.1640625" style="2" hidden="1"/>
+    <col min="3343" max="3343" width="9.5" style="2" hidden="1"/>
+    <col min="3344" max="3344" width="12.1640625" style="2" hidden="1"/>
+    <col min="3345" max="3345" width="2.1640625" style="2" hidden="1"/>
+    <col min="3346" max="3585" width="9.1640625" style="2" hidden="1"/>
+    <col min="3586" max="3586" width="2.1640625" style="2" hidden="1"/>
+    <col min="3587" max="3587" width="1.83203125" style="2" hidden="1"/>
+    <col min="3588" max="3588" width="2.1640625" style="2" hidden="1"/>
+    <col min="3589" max="3589" width="0.83203125" style="2" hidden="1"/>
+    <col min="3590" max="3592" width="14.5" style="2" hidden="1"/>
+    <col min="3593" max="3593" width="3.1640625" style="2" hidden="1"/>
+    <col min="3594" max="3594" width="1.83203125" style="2" hidden="1"/>
+    <col min="3595" max="3595" width="2.1640625" style="2" hidden="1"/>
+    <col min="3596" max="3596" width="0.83203125" style="2" hidden="1"/>
+    <col min="3597" max="3597" width="13.83203125" style="2" hidden="1"/>
+    <col min="3598" max="3598" width="3.1640625" style="2" hidden="1"/>
+    <col min="3599" max="3599" width="9.5" style="2" hidden="1"/>
+    <col min="3600" max="3600" width="12.1640625" style="2" hidden="1"/>
+    <col min="3601" max="3601" width="2.1640625" style="2" hidden="1"/>
+    <col min="3602" max="3841" width="9.1640625" style="2" hidden="1"/>
+    <col min="3842" max="3842" width="2.1640625" style="2" hidden="1"/>
+    <col min="3843" max="3843" width="1.83203125" style="2" hidden="1"/>
+    <col min="3844" max="3844" width="2.1640625" style="2" hidden="1"/>
+    <col min="3845" max="3845" width="0.83203125" style="2" hidden="1"/>
+    <col min="3846" max="3848" width="14.5" style="2" hidden="1"/>
+    <col min="3849" max="3849" width="3.1640625" style="2" hidden="1"/>
+    <col min="3850" max="3850" width="1.83203125" style="2" hidden="1"/>
+    <col min="3851" max="3851" width="2.1640625" style="2" hidden="1"/>
+    <col min="3852" max="3852" width="0.83203125" style="2" hidden="1"/>
+    <col min="3853" max="3853" width="13.83203125" style="2" hidden="1"/>
+    <col min="3854" max="3854" width="3.1640625" style="2" hidden="1"/>
+    <col min="3855" max="3855" width="9.5" style="2" hidden="1"/>
+    <col min="3856" max="3856" width="12.1640625" style="2" hidden="1"/>
+    <col min="3857" max="3857" width="2.1640625" style="2" hidden="1"/>
+    <col min="3858" max="4097" width="9.1640625" style="2" hidden="1"/>
+    <col min="4098" max="4098" width="2.1640625" style="2" hidden="1"/>
+    <col min="4099" max="4099" width="1.83203125" style="2" hidden="1"/>
+    <col min="4100" max="4100" width="2.1640625" style="2" hidden="1"/>
+    <col min="4101" max="4101" width="0.83203125" style="2" hidden="1"/>
+    <col min="4102" max="4104" width="14.5" style="2" hidden="1"/>
+    <col min="4105" max="4105" width="3.1640625" style="2" hidden="1"/>
+    <col min="4106" max="4106" width="1.83203125" style="2" hidden="1"/>
+    <col min="4107" max="4107" width="2.1640625" style="2" hidden="1"/>
+    <col min="4108" max="4108" width="0.83203125" style="2" hidden="1"/>
+    <col min="4109" max="4109" width="13.83203125" style="2" hidden="1"/>
+    <col min="4110" max="4110" width="3.1640625" style="2" hidden="1"/>
+    <col min="4111" max="4111" width="9.5" style="2" hidden="1"/>
+    <col min="4112" max="4112" width="12.1640625" style="2" hidden="1"/>
+    <col min="4113" max="4113" width="2.1640625" style="2" hidden="1"/>
+    <col min="4114" max="4353" width="9.1640625" style="2" hidden="1"/>
+    <col min="4354" max="4354" width="2.1640625" style="2" hidden="1"/>
+    <col min="4355" max="4355" width="1.83203125" style="2" hidden="1"/>
+    <col min="4356" max="4356" width="2.1640625" style="2" hidden="1"/>
+    <col min="4357" max="4357" width="0.83203125" style="2" hidden="1"/>
+    <col min="4358" max="4360" width="14.5" style="2" hidden="1"/>
+    <col min="4361" max="4361" width="3.1640625" style="2" hidden="1"/>
+    <col min="4362" max="4362" width="1.83203125" style="2" hidden="1"/>
+    <col min="4363" max="4363" width="2.1640625" style="2" hidden="1"/>
+    <col min="4364" max="4364" width="0.83203125" style="2" hidden="1"/>
+    <col min="4365" max="4365" width="13.83203125" style="2" hidden="1"/>
+    <col min="4366" max="4366" width="3.1640625" style="2" hidden="1"/>
+    <col min="4367" max="4367" width="9.5" style="2" hidden="1"/>
+    <col min="4368" max="4368" width="12.1640625" style="2" hidden="1"/>
+    <col min="4369" max="4369" width="2.1640625" style="2" hidden="1"/>
+    <col min="4370" max="4609" width="9.1640625" style="2" hidden="1"/>
+    <col min="4610" max="4610" width="2.1640625" style="2" hidden="1"/>
+    <col min="4611" max="4611" width="1.83203125" style="2" hidden="1"/>
+    <col min="4612" max="4612" width="2.1640625" style="2" hidden="1"/>
+    <col min="4613" max="4613" width="0.83203125" style="2" hidden="1"/>
+    <col min="4614" max="4616" width="14.5" style="2" hidden="1"/>
+    <col min="4617" max="4617" width="3.1640625" style="2" hidden="1"/>
+    <col min="4618" max="4618" width="1.83203125" style="2" hidden="1"/>
+    <col min="4619" max="4619" width="2.1640625" style="2" hidden="1"/>
+    <col min="4620" max="4620" width="0.83203125" style="2" hidden="1"/>
+    <col min="4621" max="4621" width="13.83203125" style="2" hidden="1"/>
+    <col min="4622" max="4622" width="3.1640625" style="2" hidden="1"/>
+    <col min="4623" max="4623" width="9.5" style="2" hidden="1"/>
+    <col min="4624" max="4624" width="12.1640625" style="2" hidden="1"/>
+    <col min="4625" max="4625" width="2.1640625" style="2" hidden="1"/>
+    <col min="4626" max="4865" width="9.1640625" style="2" hidden="1"/>
+    <col min="4866" max="4866" width="2.1640625" style="2" hidden="1"/>
+    <col min="4867" max="4867" width="1.83203125" style="2" hidden="1"/>
+    <col min="4868" max="4868" width="2.1640625" style="2" hidden="1"/>
+    <col min="4869" max="4869" width="0.83203125" style="2" hidden="1"/>
+    <col min="4870" max="4872" width="14.5" style="2" hidden="1"/>
+    <col min="4873" max="4873" width="3.1640625" style="2" hidden="1"/>
+    <col min="4874" max="4874" width="1.83203125" style="2" hidden="1"/>
+    <col min="4875" max="4875" width="2.1640625" style="2" hidden="1"/>
+    <col min="4876" max="4876" width="0.83203125" style="2" hidden="1"/>
+    <col min="4877" max="4877" width="13.83203125" style="2" hidden="1"/>
+    <col min="4878" max="4878" width="3.1640625" style="2" hidden="1"/>
+    <col min="4879" max="4879" width="9.5" style="2" hidden="1"/>
+    <col min="4880" max="4880" width="12.1640625" style="2" hidden="1"/>
+    <col min="4881" max="4881" width="2.1640625" style="2" hidden="1"/>
+    <col min="4882" max="5121" width="9.1640625" style="2" hidden="1"/>
+    <col min="5122" max="5122" width="2.1640625" style="2" hidden="1"/>
+    <col min="5123" max="5123" width="1.83203125" style="2" hidden="1"/>
+    <col min="5124" max="5124" width="2.1640625" style="2" hidden="1"/>
+    <col min="5125" max="5125" width="0.83203125" style="2" hidden="1"/>
+    <col min="5126" max="5128" width="14.5" style="2" hidden="1"/>
+    <col min="5129" max="5129" width="3.1640625" style="2" hidden="1"/>
+    <col min="5130" max="5130" width="1.83203125" style="2" hidden="1"/>
+    <col min="5131" max="5131" width="2.1640625" style="2" hidden="1"/>
+    <col min="5132" max="5132" width="0.83203125" style="2" hidden="1"/>
+    <col min="5133" max="5133" width="13.83203125" style="2" hidden="1"/>
+    <col min="5134" max="5134" width="3.1640625" style="2" hidden="1"/>
+    <col min="5135" max="5135" width="9.5" style="2" hidden="1"/>
+    <col min="5136" max="5136" width="12.1640625" style="2" hidden="1"/>
+    <col min="5137" max="5137" width="2.1640625" style="2" hidden="1"/>
+    <col min="5138" max="5377" width="9.1640625" style="2" hidden="1"/>
+    <col min="5378" max="5378" width="2.1640625" style="2" hidden="1"/>
+    <col min="5379" max="5379" width="1.83203125" style="2" hidden="1"/>
+    <col min="5380" max="5380" width="2.1640625" style="2" hidden="1"/>
+    <col min="5381" max="5381" width="0.83203125" style="2" hidden="1"/>
+    <col min="5382" max="5384" width="14.5" style="2" hidden="1"/>
+    <col min="5385" max="5385" width="3.1640625" style="2" hidden="1"/>
+    <col min="5386" max="5386" width="1.83203125" style="2" hidden="1"/>
+    <col min="5387" max="5387" width="2.1640625" style="2" hidden="1"/>
+    <col min="5388" max="5388" width="0.83203125" style="2" hidden="1"/>
+    <col min="5389" max="5389" width="13.83203125" style="2" hidden="1"/>
+    <col min="5390" max="5390" width="3.1640625" style="2" hidden="1"/>
+    <col min="5391" max="5391" width="9.5" style="2" hidden="1"/>
+    <col min="5392" max="5392" width="12.1640625" style="2" hidden="1"/>
+    <col min="5393" max="5393" width="2.1640625" style="2" hidden="1"/>
+    <col min="5394" max="5633" width="9.1640625" style="2" hidden="1"/>
+    <col min="5634" max="5634" width="2.1640625" style="2" hidden="1"/>
+    <col min="5635" max="5635" width="1.83203125" style="2" hidden="1"/>
+    <col min="5636" max="5636" width="2.1640625" style="2" hidden="1"/>
+    <col min="5637" max="5637" width="0.83203125" style="2" hidden="1"/>
+    <col min="5638" max="5640" width="14.5" style="2" hidden="1"/>
+    <col min="5641" max="5641" width="3.1640625" style="2" hidden="1"/>
+    <col min="5642" max="5642" width="1.83203125" style="2" hidden="1"/>
+    <col min="5643" max="5643" width="2.1640625" style="2" hidden="1"/>
+    <col min="5644" max="5644" width="0.83203125" style="2" hidden="1"/>
+    <col min="5645" max="5645" width="13.83203125" style="2" hidden="1"/>
+    <col min="5646" max="5646" width="3.1640625" style="2" hidden="1"/>
+    <col min="5647" max="5647" width="9.5" style="2" hidden="1"/>
+    <col min="5648" max="5648" width="12.1640625" style="2" hidden="1"/>
+    <col min="5649" max="5649" width="2.1640625" style="2" hidden="1"/>
+    <col min="5650" max="5889" width="9.1640625" style="2" hidden="1"/>
+    <col min="5890" max="5890" width="2.1640625" style="2" hidden="1"/>
+    <col min="5891" max="5891" width="1.83203125" style="2" hidden="1"/>
+    <col min="5892" max="5892" width="2.1640625" style="2" hidden="1"/>
+    <col min="5893" max="5893" width="0.83203125" style="2" hidden="1"/>
+    <col min="5894" max="5896" width="14.5" style="2" hidden="1"/>
+    <col min="5897" max="5897" width="3.1640625" style="2" hidden="1"/>
+    <col min="5898" max="5898" width="1.83203125" style="2" hidden="1"/>
+    <col min="5899" max="5899" width="2.1640625" style="2" hidden="1"/>
+    <col min="5900" max="5900" width="0.83203125" style="2" hidden="1"/>
+    <col min="5901" max="5901" width="13.83203125" style="2" hidden="1"/>
+    <col min="5902" max="5902" width="3.1640625" style="2" hidden="1"/>
+    <col min="5903" max="5903" width="9.5" style="2" hidden="1"/>
+    <col min="5904" max="5904" width="12.1640625" style="2" hidden="1"/>
+    <col min="5905" max="5905" width="2.1640625" style="2" hidden="1"/>
+    <col min="5906" max="6145" width="9.1640625" style="2" hidden="1"/>
+    <col min="6146" max="6146" width="2.1640625" style="2" hidden="1"/>
+    <col min="6147" max="6147" width="1.83203125" style="2" hidden="1"/>
+    <col min="6148" max="6148" width="2.1640625" style="2" hidden="1"/>
+    <col min="6149" max="6149" width="0.83203125" style="2" hidden="1"/>
+    <col min="6150" max="6152" width="14.5" style="2" hidden="1"/>
+    <col min="6153" max="6153" width="3.1640625" style="2" hidden="1"/>
+    <col min="6154" max="6154" width="1.83203125" style="2" hidden="1"/>
+    <col min="6155" max="6155" width="2.1640625" style="2" hidden="1"/>
+    <col min="6156" max="6156" width="0.83203125" style="2" hidden="1"/>
+    <col min="6157" max="6157" width="13.83203125" style="2" hidden="1"/>
+    <col min="6158" max="6158" width="3.1640625" style="2" hidden="1"/>
+    <col min="6159" max="6159" width="9.5" style="2" hidden="1"/>
+    <col min="6160" max="6160" width="12.1640625" style="2" hidden="1"/>
+    <col min="6161" max="6161" width="2.1640625" style="2" hidden="1"/>
+    <col min="6162" max="6401" width="9.1640625" style="2" hidden="1"/>
+    <col min="6402" max="6402" width="2.1640625" style="2" hidden="1"/>
+    <col min="6403" max="6403" width="1.83203125" style="2" hidden="1"/>
+    <col min="6404" max="6404" width="2.1640625" style="2" hidden="1"/>
+    <col min="6405" max="6405" width="0.83203125" style="2" hidden="1"/>
+    <col min="6406" max="6408" width="14.5" style="2" hidden="1"/>
+    <col min="6409" max="6409" width="3.1640625" style="2" hidden="1"/>
+    <col min="6410" max="6410" width="1.83203125" style="2" hidden="1"/>
+    <col min="6411" max="6411" width="2.1640625" style="2" hidden="1"/>
+    <col min="6412" max="6412" width="0.83203125" style="2" hidden="1"/>
+    <col min="6413" max="6413" width="13.83203125" style="2" hidden="1"/>
+    <col min="6414" max="6414" width="3.1640625" style="2" hidden="1"/>
+    <col min="6415" max="6415" width="9.5" style="2" hidden="1"/>
+    <col min="6416" max="6416" width="12.1640625" style="2" hidden="1"/>
+    <col min="6417" max="6417" width="2.1640625" style="2" hidden="1"/>
+    <col min="6418" max="6657" width="9.1640625" style="2" hidden="1"/>
+    <col min="6658" max="6658" width="2.1640625" style="2" hidden="1"/>
+    <col min="6659" max="6659" width="1.83203125" style="2" hidden="1"/>
+    <col min="6660" max="6660" width="2.1640625" style="2" hidden="1"/>
+    <col min="6661" max="6661" width="0.83203125" style="2" hidden="1"/>
+    <col min="6662" max="6664" width="14.5" style="2" hidden="1"/>
+    <col min="6665" max="6665" width="3.1640625" style="2" hidden="1"/>
+    <col min="6666" max="6666" width="1.83203125" style="2" hidden="1"/>
+    <col min="6667" max="6667" width="2.1640625" style="2" hidden="1"/>
+    <col min="6668" max="6668" width="0.83203125" style="2" hidden="1"/>
+    <col min="6669" max="6669" width="13.83203125" style="2" hidden="1"/>
+    <col min="6670" max="6670" width="3.1640625" style="2" hidden="1"/>
+    <col min="6671" max="6671" width="9.5" style="2" hidden="1"/>
+    <col min="6672" max="6672" width="12.1640625" style="2" hidden="1"/>
+    <col min="6673" max="6673" width="2.1640625" style="2" hidden="1"/>
+    <col min="6674" max="6913" width="9.1640625" style="2" hidden="1"/>
+    <col min="6914" max="6914" width="2.1640625" style="2" hidden="1"/>
+    <col min="6915" max="6915" width="1.83203125" style="2" hidden="1"/>
+    <col min="6916" max="6916" width="2.1640625" style="2" hidden="1"/>
+    <col min="6917" max="6917" width="0.83203125" style="2" hidden="1"/>
+    <col min="6918" max="6920" width="14.5" style="2" hidden="1"/>
+    <col min="6921" max="6921" width="3.1640625" style="2" hidden="1"/>
+    <col min="6922" max="6922" width="1.83203125" style="2" hidden="1"/>
+    <col min="6923" max="6923" width="2.1640625" style="2" hidden="1"/>
+    <col min="6924" max="6924" width="0.83203125" style="2" hidden="1"/>
+    <col min="6925" max="6925" width="13.83203125" style="2" hidden="1"/>
+    <col min="6926" max="6926" width="3.1640625" style="2" hidden="1"/>
+    <col min="6927" max="6927" width="9.5" style="2" hidden="1"/>
+    <col min="6928" max="6928" width="12.1640625" style="2" hidden="1"/>
+    <col min="6929" max="6929" width="2.1640625" style="2" hidden="1"/>
+    <col min="6930" max="7169" width="9.1640625" style="2" hidden="1"/>
+    <col min="7170" max="7170" width="2.1640625" style="2" hidden="1"/>
+    <col min="7171" max="7171" width="1.83203125" style="2" hidden="1"/>
+    <col min="7172" max="7172" width="2.1640625" style="2" hidden="1"/>
+    <col min="7173" max="7173" width="0.83203125" style="2" hidden="1"/>
+    <col min="7174" max="7176" width="14.5" style="2" hidden="1"/>
+    <col min="7177" max="7177" width="3.1640625" style="2" hidden="1"/>
+    <col min="7178" max="7178" width="1.83203125" style="2" hidden="1"/>
+    <col min="7179" max="7179" width="2.1640625" style="2" hidden="1"/>
+    <col min="7180" max="7180" width="0.83203125" style="2" hidden="1"/>
+    <col min="7181" max="7181" width="13.83203125" style="2" hidden="1"/>
+    <col min="7182" max="7182" width="3.1640625" style="2" hidden="1"/>
+    <col min="7183" max="7183" width="9.5" style="2" hidden="1"/>
+    <col min="7184" max="7184" width="12.1640625" style="2" hidden="1"/>
+    <col min="7185" max="7185" width="2.1640625" style="2" hidden="1"/>
+    <col min="7186" max="7425" width="9.1640625" style="2" hidden="1"/>
+    <col min="7426" max="7426" width="2.1640625" style="2" hidden="1"/>
+    <col min="7427" max="7427" width="1.83203125" style="2" hidden="1"/>
+    <col min="7428" max="7428" width="2.1640625" style="2" hidden="1"/>
+    <col min="7429" max="7429" width="0.83203125" style="2" hidden="1"/>
+    <col min="7430" max="7432" width="14.5" style="2" hidden="1"/>
+    <col min="7433" max="7433" width="3.1640625" style="2" hidden="1"/>
+    <col min="7434" max="7434" width="1.83203125" style="2" hidden="1"/>
+    <col min="7435" max="7435" width="2.1640625" style="2" hidden="1"/>
+    <col min="7436" max="7436" width="0.83203125" style="2" hidden="1"/>
+    <col min="7437" max="7437" width="13.83203125" style="2" hidden="1"/>
+    <col min="7438" max="7438" width="3.1640625" style="2" hidden="1"/>
+    <col min="7439" max="7439" width="9.5" style="2" hidden="1"/>
+    <col min="7440" max="7440" width="12.1640625" style="2" hidden="1"/>
+    <col min="7441" max="7441" width="2.1640625" style="2" hidden="1"/>
+    <col min="7442" max="7681" width="9.1640625" style="2" hidden="1"/>
+    <col min="7682" max="7682" width="2.1640625" style="2" hidden="1"/>
+    <col min="7683" max="7683" width="1.83203125" style="2" hidden="1"/>
+    <col min="7684" max="7684" width="2.1640625" style="2" hidden="1"/>
+    <col min="7685" max="7685" width="0.83203125" style="2" hidden="1"/>
+    <col min="7686" max="7688" width="14.5" style="2" hidden="1"/>
+    <col min="7689" max="7689" width="3.1640625" style="2" hidden="1"/>
+    <col min="7690" max="7690" width="1.83203125" style="2" hidden="1"/>
+    <col min="7691" max="7691" width="2.1640625" style="2" hidden="1"/>
+    <col min="7692" max="7692" width="0.83203125" style="2" hidden="1"/>
+    <col min="7693" max="7693" width="13.83203125" style="2" hidden="1"/>
+    <col min="7694" max="7694" width="3.1640625" style="2" hidden="1"/>
+    <col min="7695" max="7695" width="9.5" style="2" hidden="1"/>
+    <col min="7696" max="7696" width="12.1640625" style="2" hidden="1"/>
+    <col min="7697" max="7697" width="2.1640625" style="2" hidden="1"/>
+    <col min="7698" max="7937" width="9.1640625" style="2" hidden="1"/>
+    <col min="7938" max="7938" width="2.1640625" style="2" hidden="1"/>
+    <col min="7939" max="7939" width="1.83203125" style="2" hidden="1"/>
+    <col min="7940" max="7940" width="2.1640625" style="2" hidden="1"/>
+    <col min="7941" max="7941" width="0.83203125" style="2" hidden="1"/>
+    <col min="7942" max="7944" width="14.5" style="2" hidden="1"/>
+    <col min="7945" max="7945" width="3.1640625" style="2" hidden="1"/>
+    <col min="7946" max="7946" width="1.83203125" style="2" hidden="1"/>
+    <col min="7947" max="7947" width="2.1640625" style="2" hidden="1"/>
+    <col min="7948" max="7948" width="0.83203125" style="2" hidden="1"/>
+    <col min="7949" max="7949" width="13.83203125" style="2" hidden="1"/>
+    <col min="7950" max="7950" width="3.1640625" style="2" hidden="1"/>
+    <col min="7951" max="7951" width="9.5" style="2" hidden="1"/>
+    <col min="7952" max="7952" width="12.1640625" style="2" hidden="1"/>
+    <col min="7953" max="7953" width="2.1640625" style="2" hidden="1"/>
+    <col min="7954" max="8193" width="9.1640625" style="2" hidden="1"/>
+    <col min="8194" max="8194" width="2.1640625" style="2" hidden="1"/>
+    <col min="8195" max="8195" width="1.83203125" style="2" hidden="1"/>
+    <col min="8196" max="8196" width="2.1640625" style="2" hidden="1"/>
+    <col min="8197" max="8197" width="0.83203125" style="2" hidden="1"/>
+    <col min="8198" max="8200" width="14.5" style="2" hidden="1"/>
+    <col min="8201" max="8201" width="3.1640625" style="2" hidden="1"/>
+    <col min="8202" max="8202" width="1.83203125" style="2" hidden="1"/>
+    <col min="8203" max="8203" width="2.1640625" style="2" hidden="1"/>
+    <col min="8204" max="8204" width="0.83203125" style="2" hidden="1"/>
+    <col min="8205" max="8205" width="13.83203125" style="2" hidden="1"/>
+    <col min="8206" max="8206" width="3.1640625" style="2" hidden="1"/>
+    <col min="8207" max="8207" width="9.5" style="2" hidden="1"/>
+    <col min="8208" max="8208" width="12.1640625" style="2" hidden="1"/>
+    <col min="8209" max="8209" width="2.1640625" style="2" hidden="1"/>
+    <col min="8210" max="8449" width="9.1640625" style="2" hidden="1"/>
+    <col min="8450" max="8450" width="2.1640625" style="2" hidden="1"/>
+    <col min="8451" max="8451" width="1.83203125" style="2" hidden="1"/>
+    <col min="8452" max="8452" width="2.1640625" style="2" hidden="1"/>
+    <col min="8453" max="8453" width="0.83203125" style="2" hidden="1"/>
+    <col min="8454" max="8456" width="14.5" style="2" hidden="1"/>
+    <col min="8457" max="8457" width="3.1640625" style="2" hidden="1"/>
+    <col min="8458" max="8458" width="1.83203125" style="2" hidden="1"/>
+    <col min="8459" max="8459" width="2.1640625" style="2" hidden="1"/>
+    <col min="8460" max="8460" width="0.83203125" style="2" hidden="1"/>
+    <col min="8461" max="8461" width="13.83203125" style="2" hidden="1"/>
+    <col min="8462" max="8462" width="3.1640625" style="2" hidden="1"/>
+    <col min="8463" max="8463" width="9.5" style="2" hidden="1"/>
+    <col min="8464" max="8464" width="12.1640625" style="2" hidden="1"/>
+    <col min="8465" max="8465" width="2.1640625" style="2" hidden="1"/>
+    <col min="8466" max="8705" width="9.1640625" style="2" hidden="1"/>
+    <col min="8706" max="8706" width="2.1640625" style="2" hidden="1"/>
+    <col min="8707" max="8707" width="1.83203125" style="2" hidden="1"/>
+    <col min="8708" max="8708" width="2.1640625" style="2" hidden="1"/>
+    <col min="8709" max="8709" width="0.83203125" style="2" hidden="1"/>
+    <col min="8710" max="8712" width="14.5" style="2" hidden="1"/>
+    <col min="8713" max="8713" width="3.1640625" style="2" hidden="1"/>
+    <col min="8714" max="8714" width="1.83203125" style="2" hidden="1"/>
+    <col min="8715" max="8715" width="2.1640625" style="2" hidden="1"/>
+    <col min="8716" max="8716" width="0.83203125" style="2" hidden="1"/>
+    <col min="8717" max="8717" width="13.83203125" style="2" hidden="1"/>
+    <col min="8718" max="8718" width="3.1640625" style="2" hidden="1"/>
+    <col min="8719" max="8719" width="9.5" style="2" hidden="1"/>
+    <col min="8720" max="8720" width="12.1640625" style="2" hidden="1"/>
+    <col min="8721" max="8721" width="2.1640625" style="2" hidden="1"/>
+    <col min="8722" max="8961" width="9.1640625" style="2" hidden="1"/>
+    <col min="8962" max="8962" width="2.1640625" style="2" hidden="1"/>
+    <col min="8963" max="8963" width="1.83203125" style="2" hidden="1"/>
+    <col min="8964" max="8964" width="2.1640625" style="2" hidden="1"/>
+    <col min="8965" max="8965" width="0.83203125" style="2" hidden="1"/>
+    <col min="8966" max="8968" width="14.5" style="2" hidden="1"/>
+    <col min="8969" max="8969" width="3.1640625" style="2" hidden="1"/>
+    <col min="8970" max="8970" width="1.83203125" style="2" hidden="1"/>
+    <col min="8971" max="8971" width="2.1640625" style="2" hidden="1"/>
+    <col min="8972" max="8972" width="0.83203125" style="2" hidden="1"/>
+    <col min="8973" max="8973" width="13.83203125" style="2" hidden="1"/>
+    <col min="8974" max="8974" width="3.1640625" style="2" hidden="1"/>
+    <col min="8975" max="8975" width="9.5" style="2" hidden="1"/>
+    <col min="8976" max="8976" width="12.1640625" style="2" hidden="1"/>
+    <col min="8977" max="8977" width="2.1640625" style="2" hidden="1"/>
+    <col min="8978" max="9217" width="9.1640625" style="2" hidden="1"/>
+    <col min="9218" max="9218" width="2.1640625" style="2" hidden="1"/>
+    <col min="9219" max="9219" width="1.83203125" style="2" hidden="1"/>
+    <col min="9220" max="9220" width="2.1640625" style="2" hidden="1"/>
+    <col min="9221" max="9221" width="0.83203125" style="2" hidden="1"/>
+    <col min="9222" max="9224" width="14.5" style="2" hidden="1"/>
+    <col min="9225" max="9225" width="3.1640625" style="2" hidden="1"/>
+    <col min="9226" max="9226" width="1.83203125" style="2" hidden="1"/>
+    <col min="9227" max="9227" width="2.1640625" style="2" hidden="1"/>
+    <col min="9228" max="9228" width="0.83203125" style="2" hidden="1"/>
+    <col min="9229" max="9229" width="13.83203125" style="2" hidden="1"/>
+    <col min="9230" max="9230" width="3.1640625" style="2" hidden="1"/>
+    <col min="9231" max="9231" width="9.5" style="2" hidden="1"/>
+    <col min="9232" max="9232" width="12.1640625" style="2" hidden="1"/>
+    <col min="9233" max="9233" width="2.1640625" style="2" hidden="1"/>
+    <col min="9234" max="9473" width="9.1640625" style="2" hidden="1"/>
+    <col min="9474" max="9474" width="2.1640625" style="2" hidden="1"/>
+    <col min="9475" max="9475" width="1.83203125" style="2" hidden="1"/>
+    <col min="9476" max="9476" width="2.1640625" style="2" hidden="1"/>
+    <col min="9477" max="9477" width="0.83203125" style="2" hidden="1"/>
+    <col min="9478" max="9480" width="14.5" style="2" hidden="1"/>
+    <col min="9481" max="9481" width="3.1640625" style="2" hidden="1"/>
+    <col min="9482" max="9482" width="1.83203125" style="2" hidden="1"/>
+    <col min="9483" max="9483" width="2.1640625" style="2" hidden="1"/>
+    <col min="9484" max="9484" width="0.83203125" style="2" hidden="1"/>
+    <col min="9485" max="9485" width="13.83203125" style="2" hidden="1"/>
+    <col min="9486" max="9486" width="3.1640625" style="2" hidden="1"/>
+    <col min="9487" max="9487" width="9.5" style="2" hidden="1"/>
+    <col min="9488" max="9488" width="12.1640625" style="2" hidden="1"/>
+    <col min="9489" max="9489" width="2.1640625" style="2" hidden="1"/>
+    <col min="9490" max="9729" width="9.1640625" style="2" hidden="1"/>
+    <col min="9730" max="9730" width="2.1640625" style="2" hidden="1"/>
+    <col min="9731" max="9731" width="1.83203125" style="2" hidden="1"/>
+    <col min="9732" max="9732" width="2.1640625" style="2" hidden="1"/>
+    <col min="9733" max="9733" width="0.83203125" style="2" hidden="1"/>
+    <col min="9734" max="9736" width="14.5" style="2" hidden="1"/>
+    <col min="9737" max="9737" width="3.1640625" style="2" hidden="1"/>
+    <col min="9738" max="9738" width="1.83203125" style="2" hidden="1"/>
+    <col min="9739" max="9739" width="2.1640625" style="2" hidden="1"/>
+    <col min="9740" max="9740" width="0.83203125" style="2" hidden="1"/>
+    <col min="9741" max="9741" width="13.83203125" style="2" hidden="1"/>
+    <col min="9742" max="9742" width="3.1640625" style="2" hidden="1"/>
+    <col min="9743" max="9743" width="9.5" style="2" hidden="1"/>
+    <col min="9744" max="9744" width="12.1640625" style="2" hidden="1"/>
+    <col min="9745" max="9745" width="2.1640625" style="2" hidden="1"/>
+    <col min="9746" max="9985" width="9.1640625" style="2" hidden="1"/>
+    <col min="9986" max="9986" width="2.1640625" style="2" hidden="1"/>
+    <col min="9987" max="9987" width="1.83203125" style="2" hidden="1"/>
+    <col min="9988" max="9988" width="2.1640625" style="2" hidden="1"/>
+    <col min="9989" max="9989" width="0.83203125" style="2" hidden="1"/>
+    <col min="9990" max="9992" width="14.5" style="2" hidden="1"/>
+    <col min="9993" max="9993" width="3.1640625" style="2" hidden="1"/>
+    <col min="9994" max="9994" width="1.83203125" style="2" hidden="1"/>
+    <col min="9995" max="9995" width="2.1640625" style="2" hidden="1"/>
+    <col min="9996" max="9996" width="0.83203125" style="2" hidden="1"/>
+    <col min="9997" max="9997" width="13.83203125" style="2" hidden="1"/>
+    <col min="9998" max="9998" width="3.1640625" style="2" hidden="1"/>
+    <col min="9999" max="9999" width="9.5" style="2" hidden="1"/>
+    <col min="10000" max="10000" width="12.1640625" style="2" hidden="1"/>
+    <col min="10001" max="10001" width="2.1640625" style="2" hidden="1"/>
+    <col min="10002" max="10241" width="9.1640625" style="2" hidden="1"/>
+    <col min="10242" max="10242" width="2.1640625" style="2" hidden="1"/>
+    <col min="10243" max="10243" width="1.83203125" style="2" hidden="1"/>
+    <col min="10244" max="10244" width="2.1640625" style="2" hidden="1"/>
+    <col min="10245" max="10245" width="0.83203125" style="2" hidden="1"/>
+    <col min="10246" max="10248" width="14.5" style="2" hidden="1"/>
+    <col min="10249" max="10249" width="3.1640625" style="2" hidden="1"/>
+    <col min="10250" max="10250" width="1.83203125" style="2" hidden="1"/>
+    <col min="10251" max="10251" width="2.1640625" style="2" hidden="1"/>
+    <col min="10252" max="10252" width="0.83203125" style="2" hidden="1"/>
+    <col min="10253" max="10253" width="13.83203125" style="2" hidden="1"/>
+    <col min="10254" max="10254" width="3.1640625" style="2" hidden="1"/>
+    <col min="10255" max="10255" width="9.5" style="2" hidden="1"/>
+    <col min="10256" max="10256" width="12.1640625" style="2" hidden="1"/>
+    <col min="10257" max="10257" width="2.1640625" style="2" hidden="1"/>
+    <col min="10258" max="10497" width="9.1640625" style="2" hidden="1"/>
+    <col min="10498" max="10498" width="2.1640625" style="2" hidden="1"/>
+    <col min="10499" max="10499" width="1.83203125" style="2" hidden="1"/>
+    <col min="10500" max="10500" width="2.1640625" style="2" hidden="1"/>
+    <col min="10501" max="10501" width="0.83203125" style="2" hidden="1"/>
+    <col min="10502" max="10504" width="14.5" style="2" hidden="1"/>
+    <col min="10505" max="10505" width="3.1640625" style="2" hidden="1"/>
+    <col min="10506" max="10506" width="1.83203125" style="2" hidden="1"/>
+    <col min="10507" max="10507" width="2.1640625" style="2" hidden="1"/>
+    <col min="10508" max="10508" width="0.83203125" style="2" hidden="1"/>
+    <col min="10509" max="10509" width="13.83203125" style="2" hidden="1"/>
+    <col min="10510" max="10510" width="3.1640625" style="2" hidden="1"/>
+    <col min="10511" max="10511" width="9.5" style="2" hidden="1"/>
+    <col min="10512" max="10512" width="12.1640625" style="2" hidden="1"/>
+    <col min="10513" max="10513" width="2.1640625" style="2" hidden="1"/>
+    <col min="10514" max="10753" width="9.1640625" style="2" hidden="1"/>
+    <col min="10754" max="10754" width="2.1640625" style="2" hidden="1"/>
+    <col min="10755" max="10755" width="1.83203125" style="2" hidden="1"/>
+    <col min="10756" max="10756" width="2.1640625" style="2" hidden="1"/>
+    <col min="10757" max="10757" width="0.83203125" style="2" hidden="1"/>
+    <col min="10758" max="10760" width="14.5" style="2" hidden="1"/>
+    <col min="10761" max="10761" width="3.1640625" style="2" hidden="1"/>
+    <col min="10762" max="10762" width="1.83203125" style="2" hidden="1"/>
+    <col min="10763" max="10763" width="2.1640625" style="2" hidden="1"/>
+    <col min="10764" max="10764" width="0.83203125" style="2" hidden="1"/>
+    <col min="10765" max="10765" width="13.83203125" style="2" hidden="1"/>
+    <col min="10766" max="10766" width="3.1640625" style="2" hidden="1"/>
+    <col min="10767" max="10767" width="9.5" style="2" hidden="1"/>
+    <col min="10768" max="10768" width="12.1640625" style="2" hidden="1"/>
+    <col min="10769" max="10769" width="2.1640625" style="2" hidden="1"/>
+    <col min="10770" max="11009" width="9.1640625" style="2" hidden="1"/>
+    <col min="11010" max="11010" width="2.1640625" style="2" hidden="1"/>
+    <col min="11011" max="11011" width="1.83203125" style="2" hidden="1"/>
+    <col min="11012" max="11012" width="2.1640625" style="2" hidden="1"/>
+    <col min="11013" max="11013" width="0.83203125" style="2" hidden="1"/>
+    <col min="11014" max="11016" width="14.5" style="2" hidden="1"/>
+    <col min="11017" max="11017" width="3.1640625" style="2" hidden="1"/>
+    <col min="11018" max="11018" width="1.83203125" style="2" hidden="1"/>
+    <col min="11019" max="11019" width="2.1640625" style="2" hidden="1"/>
+    <col min="11020" max="11020" width="0.83203125" style="2" hidden="1"/>
+    <col min="11021" max="11021" width="13.83203125" style="2" hidden="1"/>
+    <col min="11022" max="11022" width="3.1640625" style="2" hidden="1"/>
+    <col min="11023" max="11023" width="9.5" style="2" hidden="1"/>
+    <col min="11024" max="11024" width="12.1640625" style="2" hidden="1"/>
+    <col min="11025" max="11025" width="2.1640625" style="2" hidden="1"/>
+    <col min="11026" max="11265" width="9.1640625" style="2" hidden="1"/>
+    <col min="11266" max="11266" width="2.1640625" style="2" hidden="1"/>
+    <col min="11267" max="11267" width="1.83203125" style="2" hidden="1"/>
+    <col min="11268" max="11268" width="2.1640625" style="2" hidden="1"/>
+    <col min="11269" max="11269" width="0.83203125" style="2" hidden="1"/>
+    <col min="11270" max="11272" width="14.5" style="2" hidden="1"/>
+    <col min="11273" max="11273" width="3.1640625" style="2" hidden="1"/>
+    <col min="11274" max="11274" width="1.83203125" style="2" hidden="1"/>
+    <col min="11275" max="11275" width="2.1640625" style="2" hidden="1"/>
+    <col min="11276" max="11276" width="0.83203125" style="2" hidden="1"/>
+    <col min="11277" max="11277" width="13.83203125" style="2" hidden="1"/>
+    <col min="11278" max="11278" width="3.1640625" style="2" hidden="1"/>
+    <col min="11279" max="11279" width="9.5" style="2" hidden="1"/>
+    <col min="11280" max="11280" width="12.1640625" style="2" hidden="1"/>
+    <col min="11281" max="11281" width="2.1640625" style="2" hidden="1"/>
+    <col min="11282" max="11521" width="9.1640625" style="2" hidden="1"/>
+    <col min="11522" max="11522" width="2.1640625" style="2" hidden="1"/>
+    <col min="11523" max="11523" width="1.83203125" style="2" hidden="1"/>
+    <col min="11524" max="11524" width="2.1640625" style="2" hidden="1"/>
+    <col min="11525" max="11525" width="0.83203125" style="2" hidden="1"/>
+    <col min="11526" max="11528" width="14.5" style="2" hidden="1"/>
+    <col min="11529" max="11529" width="3.1640625" style="2" hidden="1"/>
+    <col min="11530" max="11530" width="1.83203125" style="2" hidden="1"/>
+    <col min="11531" max="11531" width="2.1640625" style="2" hidden="1"/>
+    <col min="11532" max="11532" width="0.83203125" style="2" hidden="1"/>
+    <col min="11533" max="11533" width="13.83203125" style="2" hidden="1"/>
+    <col min="11534" max="11534" width="3.1640625" style="2" hidden="1"/>
+    <col min="11535" max="11535" width="9.5" style="2" hidden="1"/>
+    <col min="11536" max="11536" width="12.1640625" style="2" hidden="1"/>
+    <col min="11537" max="11537" width="2.1640625" style="2" hidden="1"/>
+    <col min="11538" max="11777" width="9.1640625" style="2" hidden="1"/>
+    <col min="11778" max="11778" width="2.1640625" style="2" hidden="1"/>
+    <col min="11779" max="11779" width="1.83203125" style="2" hidden="1"/>
+    <col min="11780" max="11780" width="2.1640625" style="2" hidden="1"/>
+    <col min="11781" max="11781" width="0.83203125" style="2" hidden="1"/>
+    <col min="11782" max="11784" width="14.5" style="2" hidden="1"/>
+    <col min="11785" max="11785" width="3.1640625" style="2" hidden="1"/>
+    <col min="11786" max="11786" width="1.83203125" style="2" hidden="1"/>
+    <col min="11787" max="11787" width="2.1640625" style="2" hidden="1"/>
+    <col min="11788" max="11788" width="0.83203125" style="2" hidden="1"/>
+    <col min="11789" max="11789" width="13.83203125" style="2" hidden="1"/>
+    <col min="11790" max="11790" width="3.1640625" style="2" hidden="1"/>
+    <col min="11791" max="11791" width="9.5" style="2" hidden="1"/>
+    <col min="11792" max="11792" width="12.1640625" style="2" hidden="1"/>
+    <col min="11793" max="11793" width="2.1640625" style="2" hidden="1"/>
+    <col min="11794" max="12033" width="9.1640625" style="2" hidden="1"/>
+    <col min="12034" max="12034" width="2.1640625" style="2" hidden="1"/>
+    <col min="12035" max="12035" width="1.83203125" style="2" hidden="1"/>
+    <col min="12036" max="12036" width="2.1640625" style="2" hidden="1"/>
+    <col min="12037" max="12037" width="0.83203125" style="2" hidden="1"/>
+    <col min="12038" max="12040" width="14.5" style="2" hidden="1"/>
+    <col min="12041" max="12041" width="3.1640625" style="2" hidden="1"/>
+    <col min="12042" max="12042" width="1.83203125" style="2" hidden="1"/>
+    <col min="12043" max="12043" width="2.1640625" style="2" hidden="1"/>
+    <col min="12044" max="12044" width="0.83203125" style="2" hidden="1"/>
+    <col min="12045" max="12045" width="13.83203125" style="2" hidden="1"/>
+    <col min="12046" max="12046" width="3.1640625" style="2" hidden="1"/>
+    <col min="12047" max="12047" width="9.5" style="2" hidden="1"/>
+    <col min="12048" max="12048" width="12.1640625" style="2" hidden="1"/>
+    <col min="12049" max="12049" width="2.1640625" style="2" hidden="1"/>
+    <col min="12050" max="12289" width="9.1640625" style="2" hidden="1"/>
+    <col min="12290" max="12290" width="2.1640625" style="2" hidden="1"/>
+    <col min="12291" max="12291" width="1.83203125" style="2" hidden="1"/>
+    <col min="12292" max="12292" width="2.1640625" style="2" hidden="1"/>
+    <col min="12293" max="12293" width="0.83203125" style="2" hidden="1"/>
+    <col min="12294" max="12296" width="14.5" style="2" hidden="1"/>
+    <col min="12297" max="12297" width="3.1640625" style="2" hidden="1"/>
+    <col min="12298" max="12298" width="1.83203125" style="2" hidden="1"/>
+    <col min="12299" max="12299" width="2.1640625" style="2" hidden="1"/>
+    <col min="12300" max="12300" width="0.83203125" style="2" hidden="1"/>
+    <col min="12301" max="12301" width="13.83203125" style="2" hidden="1"/>
+    <col min="12302" max="12302" width="3.1640625" style="2" hidden="1"/>
+    <col min="12303" max="12303" width="9.5" style="2" hidden="1"/>
+    <col min="12304" max="12304" width="12.1640625" style="2" hidden="1"/>
+    <col min="12305" max="12305" width="2.1640625" style="2" hidden="1"/>
+    <col min="12306" max="12545" width="9.1640625" style="2" hidden="1"/>
+    <col min="12546" max="12546" width="2.1640625" style="2" hidden="1"/>
+    <col min="12547" max="12547" width="1.83203125" style="2" hidden="1"/>
+    <col min="12548" max="12548" width="2.1640625" style="2" hidden="1"/>
+    <col min="12549" max="12549" width="0.83203125" style="2" hidden="1"/>
+    <col min="12550" max="12552" width="14.5" style="2" hidden="1"/>
+    <col min="12553" max="12553" width="3.1640625" style="2" hidden="1"/>
+    <col min="12554" max="12554" width="1.83203125" style="2" hidden="1"/>
+    <col min="12555" max="12555" width="2.1640625" style="2" hidden="1"/>
+    <col min="12556" max="12556" width="0.83203125" style="2" hidden="1"/>
+    <col min="12557" max="12557" width="13.83203125" style="2" hidden="1"/>
+    <col min="12558" max="12558" width="3.1640625" style="2" hidden="1"/>
+    <col min="12559" max="12559" width="9.5" style="2" hidden="1"/>
+    <col min="12560" max="12560" width="12.1640625" style="2" hidden="1"/>
+    <col min="12561" max="12561" width="2.1640625" style="2" hidden="1"/>
+    <col min="12562" max="12801" width="9.1640625" style="2" hidden="1"/>
+    <col min="12802" max="12802" width="2.1640625" style="2" hidden="1"/>
+    <col min="12803" max="12803" width="1.83203125" style="2" hidden="1"/>
+    <col min="12804" max="12804" width="2.1640625" style="2" hidden="1"/>
+    <col min="12805" max="12805" width="0.83203125" style="2" hidden="1"/>
+    <col min="12806" max="12808" width="14.5" style="2" hidden="1"/>
+    <col min="12809" max="12809" width="3.1640625" style="2" hidden="1"/>
+    <col min="12810" max="12810" width="1.83203125" style="2" hidden="1"/>
+    <col min="12811" max="12811" width="2.1640625" style="2" hidden="1"/>
+    <col min="12812" max="12812" width="0.83203125" style="2" hidden="1"/>
+    <col min="12813" max="12813" width="13.83203125" style="2" hidden="1"/>
+    <col min="12814" max="12814" width="3.1640625" style="2" hidden="1"/>
+    <col min="12815" max="12815" width="9.5" style="2" hidden="1"/>
+    <col min="12816" max="12816" width="12.1640625" style="2" hidden="1"/>
+    <col min="12817" max="12817" width="2.1640625" style="2" hidden="1"/>
+    <col min="12818" max="13057" width="9.1640625" style="2" hidden="1"/>
+    <col min="13058" max="13058" width="2.1640625" style="2" hidden="1"/>
+    <col min="13059" max="13059" width="1.83203125" style="2" hidden="1"/>
+    <col min="13060" max="13060" width="2.1640625" style="2" hidden="1"/>
+    <col min="13061" max="13061" width="0.83203125" style="2" hidden="1"/>
+    <col min="13062" max="13064" width="14.5" style="2" hidden="1"/>
+    <col min="13065" max="13065" width="3.1640625" style="2" hidden="1"/>
+    <col min="13066" max="13066" width="1.83203125" style="2" hidden="1"/>
+    <col min="13067" max="13067" width="2.1640625" style="2" hidden="1"/>
+    <col min="13068" max="13068" width="0.83203125" style="2" hidden="1"/>
+    <col min="13069" max="13069" width="13.83203125" style="2" hidden="1"/>
+    <col min="13070" max="13070" width="3.1640625" style="2" hidden="1"/>
+    <col min="13071" max="13071" width="9.5" style="2" hidden="1"/>
+    <col min="13072" max="13072" width="12.1640625" style="2" hidden="1"/>
+    <col min="13073" max="13073" width="2.1640625" style="2" hidden="1"/>
+    <col min="13074" max="13313" width="9.1640625" style="2" hidden="1"/>
+    <col min="13314" max="13314" width="2.1640625" style="2" hidden="1"/>
+    <col min="13315" max="13315" width="1.83203125" style="2" hidden="1"/>
+    <col min="13316" max="13316" width="2.1640625" style="2" hidden="1"/>
+    <col min="13317" max="13317" width="0.83203125" style="2" hidden="1"/>
+    <col min="13318" max="13320" width="14.5" style="2" hidden="1"/>
+    <col min="13321" max="13321" width="3.1640625" style="2" hidden="1"/>
+    <col min="13322" max="13322" width="1.83203125" style="2" hidden="1"/>
+    <col min="13323" max="13323" width="2.1640625" style="2" hidden="1"/>
+    <col min="13324" max="13324" width="0.83203125" style="2" hidden="1"/>
+    <col min="13325" max="13325" width="13.83203125" style="2" hidden="1"/>
+    <col min="13326" max="13326" width="3.1640625" style="2" hidden="1"/>
+    <col min="13327" max="13327" width="9.5" style="2" hidden="1"/>
+    <col min="13328" max="13328" width="12.1640625" style="2" hidden="1"/>
+    <col min="13329" max="13329" width="2.1640625" style="2" hidden="1"/>
+    <col min="13330" max="13569" width="9.1640625" style="2" hidden="1"/>
+    <col min="13570" max="13570" width="2.1640625" style="2" hidden="1"/>
+    <col min="13571" max="13571" width="1.83203125" style="2" hidden="1"/>
+    <col min="13572" max="13572" width="2.1640625" style="2" hidden="1"/>
+    <col min="13573" max="13573" width="0.83203125" style="2" hidden="1"/>
+    <col min="13574" max="13576" width="14.5" style="2" hidden="1"/>
+    <col min="13577" max="13577" width="3.1640625" style="2" hidden="1"/>
+    <col min="13578" max="13578" width="1.83203125" style="2" hidden="1"/>
+    <col min="13579" max="13579" width="2.1640625" style="2" hidden="1"/>
+    <col min="13580" max="13580" width="0.83203125" style="2" hidden="1"/>
+    <col min="13581" max="13581" width="13.83203125" style="2" hidden="1"/>
+    <col min="13582" max="13582" width="3.1640625" style="2" hidden="1"/>
+    <col min="13583" max="13583" width="9.5" style="2" hidden="1"/>
+    <col min="13584" max="13584" width="12.1640625" style="2" hidden="1"/>
+    <col min="13585" max="13585" width="2.1640625" style="2" hidden="1"/>
+    <col min="13586" max="13825" width="9.1640625" style="2" hidden="1"/>
+    <col min="13826" max="13826" width="2.1640625" style="2" hidden="1"/>
+    <col min="13827" max="13827" width="1.83203125" style="2" hidden="1"/>
+    <col min="13828" max="13828" width="2.1640625" style="2" hidden="1"/>
+    <col min="13829" max="13829" width="0.83203125" style="2" hidden="1"/>
+    <col min="13830" max="13832" width="14.5" style="2" hidden="1"/>
+    <col min="13833" max="13833" width="3.1640625" style="2" hidden="1"/>
+    <col min="13834" max="13834" width="1.83203125" style="2" hidden="1"/>
+    <col min="13835" max="13835" width="2.1640625" style="2" hidden="1"/>
+    <col min="13836" max="13836" width="0.83203125" style="2" hidden="1"/>
+    <col min="13837" max="13837" width="13.83203125" style="2" hidden="1"/>
+    <col min="13838" max="13838" width="3.1640625" style="2" hidden="1"/>
+    <col min="13839" max="13839" width="9.5" style="2" hidden="1"/>
+    <col min="13840" max="13840" width="12.1640625" style="2" hidden="1"/>
+    <col min="13841" max="13841" width="2.1640625" style="2" hidden="1"/>
+    <col min="13842" max="14081" width="9.1640625" style="2" hidden="1"/>
+    <col min="14082" max="14082" width="2.1640625" style="2" hidden="1"/>
+    <col min="14083" max="14083" width="1.83203125" style="2" hidden="1"/>
+    <col min="14084" max="14084" width="2.1640625" style="2" hidden="1"/>
+    <col min="14085" max="14085" width="0.83203125" style="2" hidden="1"/>
+    <col min="14086" max="14088" width="14.5" style="2" hidden="1"/>
+    <col min="14089" max="14089" width="3.1640625" style="2" hidden="1"/>
+    <col min="14090" max="14090" width="1.83203125" style="2" hidden="1"/>
+    <col min="14091" max="14091" width="2.1640625" style="2" hidden="1"/>
+    <col min="14092" max="14092" width="0.83203125" style="2" hidden="1"/>
+    <col min="14093" max="14093" width="13.83203125" style="2" hidden="1"/>
+    <col min="14094" max="14094" width="3.1640625" style="2" hidden="1"/>
+    <col min="14095" max="14095" width="9.5" style="2" hidden="1"/>
+    <col min="14096" max="14096" width="12.1640625" style="2" hidden="1"/>
+    <col min="14097" max="14097" width="2.1640625" style="2" hidden="1"/>
+    <col min="14098" max="14337" width="9.1640625" style="2" hidden="1"/>
+    <col min="14338" max="14338" width="2.1640625" style="2" hidden="1"/>
+    <col min="14339" max="14339" width="1.83203125" style="2" hidden="1"/>
+    <col min="14340" max="14340" width="2.1640625" style="2" hidden="1"/>
+    <col min="14341" max="14341" width="0.83203125" style="2" hidden="1"/>
+    <col min="14342" max="14344" width="14.5" style="2" hidden="1"/>
+    <col min="14345" max="14345" width="3.1640625" style="2" hidden="1"/>
+    <col min="14346" max="14346" width="1.83203125" style="2" hidden="1"/>
+    <col min="14347" max="14347" width="2.1640625" style="2" hidden="1"/>
+    <col min="14348" max="14348" width="0.83203125" style="2" hidden="1"/>
+    <col min="14349" max="14349" width="13.83203125" style="2" hidden="1"/>
+    <col min="14350" max="14350" width="3.1640625" style="2" hidden="1"/>
+    <col min="14351" max="14351" width="9.5" style="2" hidden="1"/>
+    <col min="14352" max="14352" width="12.1640625" style="2" hidden="1"/>
+    <col min="14353" max="14353" width="2.1640625" style="2" hidden="1"/>
+    <col min="14354" max="14593" width="9.1640625" style="2" hidden="1"/>
+    <col min="14594" max="14594" width="2.1640625" style="2" hidden="1"/>
+    <col min="14595" max="14595" width="1.83203125" style="2" hidden="1"/>
+    <col min="14596" max="14596" width="2.1640625" style="2" hidden="1"/>
+    <col min="14597" max="14597" width="0.83203125" style="2" hidden="1"/>
+    <col min="14598" max="14600" width="14.5" style="2" hidden="1"/>
+    <col min="14601" max="14601" width="3.1640625" style="2" hidden="1"/>
+    <col min="14602" max="14602" width="1.83203125" style="2" hidden="1"/>
+    <col min="14603" max="14603" width="2.1640625" style="2" hidden="1"/>
+    <col min="14604" max="14604" width="0.83203125" style="2" hidden="1"/>
+    <col min="14605" max="14605" width="13.83203125" style="2" hidden="1"/>
+    <col min="14606" max="14606" width="3.1640625" style="2" hidden="1"/>
+    <col min="14607" max="14607" width="9.5" style="2" hidden="1"/>
+    <col min="14608" max="14608" width="12.1640625" style="2" hidden="1"/>
+    <col min="14609" max="14609" width="2.1640625" style="2" hidden="1"/>
+    <col min="14610" max="14849" width="9.1640625" style="2" hidden="1"/>
+    <col min="14850" max="14850" width="2.1640625" style="2" hidden="1"/>
+    <col min="14851" max="14851" width="1.83203125" style="2" hidden="1"/>
+    <col min="14852" max="14852" width="2.1640625" style="2" hidden="1"/>
+    <col min="14853" max="14853" width="0.83203125" style="2" hidden="1"/>
+    <col min="14854" max="14856" width="14.5" style="2" hidden="1"/>
+    <col min="14857" max="14857" width="3.1640625" style="2" hidden="1"/>
+    <col min="14858" max="14858" width="1.83203125" style="2" hidden="1"/>
+    <col min="14859" max="14859" width="2.1640625" style="2" hidden="1"/>
+    <col min="14860" max="14860" width="0.83203125" style="2" hidden="1"/>
+    <col min="14861" max="14861" width="13.83203125" style="2" hidden="1"/>
+    <col min="14862" max="14862" width="3.1640625" style="2" hidden="1"/>
+    <col min="14863" max="14863" width="9.5" style="2" hidden="1"/>
+    <col min="14864" max="14864" width="12.1640625" style="2" hidden="1"/>
+    <col min="14865" max="14865" width="2.1640625" style="2" hidden="1"/>
+    <col min="14866" max="15105" width="9.1640625" style="2" hidden="1"/>
+    <col min="15106" max="15106" width="2.1640625" style="2" hidden="1"/>
+    <col min="15107" max="15107" width="1.83203125" style="2" hidden="1"/>
+    <col min="15108" max="15108" width="2.1640625" style="2" hidden="1"/>
+    <col min="15109" max="15109" width="0.83203125" style="2" hidden="1"/>
+    <col min="15110" max="15112" width="14.5" style="2" hidden="1"/>
+    <col min="15113" max="15113" width="3.1640625" style="2" hidden="1"/>
+    <col min="15114" max="15114" width="1.83203125" style="2" hidden="1"/>
+    <col min="15115" max="15115" width="2.1640625" style="2" hidden="1"/>
+    <col min="15116" max="15116" width="0.83203125" style="2" hidden="1"/>
+    <col min="15117" max="15117" width="13.83203125" style="2" hidden="1"/>
+    <col min="15118" max="15118" width="3.1640625" style="2" hidden="1"/>
+    <col min="15119" max="15119" width="9.5" style="2" hidden="1"/>
+    <col min="15120" max="15120" width="12.1640625" style="2" hidden="1"/>
+    <col min="15121" max="15121" width="2.1640625" style="2" hidden="1"/>
+    <col min="15122" max="15361" width="9.1640625" style="2" hidden="1"/>
+    <col min="15362" max="15362" width="2.1640625" style="2" hidden="1"/>
+    <col min="15363" max="15363" width="1.83203125" style="2" hidden="1"/>
+    <col min="15364" max="15364" width="2.1640625" style="2" hidden="1"/>
+    <col min="15365" max="15365" width="0.83203125" style="2" hidden="1"/>
+    <col min="15366" max="15368" width="14.5" style="2" hidden="1"/>
+    <col min="15369" max="15369" width="3.1640625" style="2" hidden="1"/>
+    <col min="15370" max="15370" width="1.83203125" style="2" hidden="1"/>
+    <col min="15371" max="15371" width="2.1640625" style="2" hidden="1"/>
+    <col min="15372" max="15372" width="0.83203125" style="2" hidden="1"/>
+    <col min="15373" max="15373" width="13.83203125" style="2" hidden="1"/>
+    <col min="15374" max="15374" width="3.1640625" style="2" hidden="1"/>
+    <col min="15375" max="15375" width="9.5" style="2" hidden="1"/>
+    <col min="15376" max="15376" width="12.1640625" style="2" hidden="1"/>
+    <col min="15377" max="15377" width="2.1640625" style="2" hidden="1"/>
+    <col min="15378" max="15617" width="9.1640625" style="2" hidden="1"/>
+    <col min="15618" max="15618" width="2.1640625" style="2" hidden="1"/>
+    <col min="15619" max="15619" width="1.83203125" style="2" hidden="1"/>
+    <col min="15620" max="15620" width="2.1640625" style="2" hidden="1"/>
+    <col min="15621" max="15621" width="0.83203125" style="2" hidden="1"/>
+    <col min="15622" max="15624" width="14.5" style="2" hidden="1"/>
+    <col min="15625" max="15625" width="3.1640625" style="2" hidden="1"/>
+    <col min="15626" max="15626" width="1.83203125" style="2" hidden="1"/>
+    <col min="15627" max="15627" width="2.1640625" style="2" hidden="1"/>
+    <col min="15628" max="15628" width="0.83203125" style="2" hidden="1"/>
+    <col min="15629" max="15629" width="13.83203125" style="2" hidden="1"/>
+    <col min="15630" max="15630" width="3.1640625" style="2" hidden="1"/>
+    <col min="15631" max="15631" width="9.5" style="2" hidden="1"/>
+    <col min="15632" max="15632" width="12.1640625" style="2" hidden="1"/>
+    <col min="15633" max="15633" width="2.1640625" style="2" hidden="1"/>
+    <col min="15634" max="15873" width="9.1640625" style="2" hidden="1"/>
+    <col min="15874" max="15874" width="2.1640625" style="2" hidden="1"/>
+    <col min="15875" max="15875" width="1.83203125" style="2" hidden="1"/>
+    <col min="15876" max="15876" width="2.1640625" style="2" hidden="1"/>
+    <col min="15877" max="15877" width="0.83203125" style="2" hidden="1"/>
+    <col min="15878" max="15880" width="14.5" style="2" hidden="1"/>
+    <col min="15881" max="15881" width="3.1640625" style="2" hidden="1"/>
+    <col min="15882" max="15882" width="1.83203125" style="2" hidden="1"/>
+    <col min="15883" max="15883" width="2.1640625" style="2" hidden="1"/>
+    <col min="15884" max="15884" width="0.83203125" style="2" hidden="1"/>
+    <col min="15885" max="15885" width="13.83203125" style="2" hidden="1"/>
+    <col min="15886" max="15886" width="3.1640625" style="2" hidden="1"/>
+    <col min="15887" max="15887" width="9.5" style="2" hidden="1"/>
+    <col min="15888" max="15888" width="12.1640625" style="2" hidden="1"/>
+    <col min="15889" max="15889" width="2.1640625" style="2" hidden="1"/>
+    <col min="15890" max="16129" width="9.1640625" style="2" hidden="1"/>
+    <col min="16130" max="16130" width="2.1640625" style="2" hidden="1"/>
+    <col min="16131" max="16131" width="1.83203125" style="2" hidden="1"/>
+    <col min="16132" max="16132" width="2.1640625" style="2" hidden="1"/>
+    <col min="16133" max="16133" width="0.83203125" style="2" hidden="1"/>
+    <col min="16134" max="16136" width="14.5" style="2" hidden="1"/>
+    <col min="16137" max="16137" width="3.1640625" style="2" hidden="1"/>
+    <col min="16138" max="16138" width="1.83203125" style="2" hidden="1"/>
+    <col min="16139" max="16139" width="2.1640625" style="2" hidden="1"/>
+    <col min="16140" max="16140" width="0.83203125" style="2" hidden="1"/>
+    <col min="16141" max="16141" width="13.83203125" style="2" hidden="1"/>
+    <col min="16142" max="16142" width="3.1640625" style="2" hidden="1"/>
+    <col min="16143" max="16143" width="9.5" style="2" hidden="1"/>
+    <col min="16144" max="16144" width="12.1640625" style="2" hidden="1"/>
+    <col min="16145" max="16145" width="2.1640625" style="2" hidden="1"/>
+    <col min="16146" max="16384" width="9.1640625" style="2" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="O1" s="3"/>
-    </row>
-    <row r="2" spans="1:15" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P1" s="3"/>
+    </row>
+    <row r="2" spans="1:16" ht="12" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.15">
       <c r="A3" s="46" t="s">
         <v>2</v>
       </c>
@@ -2945,8 +2918,9 @@
       <c r="M3" s="46"/>
       <c r="N3" s="46"/>
       <c r="O3" s="46"/>
-    </row>
-    <row r="4" spans="1:15" ht="10.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P3" s="46"/>
+    </row>
+    <row r="4" spans="1:16" ht="11" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="47" t="s">
         <v>69</v>
       </c>
@@ -2964,8 +2938,9 @@
       <c r="M4" s="47"/>
       <c r="N4" s="47"/>
       <c r="O4" s="47"/>
-    </row>
-    <row r="5" spans="1:15" ht="10.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P4" s="47"/>
+    </row>
+    <row r="5" spans="1:16" ht="11" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="48" t="s">
         <v>68</v>
       </c>
@@ -2983,8 +2958,9 @@
       <c r="M5" s="48"/>
       <c r="N5" s="48"/>
       <c r="O5" s="48"/>
-    </row>
-    <row r="6" spans="1:15" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P5" s="48"/>
+    </row>
+    <row r="6" spans="1:16" ht="4.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="49"/>
       <c r="B6" s="49"/>
       <c r="C6" s="49"/>
@@ -3000,8 +2976,9 @@
       <c r="M6" s="49"/>
       <c r="N6" s="49"/>
       <c r="O6" s="49"/>
-    </row>
-    <row r="7" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P6" s="49"/>
+    </row>
+    <row r="7" spans="1:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="50" t="s">
         <v>3</v>
       </c>
@@ -3019,8 +2996,9 @@
       <c r="M7" s="50"/>
       <c r="N7" s="50"/>
       <c r="O7" s="50"/>
-    </row>
-    <row r="8" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P7" s="50"/>
+    </row>
+    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B8" s="4" t="s">
         <v>4</v>
       </c>
@@ -3030,30 +3008,30 @@
       <c r="F8" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="51" t="s">
+      <c r="G8" s="12"/>
+      <c r="H8" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="H8" s="51"/>
-      <c r="I8" s="51" t="s">
+      <c r="I8" s="51"/>
+      <c r="J8" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="J8" s="51"/>
       <c r="K8" s="51"/>
       <c r="L8" s="51"/>
       <c r="M8" s="51"/>
-      <c r="N8" s="51" t="s">
+      <c r="N8" s="51"/>
+      <c r="O8" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="O8" s="52"/>
-    </row>
-    <row r="9" spans="1:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P8" s="52"/>
+    </row>
+    <row r="9" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B9" s="7"/>
       <c r="C9" s="53" t="s">
         <v>72</v>
       </c>
       <c r="D9" s="53"/>
       <c r="E9" s="53"/>
-      <c r="G9" s="54"/>
       <c r="H9" s="54"/>
       <c r="I9" s="54"/>
       <c r="J9" s="54"/>
@@ -3061,9 +3039,10 @@
       <c r="L9" s="54"/>
       <c r="M9" s="54"/>
       <c r="N9" s="54"/>
-      <c r="O9" s="55"/>
-    </row>
-    <row r="10" spans="1:15" ht="2.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O9" s="54"/>
+      <c r="P9" s="55"/>
+    </row>
+    <row r="10" spans="1:16" ht="2.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B10" s="8"/>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
@@ -3077,9 +3056,10 @@
       <c r="L10" s="9"/>
       <c r="M10" s="9"/>
       <c r="N10" s="9"/>
-      <c r="O10" s="10"/>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O10" s="9"/>
+      <c r="P10" s="10"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.15">
       <c r="B11" s="4" t="s">
         <v>9</v>
       </c>
@@ -3087,21 +3067,22 @@
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
       <c r="F11" s="11"/>
-      <c r="G11" s="12" t="s">
+      <c r="G11" s="79"/>
+      <c r="H11" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="H11" s="56"/>
       <c r="I11" s="56"/>
       <c r="J11" s="56"/>
       <c r="K11" s="56"/>
       <c r="L11" s="56"/>
-      <c r="M11" s="13"/>
-      <c r="N11" s="5" t="s">
+      <c r="M11" s="56"/>
+      <c r="N11" s="13"/>
+      <c r="O11" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="O11" s="14"/>
-    </row>
-    <row r="12" spans="1:15" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P11" s="14"/>
+    </row>
+    <row r="12" spans="1:16" ht="5.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B12" s="8"/>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
@@ -3115,10 +3096,11 @@
       <c r="L12" s="9"/>
       <c r="M12" s="9"/>
       <c r="N12" s="9"/>
-      <c r="O12" s="10"/>
-    </row>
-    <row r="13" spans="1:15" ht="2.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O12" s="9"/>
+      <c r="P12" s="10"/>
+    </row>
+    <row r="13" spans="1:16" ht="2.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.15">
       <c r="B14" s="43" t="s">
         <v>12</v>
       </c>
@@ -3134,13 +3116,14 @@
       <c r="L14" s="44"/>
       <c r="M14" s="44"/>
       <c r="N14" s="44"/>
-      <c r="O14" s="45"/>
-    </row>
-    <row r="15" spans="1:15" ht="2.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O14" s="44"/>
+      <c r="P14" s="45"/>
+    </row>
+    <row r="15" spans="1:16" ht="2.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B15" s="15"/>
       <c r="C15" s="15"/>
     </row>
-    <row r="16" spans="1:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B16" s="16" t="s">
         <v>13</v>
       </c>
@@ -3149,658 +3132,674 @@
       <c r="E16" s="6"/>
       <c r="F16" s="6"/>
       <c r="G16" s="6"/>
-      <c r="H16" s="17"/>
-      <c r="I16" s="16" t="s">
+      <c r="H16" s="6"/>
+      <c r="I16" s="17"/>
+      <c r="J16" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="J16" s="18"/>
       <c r="K16" s="18"/>
       <c r="L16" s="18"/>
       <c r="M16" s="18"/>
-      <c r="N16" s="6"/>
-      <c r="O16" s="17"/>
-    </row>
-    <row r="17" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N16" s="18"/>
+      <c r="O16" s="6"/>
+      <c r="P16" s="17"/>
+    </row>
+    <row r="17" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B17" s="7"/>
       <c r="C17" s="19"/>
       <c r="E17" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="H17" s="21"/>
-      <c r="I17" s="7"/>
-      <c r="J17" s="22" t="s">
+      <c r="I17" s="21"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="L17" s="23"/>
       <c r="M17" s="23"/>
-      <c r="O17" s="21"/>
-    </row>
-    <row r="18" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N17" s="23"/>
+      <c r="P17" s="21"/>
+    </row>
+    <row r="18" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7"/>
       <c r="C18" s="19"/>
       <c r="E18" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="H18" s="21"/>
-      <c r="I18" s="7"/>
-      <c r="J18" s="19"/>
-      <c r="L18" s="20" t="s">
+      <c r="I18" s="21"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="19"/>
+      <c r="M18" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="M18" s="20"/>
-      <c r="N18" s="9"/>
-      <c r="O18" s="10"/>
-    </row>
-    <row r="19" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N18" s="20"/>
+      <c r="O18" s="9"/>
+      <c r="P18" s="10"/>
+    </row>
+    <row r="19" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B19" s="7"/>
       <c r="C19" s="19"/>
       <c r="E19" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="H19" s="21"/>
-      <c r="I19" s="7"/>
-      <c r="J19" s="19"/>
-      <c r="L19" s="20" t="s">
+      <c r="I19" s="21"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="19"/>
+      <c r="M19" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="M19" s="20"/>
-      <c r="N19" s="25"/>
-      <c r="O19" s="26"/>
-    </row>
-    <row r="20" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N19" s="20"/>
+      <c r="O19" s="25"/>
+      <c r="P19" s="26"/>
+    </row>
+    <row r="20" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B20" s="7"/>
       <c r="C20" s="19"/>
       <c r="E20" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="H20" s="21"/>
-      <c r="I20" s="7"/>
-      <c r="J20" s="27" t="s">
+      <c r="I20" s="21"/>
+      <c r="J20" s="7"/>
+      <c r="K20" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="O20" s="21"/>
-    </row>
-    <row r="21" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P20" s="21"/>
+    </row>
+    <row r="21" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7"/>
       <c r="C21" s="19"/>
       <c r="E21" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="H21" s="21"/>
-      <c r="I21" s="7"/>
-      <c r="J21" s="19"/>
-      <c r="L21" s="20" t="s">
+      <c r="I21" s="21"/>
+      <c r="J21" s="7"/>
+      <c r="K21" s="19"/>
+      <c r="M21" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="M21" s="20"/>
-      <c r="N21" s="9"/>
-      <c r="O21" s="10"/>
-    </row>
-    <row r="22" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N21" s="20"/>
+      <c r="O21" s="9"/>
+      <c r="P21" s="10"/>
+    </row>
+    <row r="22" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B22" s="7"/>
       <c r="C22" s="19"/>
       <c r="E22" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="H22" s="21"/>
-      <c r="I22" s="7"/>
-      <c r="J22" s="19"/>
-      <c r="L22" s="20" t="s">
+      <c r="I22" s="21"/>
+      <c r="J22" s="7"/>
+      <c r="K22" s="19"/>
+      <c r="M22" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="M22" s="20"/>
-      <c r="N22" s="9"/>
-      <c r="O22" s="10"/>
-    </row>
-    <row r="23" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N22" s="20"/>
+      <c r="O22" s="9"/>
+      <c r="P22" s="10"/>
+    </row>
+    <row r="23" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B23" s="7"/>
       <c r="C23" s="19"/>
       <c r="E23" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="H23" s="21"/>
-      <c r="I23" s="7"/>
-      <c r="J23" s="22" t="s">
+      <c r="I23" s="21"/>
+      <c r="J23" s="7"/>
+      <c r="K23" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="O23" s="21"/>
-    </row>
-    <row r="24" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P23" s="21"/>
+    </row>
+    <row r="24" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B24" s="7"/>
       <c r="C24" s="19"/>
       <c r="E24" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="H24" s="21"/>
-      <c r="I24" s="7"/>
-      <c r="K24" s="20" t="s">
+      <c r="I24" s="21"/>
+      <c r="J24" s="7"/>
+      <c r="L24" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="M24" s="9"/>
       <c r="N24" s="9"/>
-      <c r="O24" s="10"/>
-    </row>
-    <row r="25" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="O24" s="9"/>
+      <c r="P24" s="10"/>
+    </row>
+    <row r="25" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B25" s="7"/>
       <c r="C25" s="19"/>
       <c r="E25" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="H25" s="21"/>
-      <c r="I25" s="7"/>
-      <c r="J25" s="22" t="s">
+      <c r="I25" s="21"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="O25" s="21"/>
-    </row>
-    <row r="26" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P25" s="21"/>
+    </row>
+    <row r="26" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B26" s="7"/>
       <c r="C26" s="19"/>
       <c r="E26" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="H26" s="21"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="19"/>
-      <c r="L26" s="24" t="s">
+      <c r="I26" s="21"/>
+      <c r="J26" s="7"/>
+      <c r="K26" s="19"/>
+      <c r="M26" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="M26" s="24"/>
-      <c r="O26" s="21"/>
-    </row>
-    <row r="27" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N26" s="24"/>
+      <c r="P26" s="21"/>
+    </row>
+    <row r="27" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B27" s="7"/>
       <c r="C27" s="19"/>
       <c r="E27" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="H27" s="21"/>
-      <c r="I27" s="7"/>
-      <c r="J27" s="19"/>
-      <c r="L27" s="20" t="s">
+      <c r="I27" s="21"/>
+      <c r="J27" s="7"/>
+      <c r="K27" s="19"/>
+      <c r="M27" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="M27" s="20"/>
-      <c r="O27" s="21"/>
-    </row>
-    <row r="28" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N27" s="20"/>
+      <c r="P27" s="21"/>
+    </row>
+    <row r="28" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B28" s="7"/>
       <c r="C28" s="19"/>
       <c r="E28" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="H28" s="21"/>
-      <c r="I28" s="7"/>
-      <c r="L28" s="27" t="s">
+      <c r="I28" s="21"/>
+      <c r="J28" s="7"/>
+      <c r="M28" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="M28" s="28"/>
-      <c r="N28" s="9"/>
-      <c r="O28" s="10"/>
-    </row>
-    <row r="29" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N28" s="28"/>
+      <c r="O28" s="9"/>
+      <c r="P28" s="10"/>
+    </row>
+    <row r="29" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B29" s="7"/>
       <c r="C29" s="19"/>
-      <c r="E29" s="24" t="s">
-        <v>39</v>
-      </c>
-      <c r="H29" s="21"/>
-      <c r="I29" s="7"/>
-      <c r="J29" s="19"/>
-      <c r="L29" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="M29" s="24"/>
-      <c r="O29" s="21"/>
-    </row>
-    <row r="30" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E29" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="I29" s="21"/>
+      <c r="J29" s="7"/>
+      <c r="M29" s="27"/>
+      <c r="N29" s="27"/>
+      <c r="P29" s="21"/>
+    </row>
+    <row r="30" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B30" s="7"/>
       <c r="C30" s="19"/>
-      <c r="E30" s="27" t="s">
+      <c r="E30" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="I30" s="21"/>
+      <c r="J30" s="7"/>
+      <c r="K30" s="19"/>
+      <c r="M30" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="N30" s="24"/>
+      <c r="P30" s="21"/>
+    </row>
+    <row r="31" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="B31" s="7"/>
+      <c r="C31" s="19"/>
+      <c r="E31" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="F30" s="57"/>
-      <c r="G30" s="57"/>
-      <c r="H30" s="21"/>
-      <c r="I30" s="7"/>
-      <c r="J30" s="19"/>
-      <c r="L30" s="20" t="s">
+      <c r="F31" s="57"/>
+      <c r="G31" s="57"/>
+      <c r="H31" s="57"/>
+      <c r="I31" s="21"/>
+      <c r="J31" s="7"/>
+      <c r="K31" s="19"/>
+      <c r="M31" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="M30" s="20"/>
-      <c r="O30" s="21"/>
-    </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B31" s="8"/>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
-      <c r="G31" s="9"/>
-      <c r="H31" s="10"/>
-      <c r="I31" s="8"/>
-      <c r="J31" s="9"/>
-      <c r="K31" s="9"/>
-      <c r="L31" s="9"/>
-      <c r="M31" s="9"/>
-      <c r="N31" s="9"/>
-      <c r="O31" s="10"/>
-    </row>
-    <row r="32" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="16" t="s">
+      <c r="N31" s="20"/>
+      <c r="P31" s="21"/>
+    </row>
+    <row r="32" spans="2:16" x14ac:dyDescent="0.15">
+      <c r="B32" s="8"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="9"/>
+      <c r="I32" s="10"/>
+      <c r="J32" s="8"/>
+      <c r="K32" s="9"/>
+      <c r="L32" s="9"/>
+      <c r="M32" s="9"/>
+      <c r="N32" s="9"/>
+      <c r="O32" s="9"/>
+      <c r="P32" s="10"/>
+    </row>
+    <row r="33" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="B33" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="C32" s="6"/>
-      <c r="D32" s="6"/>
-      <c r="E32" s="6"/>
-      <c r="F32" s="6"/>
-      <c r="G32" s="6"/>
-      <c r="H32" s="17"/>
-      <c r="I32" s="16" t="s">
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
+      <c r="H33" s="6"/>
+      <c r="I33" s="17"/>
+      <c r="J33" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="J32" s="6"/>
-      <c r="K32" s="6"/>
-      <c r="L32" s="6"/>
-      <c r="M32" s="6"/>
-      <c r="N32" s="6"/>
-      <c r="O32" s="17"/>
-    </row>
-    <row r="33" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="7"/>
-      <c r="E33" s="66"/>
-      <c r="F33" s="66"/>
-      <c r="G33" s="66"/>
-      <c r="H33" s="21"/>
-      <c r="I33" s="7"/>
-      <c r="J33" s="19"/>
-      <c r="L33" s="20" t="s">
+      <c r="K33" s="6"/>
+      <c r="L33" s="6"/>
+      <c r="M33" s="6"/>
+      <c r="N33" s="6"/>
+      <c r="O33" s="6"/>
+      <c r="P33" s="17"/>
+    </row>
+    <row r="34" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="B34" s="7"/>
+      <c r="E34" s="66"/>
+      <c r="F34" s="66"/>
+      <c r="G34" s="66"/>
+      <c r="H34" s="66"/>
+      <c r="I34" s="21"/>
+      <c r="J34" s="7"/>
+      <c r="K34" s="19"/>
+      <c r="M34" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="M33" s="20"/>
-      <c r="O33" s="21"/>
-    </row>
-    <row r="34" spans="2:15" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="7"/>
-      <c r="D34" s="29" t="s">
+      <c r="N34" s="20"/>
+      <c r="P34" s="21"/>
+    </row>
+    <row r="35" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="B35" s="7"/>
+      <c r="D35" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="H34" s="21"/>
-      <c r="I34" s="7"/>
-      <c r="J34" s="19"/>
-      <c r="L34" s="20" t="s">
+      <c r="I35" s="21"/>
+      <c r="J35" s="7"/>
+      <c r="K35" s="19"/>
+      <c r="M35" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="M34" s="20"/>
-      <c r="O34" s="21"/>
-    </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="7"/>
-      <c r="E35" s="58"/>
-      <c r="F35" s="58"/>
-      <c r="G35" s="58"/>
-      <c r="H35" s="21"/>
-      <c r="I35" s="8"/>
-      <c r="J35" s="9"/>
-      <c r="K35" s="9"/>
-      <c r="L35" s="9"/>
-      <c r="M35" s="9"/>
-      <c r="N35" s="9"/>
-      <c r="O35" s="10"/>
-    </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="N35" s="20"/>
+      <c r="P35" s="21"/>
+    </row>
+    <row r="36" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B36" s="7"/>
-      <c r="H36" s="21"/>
-      <c r="I36" s="59" t="s">
+      <c r="E36" s="58"/>
+      <c r="F36" s="58"/>
+      <c r="G36" s="58"/>
+      <c r="H36" s="58"/>
+      <c r="I36" s="21"/>
+      <c r="J36" s="8"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="10"/>
+    </row>
+    <row r="37" spans="2:16" x14ac:dyDescent="0.15">
+      <c r="B37" s="7"/>
+      <c r="I37" s="21"/>
+      <c r="J37" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="J36" s="60"/>
-      <c r="K36" s="60"/>
-      <c r="L36" s="60"/>
-      <c r="M36" s="60"/>
-      <c r="N36" s="60"/>
-      <c r="O36" s="61"/>
-    </row>
-    <row r="37" spans="2:15" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="8"/>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-      <c r="G37" s="9"/>
-      <c r="H37" s="10"/>
-      <c r="I37" s="8"/>
-      <c r="J37" s="9"/>
-      <c r="K37" s="9"/>
-      <c r="L37" s="9"/>
-      <c r="M37" s="9"/>
-      <c r="N37" s="9"/>
-      <c r="O37" s="10"/>
-    </row>
-    <row r="38" spans="2:15" ht="2.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B39" s="43" t="s">
+      <c r="K37" s="60"/>
+      <c r="L37" s="60"/>
+      <c r="M37" s="60"/>
+      <c r="N37" s="60"/>
+      <c r="O37" s="60"/>
+      <c r="P37" s="61"/>
+    </row>
+    <row r="38" spans="2:16" ht="6" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B38" s="8"/>
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="9"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="9"/>
+      <c r="I38" s="10"/>
+      <c r="J38" s="8"/>
+      <c r="K38" s="9"/>
+      <c r="L38" s="9"/>
+      <c r="M38" s="9"/>
+      <c r="N38" s="9"/>
+      <c r="O38" s="9"/>
+      <c r="P38" s="10"/>
+    </row>
+    <row r="39" spans="2:16" ht="2.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="40" spans="2:16" x14ac:dyDescent="0.15">
+      <c r="B40" s="43" t="s">
         <v>49</v>
       </c>
-      <c r="C39" s="44"/>
-      <c r="D39" s="44"/>
-      <c r="E39" s="44"/>
-      <c r="F39" s="44"/>
-      <c r="G39" s="44"/>
-      <c r="H39" s="44"/>
-      <c r="I39" s="44"/>
-      <c r="J39" s="44"/>
-      <c r="K39" s="44"/>
-      <c r="L39" s="44"/>
-      <c r="M39" s="44"/>
-      <c r="N39" s="44"/>
-      <c r="O39" s="45"/>
-    </row>
-    <row r="40" spans="2:15" ht="2.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B41" s="16" t="s">
+      <c r="C40" s="44"/>
+      <c r="D40" s="44"/>
+      <c r="E40" s="44"/>
+      <c r="F40" s="44"/>
+      <c r="G40" s="44"/>
+      <c r="H40" s="44"/>
+      <c r="I40" s="44"/>
+      <c r="J40" s="44"/>
+      <c r="K40" s="44"/>
+      <c r="L40" s="44"/>
+      <c r="M40" s="44"/>
+      <c r="N40" s="44"/>
+      <c r="O40" s="44"/>
+      <c r="P40" s="45"/>
+    </row>
+    <row r="41" spans="2:16" ht="2.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="42" spans="2:16" x14ac:dyDescent="0.15">
+      <c r="B42" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="C41" s="6"/>
-      <c r="D41" s="6"/>
-      <c r="E41" s="6"/>
-      <c r="F41" s="6"/>
-      <c r="G41" s="6"/>
-      <c r="H41" s="6"/>
-      <c r="I41" s="16" t="s">
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="6"/>
+      <c r="F42" s="6"/>
+      <c r="G42" s="6"/>
+      <c r="H42" s="6"/>
+      <c r="I42" s="6"/>
+      <c r="J42" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="J41" s="6"/>
-      <c r="K41" s="6"/>
-      <c r="L41" s="6"/>
-      <c r="M41" s="6"/>
-      <c r="N41" s="6"/>
-      <c r="O41" s="17"/>
-    </row>
-    <row r="42" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B42" s="7"/>
-      <c r="E42" s="30" t="s">
+      <c r="K42" s="6"/>
+      <c r="L42" s="6"/>
+      <c r="M42" s="6"/>
+      <c r="N42" s="6"/>
+      <c r="O42" s="6"/>
+      <c r="P42" s="17"/>
+    </row>
+    <row r="43" spans="2:16" x14ac:dyDescent="0.15">
+      <c r="B43" s="7"/>
+      <c r="E43" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="F42" s="62"/>
-      <c r="G42" s="62"/>
-      <c r="H42" s="20"/>
-      <c r="I42" s="7"/>
-      <c r="O42" s="21"/>
-    </row>
-    <row r="43" spans="2:15" ht="2.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="7"/>
-      <c r="E43" s="30"/>
-      <c r="H43" s="20"/>
-      <c r="I43" s="7"/>
-      <c r="O43" s="21"/>
-    </row>
-    <row r="44" spans="2:15" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F43" s="62"/>
+      <c r="G43" s="62"/>
+      <c r="H43" s="62"/>
+      <c r="I43" s="20"/>
+      <c r="J43" s="7"/>
+      <c r="P43" s="21"/>
+    </row>
+    <row r="44" spans="2:16" ht="2.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B44" s="7"/>
-      <c r="E44" s="31"/>
-      <c r="F44" s="32" t="s">
+      <c r="E44" s="30"/>
+      <c r="I44" s="20"/>
+      <c r="J44" s="7"/>
+      <c r="P44" s="21"/>
+    </row>
+    <row r="45" spans="2:16" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="B45" s="7"/>
+      <c r="E45" s="31"/>
+      <c r="F45" s="32" t="s">
         <v>53</v>
       </c>
-      <c r="G44" s="32" t="s">
+      <c r="G45" s="32" t="s">
         <v>54</v>
       </c>
-      <c r="I44" s="7"/>
-      <c r="J44" s="33"/>
-      <c r="L44" s="20" t="s">
+      <c r="H45" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="J45" s="7"/>
+      <c r="K45" s="33"/>
+      <c r="M45" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="M44" s="20"/>
-      <c r="O44" s="21"/>
-    </row>
-    <row r="45" spans="2:15" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="7"/>
-      <c r="E45" s="34" t="s">
-        <v>56</v>
-      </c>
-      <c r="F45" s="35"/>
-      <c r="G45" s="35"/>
-      <c r="I45" s="7"/>
-      <c r="J45" s="33"/>
-      <c r="L45" s="20" t="s">
-        <v>57</v>
-      </c>
-      <c r="M45" s="36"/>
-      <c r="N45" s="9"/>
-      <c r="O45" s="10"/>
-    </row>
-    <row r="46" spans="2:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N45" s="20"/>
+      <c r="P45" s="21"/>
+    </row>
+    <row r="46" spans="2:16" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B46" s="7"/>
       <c r="E46" s="34" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F46" s="35"/>
       <c r="G46" s="35"/>
-      <c r="I46" s="7"/>
-      <c r="L46" s="9"/>
-      <c r="M46" s="9"/>
-      <c r="N46" s="9"/>
-      <c r="O46" s="10"/>
-    </row>
-    <row r="47" spans="2:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H46" s="35"/>
+      <c r="J46" s="7"/>
+      <c r="K46" s="33"/>
+      <c r="M46" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="N46" s="36"/>
+      <c r="O46" s="9"/>
+      <c r="P46" s="10"/>
+    </row>
+    <row r="47" spans="2:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B47" s="7"/>
       <c r="E47" s="34" t="s">
-        <v>59</v>
-      </c>
-      <c r="F47" s="35">
-        <f>F45-F46</f>
-        <v>0</v>
-      </c>
-      <c r="G47" s="35">
-        <f>G45-G46</f>
-        <v>0</v>
-      </c>
-      <c r="I47" s="7"/>
-      <c r="L47" s="9"/>
+        <v>58</v>
+      </c>
+      <c r="F47" s="35"/>
+      <c r="G47" s="35"/>
+      <c r="H47" s="35"/>
+      <c r="J47" s="7"/>
       <c r="M47" s="9"/>
       <c r="N47" s="9"/>
-      <c r="O47" s="10"/>
-    </row>
-    <row r="48" spans="2:15" ht="6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O47" s="9"/>
+      <c r="P47" s="10"/>
+    </row>
+    <row r="48" spans="2:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B48" s="7"/>
-      <c r="I48" s="7"/>
-      <c r="O48" s="21"/>
-    </row>
-    <row r="49" spans="2:15" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E48" s="34" t="s">
+        <v>59</v>
+      </c>
+      <c r="F48" s="35">
+        <f>F46-F47</f>
+        <v>0</v>
+      </c>
+      <c r="G48" s="35"/>
+      <c r="H48" s="35">
+        <f>H46-H47</f>
+        <v>0</v>
+      </c>
+      <c r="J48" s="7"/>
+      <c r="M48" s="9"/>
+      <c r="N48" s="9"/>
+      <c r="O48" s="9"/>
+      <c r="P48" s="10"/>
+    </row>
+    <row r="49" spans="2:16" ht="6" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B49" s="7"/>
-      <c r="I49" s="7"/>
-      <c r="O49" s="21"/>
-    </row>
-    <row r="50" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="J49" s="7"/>
+      <c r="P49" s="21"/>
+    </row>
+    <row r="50" spans="2:16" ht="10.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B50" s="7"/>
-      <c r="E50" s="76"/>
-      <c r="F50" s="76"/>
-      <c r="G50" s="76"/>
-      <c r="I50" s="7"/>
-      <c r="L50" s="76"/>
-      <c r="M50" s="76"/>
-      <c r="N50" s="76"/>
-      <c r="O50" s="77"/>
-    </row>
-    <row r="51" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J50" s="7"/>
+      <c r="P50" s="21"/>
+    </row>
+    <row r="51" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B51" s="7"/>
-      <c r="E51" s="67" t="s">
+      <c r="E51" s="76"/>
+      <c r="F51" s="76"/>
+      <c r="G51" s="76"/>
+      <c r="H51" s="76"/>
+      <c r="J51" s="7"/>
+      <c r="M51" s="76"/>
+      <c r="N51" s="76"/>
+      <c r="O51" s="76"/>
+      <c r="P51" s="77"/>
+    </row>
+    <row r="52" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B52" s="7"/>
+      <c r="E52" s="67" t="s">
         <v>75</v>
       </c>
-      <c r="F51" s="67"/>
-      <c r="G51" s="67"/>
-      <c r="I51" s="37"/>
-      <c r="J51" s="38"/>
-      <c r="K51" s="38"/>
-      <c r="L51" s="67" t="s">
+      <c r="F52" s="67"/>
+      <c r="G52" s="67"/>
+      <c r="H52" s="67"/>
+      <c r="J52" s="37"/>
+      <c r="K52" s="38"/>
+      <c r="L52" s="38"/>
+      <c r="M52" s="67" t="s">
         <v>71</v>
       </c>
-      <c r="M51" s="67"/>
-      <c r="N51" s="67"/>
-      <c r="O51" s="68"/>
-    </row>
-    <row r="52" spans="2:15" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="8"/>
-      <c r="C52" s="9"/>
-      <c r="D52" s="9"/>
-      <c r="E52" s="9"/>
-      <c r="F52" s="9"/>
-      <c r="G52" s="9"/>
-      <c r="H52" s="9"/>
-      <c r="I52" s="8"/>
-      <c r="J52" s="9"/>
-      <c r="K52" s="9"/>
-      <c r="L52" s="9"/>
-      <c r="M52" s="9"/>
-      <c r="N52" s="9"/>
-      <c r="O52" s="10"/>
-    </row>
-    <row r="53" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B53" s="4" t="s">
+      <c r="N52" s="67"/>
+      <c r="O52" s="67"/>
+      <c r="P52" s="68"/>
+    </row>
+    <row r="53" spans="2:16" ht="4.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B53" s="8"/>
+      <c r="C53" s="9"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="9"/>
+      <c r="F53" s="9"/>
+      <c r="G53" s="9"/>
+      <c r="H53" s="9"/>
+      <c r="I53" s="9"/>
+      <c r="J53" s="8"/>
+      <c r="K53" s="9"/>
+      <c r="L53" s="9"/>
+      <c r="M53" s="9"/>
+      <c r="N53" s="9"/>
+      <c r="O53" s="9"/>
+      <c r="P53" s="10"/>
+    </row>
+    <row r="54" spans="2:16" x14ac:dyDescent="0.15">
+      <c r="B54" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C53" s="6"/>
-      <c r="D53" s="6"/>
-      <c r="E53" s="6"/>
-      <c r="F53" s="6"/>
-      <c r="G53" s="6"/>
-      <c r="H53" s="6"/>
-      <c r="I53" s="5" t="s">
+      <c r="C54" s="6"/>
+      <c r="D54" s="6"/>
+      <c r="E54" s="6"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="6"/>
+      <c r="H54" s="6"/>
+      <c r="I54" s="6"/>
+      <c r="J54" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="J53" s="6"/>
-      <c r="K53" s="6"/>
-      <c r="L53" s="6"/>
-      <c r="M53" s="6"/>
-      <c r="N53" s="25"/>
-      <c r="O53" s="26"/>
-    </row>
-    <row r="54" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B54" s="69"/>
-      <c r="C54" s="70"/>
-      <c r="D54" s="70"/>
-      <c r="E54" s="20" t="s">
+      <c r="K54" s="6"/>
+      <c r="L54" s="6"/>
+      <c r="M54" s="6"/>
+      <c r="N54" s="6"/>
+      <c r="O54" s="25"/>
+      <c r="P54" s="26"/>
+    </row>
+    <row r="55" spans="2:16" x14ac:dyDescent="0.15">
+      <c r="B55" s="69"/>
+      <c r="C55" s="70"/>
+      <c r="D55" s="70"/>
+      <c r="E55" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="L54" s="9"/>
-      <c r="M54" s="9"/>
-      <c r="N54" s="9"/>
-      <c r="O54" s="10"/>
-    </row>
-    <row r="55" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B55" s="8"/>
-      <c r="C55" s="9"/>
-      <c r="D55" s="9"/>
-      <c r="E55" s="20" t="s">
+      <c r="M55" s="9"/>
+      <c r="N55" s="9"/>
+      <c r="O55" s="9"/>
+      <c r="P55" s="10"/>
+    </row>
+    <row r="56" spans="2:16" x14ac:dyDescent="0.15">
+      <c r="B56" s="8"/>
+      <c r="C56" s="9"/>
+      <c r="D56" s="9"/>
+      <c r="E56" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="L55" s="9"/>
-      <c r="M55" s="36"/>
-      <c r="N55" s="9"/>
-      <c r="O55" s="10"/>
-    </row>
-    <row r="56" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B56" s="40"/>
-      <c r="C56" s="25"/>
-      <c r="D56" s="25"/>
-      <c r="E56" s="20" t="s">
+      <c r="M56" s="9"/>
+      <c r="N56" s="36"/>
+      <c r="O56" s="9"/>
+      <c r="P56" s="10"/>
+    </row>
+    <row r="57" spans="2:16" x14ac:dyDescent="0.15">
+      <c r="B57" s="40"/>
+      <c r="C57" s="25"/>
+      <c r="D57" s="25"/>
+      <c r="E57" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="L56" s="9"/>
-      <c r="M56" s="9"/>
-      <c r="N56" s="9"/>
-      <c r="O56" s="10"/>
-    </row>
-    <row r="57" spans="2:15" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="7"/>
-      <c r="O57" s="21"/>
-    </row>
-    <row r="58" spans="2:15" ht="7.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M57" s="9"/>
+      <c r="N57" s="9"/>
+      <c r="O57" s="9"/>
+      <c r="P57" s="10"/>
+    </row>
+    <row r="58" spans="2:16" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B58" s="7"/>
-      <c r="G58" s="71"/>
-      <c r="H58" s="71"/>
-      <c r="I58" s="71"/>
-      <c r="J58" s="71"/>
-      <c r="K58" s="71"/>
-      <c r="L58" s="71"/>
-      <c r="O58" s="21"/>
-    </row>
-    <row r="59" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P58" s="21"/>
+    </row>
+    <row r="59" spans="2:16" ht="8" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B59" s="7"/>
-      <c r="G59" s="72" t="s">
+      <c r="H59" s="71"/>
+      <c r="I59" s="71"/>
+      <c r="J59" s="71"/>
+      <c r="K59" s="71"/>
+      <c r="L59" s="71"/>
+      <c r="M59" s="71"/>
+      <c r="P59" s="21"/>
+    </row>
+    <row r="60" spans="2:16" x14ac:dyDescent="0.15">
+      <c r="B60" s="7"/>
+      <c r="H60" s="72" t="s">
         <v>73</v>
       </c>
-      <c r="H59" s="72"/>
-      <c r="I59" s="72"/>
-      <c r="J59" s="72"/>
-      <c r="K59" s="72"/>
-      <c r="L59" s="72"/>
-      <c r="O59" s="21"/>
-    </row>
-    <row r="60" spans="2:15" ht="7.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="8"/>
-      <c r="C60" s="9"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="9"/>
-      <c r="F60" s="9"/>
-      <c r="G60" s="78" t="s">
+      <c r="I60" s="72"/>
+      <c r="J60" s="72"/>
+      <c r="K60" s="72"/>
+      <c r="L60" s="72"/>
+      <c r="M60" s="72"/>
+      <c r="P60" s="21"/>
+    </row>
+    <row r="61" spans="2:16" ht="8" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B61" s="8"/>
+      <c r="C61" s="9"/>
+      <c r="D61" s="9"/>
+      <c r="E61" s="9"/>
+      <c r="F61" s="9"/>
+      <c r="G61" s="9"/>
+      <c r="H61" s="78" t="s">
         <v>76</v>
       </c>
-      <c r="H60" s="78"/>
-      <c r="I60" s="78"/>
-      <c r="J60" s="78"/>
-      <c r="K60" s="78"/>
-      <c r="L60" s="78"/>
-      <c r="M60" s="9"/>
-      <c r="N60" s="9"/>
-      <c r="O60" s="10"/>
-    </row>
-    <row r="61" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="41" t="s">
+      <c r="I61" s="78"/>
+      <c r="J61" s="78"/>
+      <c r="K61" s="78"/>
+      <c r="L61" s="78"/>
+      <c r="M61" s="78"/>
+      <c r="N61" s="9"/>
+      <c r="O61" s="9"/>
+      <c r="P61" s="10"/>
+    </row>
+    <row r="62" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B62" s="41" t="s">
         <v>70</v>
       </c>
-      <c r="C61" s="42"/>
-    </row>
-    <row r="62" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B62" s="73" t="s">
+      <c r="C62" s="42"/>
+    </row>
+    <row r="63" spans="2:16" x14ac:dyDescent="0.15">
+      <c r="B63" s="73" t="s">
         <v>65</v>
       </c>
-      <c r="C62" s="74"/>
-      <c r="D62" s="74"/>
-      <c r="E62" s="74"/>
-      <c r="F62" s="74"/>
-      <c r="G62" s="74"/>
-      <c r="H62" s="74"/>
-      <c r="I62" s="74"/>
-      <c r="J62" s="74"/>
-      <c r="K62" s="74"/>
-      <c r="L62" s="74"/>
-      <c r="M62" s="74"/>
-      <c r="N62" s="74"/>
-      <c r="O62" s="75"/>
-    </row>
-    <row r="63" spans="2:15" ht="9" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B64" s="63" t="s">
+      <c r="C63" s="74"/>
+      <c r="D63" s="74"/>
+      <c r="E63" s="74"/>
+      <c r="F63" s="74"/>
+      <c r="G63" s="74"/>
+      <c r="H63" s="74"/>
+      <c r="I63" s="74"/>
+      <c r="J63" s="74"/>
+      <c r="K63" s="74"/>
+      <c r="L63" s="74"/>
+      <c r="M63" s="74"/>
+      <c r="N63" s="74"/>
+      <c r="O63" s="74"/>
+      <c r="P63" s="75"/>
+    </row>
+    <row r="64" spans="2:16" ht="9" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="65" spans="2:16" x14ac:dyDescent="0.15">
+      <c r="B65" s="63" t="s">
         <v>66</v>
       </c>
-      <c r="C64" s="64"/>
-      <c r="D64" s="64"/>
-      <c r="E64" s="64"/>
-      <c r="F64" s="64"/>
-      <c r="G64" s="64"/>
-      <c r="H64" s="64"/>
-      <c r="I64" s="63" t="s">
-        <v>67</v>
-      </c>
-      <c r="J64" s="64"/>
-      <c r="K64" s="64"/>
-      <c r="L64" s="64"/>
-      <c r="M64" s="64"/>
-      <c r="N64" s="64"/>
-      <c r="O64" s="64"/>
-    </row>
-    <row r="65" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B65" s="64"/>
       <c r="C65" s="64"/>
       <c r="D65" s="64"/>
       <c r="E65" s="64"/>
@@ -3808,14 +3807,17 @@
       <c r="G65" s="64"/>
       <c r="H65" s="64"/>
       <c r="I65" s="64"/>
-      <c r="J65" s="64"/>
+      <c r="J65" s="63" t="s">
+        <v>67</v>
+      </c>
       <c r="K65" s="64"/>
       <c r="L65" s="64"/>
       <c r="M65" s="64"/>
       <c r="N65" s="64"/>
       <c r="O65" s="64"/>
-    </row>
-    <row r="66" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P65" s="64"/>
+    </row>
+    <row r="66" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B66" s="64"/>
       <c r="C66" s="64"/>
       <c r="D66" s="64"/>
@@ -3830,8 +3832,9 @@
       <c r="M66" s="64"/>
       <c r="N66" s="64"/>
       <c r="O66" s="64"/>
-    </row>
-    <row r="67" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P66" s="64"/>
+    </row>
+    <row r="67" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B67" s="64"/>
       <c r="C67" s="64"/>
       <c r="D67" s="64"/>
@@ -3846,8 +3849,9 @@
       <c r="M67" s="64"/>
       <c r="N67" s="64"/>
       <c r="O67" s="64"/>
-    </row>
-    <row r="68" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P67" s="64"/>
+    </row>
+    <row r="68" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B68" s="64"/>
       <c r="C68" s="64"/>
       <c r="D68" s="64"/>
@@ -3862,8 +3866,9 @@
       <c r="M68" s="64"/>
       <c r="N68" s="64"/>
       <c r="O68" s="64"/>
-    </row>
-    <row r="69" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P68" s="64"/>
+    </row>
+    <row r="69" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B69" s="64"/>
       <c r="C69" s="64"/>
       <c r="D69" s="64"/>
@@ -3878,8 +3883,9 @@
       <c r="M69" s="64"/>
       <c r="N69" s="64"/>
       <c r="O69" s="64"/>
-    </row>
-    <row r="70" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P69" s="64"/>
+    </row>
+    <row r="70" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B70" s="64"/>
       <c r="C70" s="64"/>
       <c r="D70" s="64"/>
@@ -3894,8 +3900,9 @@
       <c r="M70" s="64"/>
       <c r="N70" s="64"/>
       <c r="O70" s="64"/>
-    </row>
-    <row r="71" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P70" s="64"/>
+    </row>
+    <row r="71" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B71" s="64"/>
       <c r="C71" s="64"/>
       <c r="D71" s="64"/>
@@ -3910,8 +3917,9 @@
       <c r="M71" s="64"/>
       <c r="N71" s="64"/>
       <c r="O71" s="64"/>
-    </row>
-    <row r="72" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P71" s="64"/>
+    </row>
+    <row r="72" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B72" s="64"/>
       <c r="C72" s="64"/>
       <c r="D72" s="64"/>
@@ -3926,8 +3934,9 @@
       <c r="M72" s="64"/>
       <c r="N72" s="64"/>
       <c r="O72" s="64"/>
-    </row>
-    <row r="73" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P72" s="64"/>
+    </row>
+    <row r="73" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B73" s="64"/>
       <c r="C73" s="64"/>
       <c r="D73" s="64"/>
@@ -3942,8 +3951,9 @@
       <c r="M73" s="64"/>
       <c r="N73" s="64"/>
       <c r="O73" s="64"/>
-    </row>
-    <row r="74" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P73" s="64"/>
+    </row>
+    <row r="74" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B74" s="64"/>
       <c r="C74" s="64"/>
       <c r="D74" s="64"/>
@@ -3958,8 +3968,9 @@
       <c r="M74" s="64"/>
       <c r="N74" s="64"/>
       <c r="O74" s="64"/>
-    </row>
-    <row r="75" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P74" s="64"/>
+    </row>
+    <row r="75" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B75" s="64"/>
       <c r="C75" s="64"/>
       <c r="D75" s="64"/>
@@ -3974,8 +3985,9 @@
       <c r="M75" s="64"/>
       <c r="N75" s="64"/>
       <c r="O75" s="64"/>
-    </row>
-    <row r="76" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P75" s="64"/>
+    </row>
+    <row r="76" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B76" s="64"/>
       <c r="C76" s="64"/>
       <c r="D76" s="64"/>
@@ -3990,8 +4002,9 @@
       <c r="M76" s="64"/>
       <c r="N76" s="64"/>
       <c r="O76" s="64"/>
-    </row>
-    <row r="77" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P76" s="64"/>
+    </row>
+    <row r="77" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B77" s="64"/>
       <c r="C77" s="64"/>
       <c r="D77" s="64"/>
@@ -4006,8 +4019,9 @@
       <c r="M77" s="64"/>
       <c r="N77" s="64"/>
       <c r="O77" s="64"/>
-    </row>
-    <row r="78" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P77" s="64"/>
+    </row>
+    <row r="78" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B78" s="64"/>
       <c r="C78" s="64"/>
       <c r="D78" s="64"/>
@@ -4022,8 +4036,9 @@
       <c r="M78" s="64"/>
       <c r="N78" s="64"/>
       <c r="O78" s="64"/>
-    </row>
-    <row r="79" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P78" s="64"/>
+    </row>
+    <row r="79" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B79" s="64"/>
       <c r="C79" s="64"/>
       <c r="D79" s="64"/>
@@ -4038,8 +4053,9 @@
       <c r="M79" s="64"/>
       <c r="N79" s="64"/>
       <c r="O79" s="64"/>
-    </row>
-    <row r="80" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P79" s="64"/>
+    </row>
+    <row r="80" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B80" s="64"/>
       <c r="C80" s="64"/>
       <c r="D80" s="64"/>
@@ -4054,8 +4070,9 @@
       <c r="M80" s="64"/>
       <c r="N80" s="64"/>
       <c r="O80" s="64"/>
-    </row>
-    <row r="81" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P80" s="64"/>
+    </row>
+    <row r="81" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B81" s="64"/>
       <c r="C81" s="64"/>
       <c r="D81" s="64"/>
@@ -4070,8 +4087,9 @@
       <c r="M81" s="64"/>
       <c r="N81" s="64"/>
       <c r="O81" s="64"/>
-    </row>
-    <row r="82" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P81" s="64"/>
+    </row>
+    <row r="82" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B82" s="64"/>
       <c r="C82" s="64"/>
       <c r="D82" s="64"/>
@@ -4086,8 +4104,9 @@
       <c r="M82" s="64"/>
       <c r="N82" s="64"/>
       <c r="O82" s="64"/>
-    </row>
-    <row r="83" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P82" s="64"/>
+    </row>
+    <row r="83" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B83" s="64"/>
       <c r="C83" s="64"/>
       <c r="D83" s="64"/>
@@ -4102,8 +4121,9 @@
       <c r="M83" s="64"/>
       <c r="N83" s="64"/>
       <c r="O83" s="64"/>
-    </row>
-    <row r="84" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P83" s="64"/>
+    </row>
+    <row r="84" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B84" s="64"/>
       <c r="C84" s="64"/>
       <c r="D84" s="64"/>
@@ -4118,8 +4138,9 @@
       <c r="M84" s="64"/>
       <c r="N84" s="64"/>
       <c r="O84" s="64"/>
-    </row>
-    <row r="85" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P84" s="64"/>
+    </row>
+    <row r="85" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B85" s="64"/>
       <c r="C85" s="64"/>
       <c r="D85" s="64"/>
@@ -4134,8 +4155,9 @@
       <c r="M85" s="64"/>
       <c r="N85" s="64"/>
       <c r="O85" s="64"/>
-    </row>
-    <row r="86" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P85" s="64"/>
+    </row>
+    <row r="86" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B86" s="64"/>
       <c r="C86" s="64"/>
       <c r="D86" s="64"/>
@@ -4150,8 +4172,9 @@
       <c r="M86" s="64"/>
       <c r="N86" s="64"/>
       <c r="O86" s="64"/>
-    </row>
-    <row r="87" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P86" s="64"/>
+    </row>
+    <row r="87" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B87" s="64"/>
       <c r="C87" s="64"/>
       <c r="D87" s="64"/>
@@ -4166,8 +4189,9 @@
       <c r="M87" s="64"/>
       <c r="N87" s="64"/>
       <c r="O87" s="64"/>
-    </row>
-    <row r="88" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P87" s="64"/>
+    </row>
+    <row r="88" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B88" s="64"/>
       <c r="C88" s="64"/>
       <c r="D88" s="64"/>
@@ -4182,8 +4206,9 @@
       <c r="M88" s="64"/>
       <c r="N88" s="64"/>
       <c r="O88" s="64"/>
-    </row>
-    <row r="89" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P88" s="64"/>
+    </row>
+    <row r="89" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B89" s="64"/>
       <c r="C89" s="64"/>
       <c r="D89" s="64"/>
@@ -4198,8 +4223,9 @@
       <c r="M89" s="64"/>
       <c r="N89" s="64"/>
       <c r="O89" s="64"/>
-    </row>
-    <row r="90" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P89" s="64"/>
+    </row>
+    <row r="90" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B90" s="64"/>
       <c r="C90" s="64"/>
       <c r="D90" s="64"/>
@@ -4214,8 +4240,9 @@
       <c r="M90" s="64"/>
       <c r="N90" s="64"/>
       <c r="O90" s="64"/>
-    </row>
-    <row r="91" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P90" s="64"/>
+    </row>
+    <row r="91" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B91" s="64"/>
       <c r="C91" s="64"/>
       <c r="D91" s="64"/>
@@ -4230,8 +4257,9 @@
       <c r="M91" s="64"/>
       <c r="N91" s="64"/>
       <c r="O91" s="64"/>
-    </row>
-    <row r="92" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P91" s="64"/>
+    </row>
+    <row r="92" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B92" s="64"/>
       <c r="C92" s="64"/>
       <c r="D92" s="64"/>
@@ -4246,8 +4274,9 @@
       <c r="M92" s="64"/>
       <c r="N92" s="64"/>
       <c r="O92" s="64"/>
-    </row>
-    <row r="93" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P92" s="64"/>
+    </row>
+    <row r="93" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B93" s="64"/>
       <c r="C93" s="64"/>
       <c r="D93" s="64"/>
@@ -4262,8 +4291,9 @@
       <c r="M93" s="64"/>
       <c r="N93" s="64"/>
       <c r="O93" s="64"/>
-    </row>
-    <row r="94" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P93" s="64"/>
+    </row>
+    <row r="94" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B94" s="64"/>
       <c r="C94" s="64"/>
       <c r="D94" s="64"/>
@@ -4278,8 +4308,9 @@
       <c r="M94" s="64"/>
       <c r="N94" s="64"/>
       <c r="O94" s="64"/>
-    </row>
-    <row r="95" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P94" s="64"/>
+    </row>
+    <row r="95" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B95" s="64"/>
       <c r="C95" s="64"/>
       <c r="D95" s="64"/>
@@ -4294,8 +4325,9 @@
       <c r="M95" s="64"/>
       <c r="N95" s="64"/>
       <c r="O95" s="64"/>
-    </row>
-    <row r="96" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P95" s="64"/>
+    </row>
+    <row r="96" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B96" s="64"/>
       <c r="C96" s="64"/>
       <c r="D96" s="64"/>
@@ -4310,8 +4342,9 @@
       <c r="M96" s="64"/>
       <c r="N96" s="64"/>
       <c r="O96" s="64"/>
-    </row>
-    <row r="97" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P96" s="64"/>
+    </row>
+    <row r="97" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B97" s="64"/>
       <c r="C97" s="64"/>
       <c r="D97" s="64"/>
@@ -4326,8 +4359,9 @@
       <c r="M97" s="64"/>
       <c r="N97" s="64"/>
       <c r="O97" s="64"/>
-    </row>
-    <row r="98" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P97" s="64"/>
+    </row>
+    <row r="98" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B98" s="64"/>
       <c r="C98" s="64"/>
       <c r="D98" s="64"/>
@@ -4342,8 +4376,9 @@
       <c r="M98" s="64"/>
       <c r="N98" s="64"/>
       <c r="O98" s="64"/>
-    </row>
-    <row r="99" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P98" s="64"/>
+    </row>
+    <row r="99" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B99" s="64"/>
       <c r="C99" s="64"/>
       <c r="D99" s="64"/>
@@ -4358,8 +4393,9 @@
       <c r="M99" s="64"/>
       <c r="N99" s="64"/>
       <c r="O99" s="64"/>
-    </row>
-    <row r="100" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P99" s="64"/>
+    </row>
+    <row r="100" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B100" s="64"/>
       <c r="C100" s="64"/>
       <c r="D100" s="64"/>
@@ -4374,8 +4410,9 @@
       <c r="M100" s="64"/>
       <c r="N100" s="64"/>
       <c r="O100" s="64"/>
-    </row>
-    <row r="101" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P100" s="64"/>
+    </row>
+    <row r="101" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B101" s="64"/>
       <c r="C101" s="64"/>
       <c r="D101" s="64"/>
@@ -4390,8 +4427,9 @@
       <c r="M101" s="64"/>
       <c r="N101" s="64"/>
       <c r="O101" s="64"/>
-    </row>
-    <row r="102" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P101" s="64"/>
+    </row>
+    <row r="102" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B102" s="64"/>
       <c r="C102" s="64"/>
       <c r="D102" s="64"/>
@@ -4406,8 +4444,9 @@
       <c r="M102" s="64"/>
       <c r="N102" s="64"/>
       <c r="O102" s="64"/>
-    </row>
-    <row r="103" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P102" s="64"/>
+    </row>
+    <row r="103" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B103" s="64"/>
       <c r="C103" s="64"/>
       <c r="D103" s="64"/>
@@ -4422,8 +4461,9 @@
       <c r="M103" s="64"/>
       <c r="N103" s="64"/>
       <c r="O103" s="64"/>
-    </row>
-    <row r="104" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P103" s="64"/>
+    </row>
+    <row r="104" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B104" s="64"/>
       <c r="C104" s="64"/>
       <c r="D104" s="64"/>
@@ -4438,8 +4478,9 @@
       <c r="M104" s="64"/>
       <c r="N104" s="64"/>
       <c r="O104" s="64"/>
-    </row>
-    <row r="105" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P104" s="64"/>
+    </row>
+    <row r="105" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B105" s="64"/>
       <c r="C105" s="64"/>
       <c r="D105" s="64"/>
@@ -4454,8 +4495,9 @@
       <c r="M105" s="64"/>
       <c r="N105" s="64"/>
       <c r="O105" s="64"/>
-    </row>
-    <row r="106" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="P105" s="64"/>
+    </row>
+    <row r="106" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B106" s="64"/>
       <c r="C106" s="64"/>
       <c r="D106" s="64"/>
@@ -4470,8 +4512,9 @@
       <c r="M106" s="64"/>
       <c r="N106" s="64"/>
       <c r="O106" s="64"/>
-    </row>
-    <row r="107" spans="2:15" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P106" s="64"/>
+    </row>
+    <row r="107" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B107" s="64"/>
       <c r="C107" s="64"/>
       <c r="D107" s="64"/>
@@ -4486,44 +4529,47 @@
       <c r="M107" s="64"/>
       <c r="N107" s="64"/>
       <c r="O107" s="64"/>
-    </row>
-    <row r="108" spans="2:15" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B108" s="39"/>
-      <c r="C108" s="39"/>
-      <c r="D108" s="39"/>
-      <c r="E108" s="39"/>
-      <c r="F108" s="39"/>
-      <c r="G108" s="39"/>
-      <c r="H108" s="39"/>
-      <c r="I108" s="39"/>
-      <c r="J108" s="39"/>
-      <c r="K108" s="39"/>
-      <c r="L108" s="39"/>
-      <c r="M108" s="39"/>
-      <c r="N108" s="39"/>
-      <c r="O108" s="39"/>
-    </row>
-    <row r="109" spans="2:15" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B110" s="65" t="s">
+      <c r="P107" s="64"/>
+    </row>
+    <row r="108" spans="2:16" ht="6.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B108" s="64"/>
+      <c r="C108" s="64"/>
+      <c r="D108" s="64"/>
+      <c r="E108" s="64"/>
+      <c r="F108" s="64"/>
+      <c r="G108" s="64"/>
+      <c r="H108" s="64"/>
+      <c r="I108" s="64"/>
+      <c r="J108" s="64"/>
+      <c r="K108" s="64"/>
+      <c r="L108" s="64"/>
+      <c r="M108" s="64"/>
+      <c r="N108" s="64"/>
+      <c r="O108" s="64"/>
+      <c r="P108" s="64"/>
+    </row>
+    <row r="109" spans="2:16" ht="6.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B109" s="39"/>
+      <c r="C109" s="39"/>
+      <c r="D109" s="39"/>
+      <c r="E109" s="39"/>
+      <c r="F109" s="39"/>
+      <c r="G109" s="39"/>
+      <c r="H109" s="39"/>
+      <c r="I109" s="39"/>
+      <c r="J109" s="39"/>
+      <c r="K109" s="39"/>
+      <c r="L109" s="39"/>
+      <c r="M109" s="39"/>
+      <c r="N109" s="39"/>
+      <c r="O109" s="39"/>
+      <c r="P109" s="39"/>
+    </row>
+    <row r="110" spans="2:16" ht="12" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="111" spans="2:16" x14ac:dyDescent="0.15">
+      <c r="B111" s="65" t="s">
         <v>74</v>
       </c>
-      <c r="C110" s="65"/>
-      <c r="D110" s="65"/>
-      <c r="E110" s="65"/>
-      <c r="F110" s="65"/>
-      <c r="G110" s="65"/>
-      <c r="H110" s="65"/>
-      <c r="I110" s="65"/>
-      <c r="J110" s="65"/>
-      <c r="K110" s="65"/>
-      <c r="L110" s="65"/>
-      <c r="M110" s="65"/>
-      <c r="N110" s="65"/>
-      <c r="O110" s="65"/>
-    </row>
-    <row r="111" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B111" s="65"/>
       <c r="C111" s="65"/>
       <c r="D111" s="65"/>
       <c r="E111" s="65"/>
@@ -4537,46 +4583,64 @@
       <c r="M111" s="65"/>
       <c r="N111" s="65"/>
       <c r="O111" s="65"/>
-    </row>
-    <row r="112" spans="2:15" x14ac:dyDescent="0.25"/>
-    <row r="113" x14ac:dyDescent="0.25"/>
-    <row r="114" x14ac:dyDescent="0.25"/>
-    <row r="115" x14ac:dyDescent="0.25"/>
-    <row r="116" x14ac:dyDescent="0.25"/>
+      <c r="P111" s="65"/>
+    </row>
+    <row r="112" spans="2:16" x14ac:dyDescent="0.15">
+      <c r="B112" s="65"/>
+      <c r="C112" s="65"/>
+      <c r="D112" s="65"/>
+      <c r="E112" s="65"/>
+      <c r="F112" s="65"/>
+      <c r="G112" s="65"/>
+      <c r="H112" s="65"/>
+      <c r="I112" s="65"/>
+      <c r="J112" s="65"/>
+      <c r="K112" s="65"/>
+      <c r="L112" s="65"/>
+      <c r="M112" s="65"/>
+      <c r="N112" s="65"/>
+      <c r="O112" s="65"/>
+      <c r="P112" s="65"/>
+    </row>
+    <row r="113" x14ac:dyDescent="0.15"/>
+    <row r="114" x14ac:dyDescent="0.15"/>
+    <row r="115" x14ac:dyDescent="0.15"/>
+    <row r="116" x14ac:dyDescent="0.15"/>
+    <row r="117" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="B64:H107"/>
-    <mergeCell ref="I64:O107"/>
-    <mergeCell ref="B110:O111"/>
-    <mergeCell ref="E33:G33"/>
-    <mergeCell ref="E51:G51"/>
-    <mergeCell ref="L51:O51"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="G58:L58"/>
-    <mergeCell ref="G59:L59"/>
-    <mergeCell ref="B62:O62"/>
-    <mergeCell ref="E50:G50"/>
-    <mergeCell ref="L50:O50"/>
-    <mergeCell ref="G60:L60"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="E35:G35"/>
-    <mergeCell ref="I36:O36"/>
-    <mergeCell ref="B39:O39"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="B14:O14"/>
-    <mergeCell ref="A3:O3"/>
-    <mergeCell ref="A4:O4"/>
-    <mergeCell ref="A5:O5"/>
-    <mergeCell ref="A6:O6"/>
-    <mergeCell ref="A7:O7"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="I8:M8"/>
-    <mergeCell ref="N8:O8"/>
+    <mergeCell ref="B65:I108"/>
+    <mergeCell ref="J65:P108"/>
+    <mergeCell ref="B111:P112"/>
+    <mergeCell ref="E34:H34"/>
+    <mergeCell ref="E52:H52"/>
+    <mergeCell ref="M52:P52"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="H59:M59"/>
+    <mergeCell ref="H60:M60"/>
+    <mergeCell ref="B63:P63"/>
+    <mergeCell ref="E51:H51"/>
+    <mergeCell ref="M51:P51"/>
+    <mergeCell ref="H61:M61"/>
+    <mergeCell ref="F31:H31"/>
+    <mergeCell ref="E36:H36"/>
+    <mergeCell ref="J37:P37"/>
+    <mergeCell ref="B40:P40"/>
+    <mergeCell ref="F43:H43"/>
+    <mergeCell ref="B14:P14"/>
+    <mergeCell ref="A3:P3"/>
+    <mergeCell ref="A4:P4"/>
+    <mergeCell ref="A5:P5"/>
+    <mergeCell ref="A6:P6"/>
+    <mergeCell ref="A7:P7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="J8:N8"/>
+    <mergeCell ref="O8:P8"/>
     <mergeCell ref="C9:E9"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="I9:M9"/>
-    <mergeCell ref="N9:O9"/>
-    <mergeCell ref="H11:L11"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="J9:N9"/>
+    <mergeCell ref="O9:P9"/>
+    <mergeCell ref="I11:M11"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>